<commit_message>
CCD-7005: Adding new componentLaunchers
</commit_message>
<xml_diff>
--- a/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_Master_Definition.xlsx
+++ b/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_Master_Definition.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jen/IdeaProjects/test-defs-jen/ccd-test-definitions/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{292B7B28-3B2C-3142-854C-3C64141921F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A640CFCE-6D02-534E-B011-5FDDF4FC549F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18020" firstSheet="14" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17880" firstSheet="12" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SearchInputFields" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16031" uniqueCount="1537">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16096" uniqueCount="1545">
   <si>
     <t>SearchInputFields</t>
   </si>
@@ -4660,13 +4660,40 @@
   </si>
   <si>
     <t>${MCA_API_BASE_URL:http://aac-manage-case-assignment-aat.service.core-compute-aat.internal}/noc/apply-decision</t>
+  </si>
+  <si>
+    <t>FT_AllDataTypes</t>
+  </si>
+  <si>
+    <t>Case Type for testing fAllDataTypes</t>
+  </si>
+  <si>
+    <t>ComponentLauncher</t>
+  </si>
+  <si>
+    <t>Summary</t>
+  </si>
+  <si>
+    <t>caseworker-autotest1</t>
+  </si>
+  <si>
+    <t>Roles</t>
+  </si>
+  <si>
+    <t>Hearings</t>
+  </si>
+  <si>
+    <t>Task</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;DD/&quot;mm&quot;/YYYY&quot;"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -4682,16 +4709,28 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -4699,15 +4738,51 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -7735,8 +7810,12 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
-  <dimension ref="A1:L152"/>
+  <dimension ref="A1:L156"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="53.83203125" customWidth="1"/>
+    <col min="8" max="8" width="28" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -11700,6 +11779,110 @@
         <v>463</v>
       </c>
       <c r="I152">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A153" s="1">
+        <v>42742</v>
+      </c>
+      <c r="C153" t="s">
+        <v>1537</v>
+      </c>
+      <c r="D153" t="s">
+        <v>887</v>
+      </c>
+      <c r="E153" t="s">
+        <v>1540</v>
+      </c>
+      <c r="F153" t="s">
+        <v>1540</v>
+      </c>
+      <c r="G153">
+        <v>1</v>
+      </c>
+      <c r="H153" t="s">
+        <v>1540</v>
+      </c>
+      <c r="I153">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A154" s="1">
+        <v>42742</v>
+      </c>
+      <c r="C154" t="s">
+        <v>1537</v>
+      </c>
+      <c r="D154" t="s">
+        <v>887</v>
+      </c>
+      <c r="E154" t="s">
+        <v>1542</v>
+      </c>
+      <c r="F154" t="s">
+        <v>1542</v>
+      </c>
+      <c r="G154">
+        <v>1</v>
+      </c>
+      <c r="H154" t="s">
+        <v>1542</v>
+      </c>
+      <c r="I154">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A155" s="1">
+        <v>42742</v>
+      </c>
+      <c r="C155" t="s">
+        <v>1537</v>
+      </c>
+      <c r="D155" t="s">
+        <v>887</v>
+      </c>
+      <c r="E155" t="s">
+        <v>1543</v>
+      </c>
+      <c r="F155" t="s">
+        <v>1543</v>
+      </c>
+      <c r="G155">
+        <v>1</v>
+      </c>
+      <c r="H155" t="s">
+        <v>1543</v>
+      </c>
+      <c r="I155">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A156" s="1">
+        <v>42742</v>
+      </c>
+      <c r="C156" t="s">
+        <v>1537</v>
+      </c>
+      <c r="D156" t="s">
+        <v>887</v>
+      </c>
+      <c r="E156" t="s">
+        <v>1544</v>
+      </c>
+      <c r="F156" t="s">
+        <v>1544</v>
+      </c>
+      <c r="G156">
+        <v>1</v>
+      </c>
+      <c r="H156" t="s">
+        <v>1544</v>
+      </c>
+      <c r="I156">
         <v>1</v>
       </c>
     </row>
@@ -31057,8 +31240,13 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
-  <dimension ref="A1:F477"/>
+  <dimension ref="A1:F481"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="32" customWidth="1"/>
+    <col min="4" max="4" width="19.83203125" customWidth="1"/>
+    <col min="5" max="5" width="29.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -39141,6 +39329,74 @@
       </c>
       <c r="F477" t="s">
         <v>716</v>
+      </c>
+    </row>
+    <row r="478" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A478" s="1">
+        <v>42743</v>
+      </c>
+      <c r="C478" t="s">
+        <v>1537</v>
+      </c>
+      <c r="D478" t="s">
+        <v>1540</v>
+      </c>
+      <c r="E478" t="s">
+        <v>1541</v>
+      </c>
+      <c r="F478" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="479" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A479" s="1">
+        <v>42743</v>
+      </c>
+      <c r="C479" t="s">
+        <v>1537</v>
+      </c>
+      <c r="D479" t="s">
+        <v>1542</v>
+      </c>
+      <c r="E479" t="s">
+        <v>1541</v>
+      </c>
+      <c r="F479" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="480" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A480" s="1">
+        <v>42743</v>
+      </c>
+      <c r="C480" t="s">
+        <v>1537</v>
+      </c>
+      <c r="D480" t="s">
+        <v>1543</v>
+      </c>
+      <c r="E480" t="s">
+        <v>1541</v>
+      </c>
+      <c r="F480" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="481" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A481" s="1">
+        <v>42743</v>
+      </c>
+      <c r="C481" t="s">
+        <v>1537</v>
+      </c>
+      <c r="D481" t="s">
+        <v>1544</v>
+      </c>
+      <c r="E481" t="s">
+        <v>1541</v>
+      </c>
+      <c r="F481" t="s">
+        <v>643</v>
       </c>
     </row>
   </sheetData>
@@ -51154,8 +51410,13 @@
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="39.83203125" customWidth="1"/>
+    <col min="4" max="4" width="28.6640625" customWidth="1"/>
+    <col min="5" max="5" width="51.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -52243,6 +52504,26 @@
         <v>177</v>
       </c>
       <c r="I55" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A56" s="1">
+        <v>42736</v>
+      </c>
+      <c r="C56" t="s">
+        <v>1537</v>
+      </c>
+      <c r="D56" t="s">
+        <v>1537</v>
+      </c>
+      <c r="E56" t="s">
+        <v>1538</v>
+      </c>
+      <c r="F56" t="s">
+        <v>177</v>
+      </c>
+      <c r="I56" t="s">
         <v>218</v>
       </c>
     </row>
@@ -56503,8 +56784,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Q310"/>
+  <dimension ref="A1:Q314"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="54" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="37.5" customWidth="1"/>
+    <col min="7" max="7" width="23.5" customWidth="1"/>
+    <col min="9" max="9" width="17.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -63658,7 +63946,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="305" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A305" s="1">
         <v>42736</v>
       </c>
@@ -63681,7 +63969,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="306" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A306" s="1">
         <v>42736</v>
       </c>
@@ -63704,7 +63992,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="307" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A307" s="1">
         <v>42736</v>
       </c>
@@ -63727,7 +64015,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="308" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="308" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A308" s="1">
         <v>42736</v>
       </c>
@@ -63756,7 +64044,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="309" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A309" s="1">
         <v>42736</v>
       </c>
@@ -63782,7 +64070,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="310" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A310" s="1">
         <v>42736</v>
       </c>
@@ -63807,6 +64095,130 @@
       <c r="N310" t="s">
         <v>197</v>
       </c>
+    </row>
+    <row r="311" spans="1:15" s="9" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A311" s="3">
+        <v>42736</v>
+      </c>
+      <c r="B311" s="3"/>
+      <c r="C311" s="4" t="s">
+        <v>1537</v>
+      </c>
+      <c r="D311" s="4" t="s">
+        <v>1540</v>
+      </c>
+      <c r="E311" s="4" t="s">
+        <v>1540</v>
+      </c>
+      <c r="F311" s="5"/>
+      <c r="G311" s="6" t="s">
+        <v>1539</v>
+      </c>
+      <c r="H311" s="7"/>
+      <c r="I311" s="8"/>
+      <c r="J311" s="8"/>
+      <c r="K311" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="L311" s="8"/>
+      <c r="M311" s="8"/>
+      <c r="N311" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="O311" s="7"/>
+    </row>
+    <row r="312" spans="1:15" s="9" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A312" s="3">
+        <v>42736</v>
+      </c>
+      <c r="B312" s="3"/>
+      <c r="C312" s="4" t="s">
+        <v>1537</v>
+      </c>
+      <c r="D312" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="E312" s="4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="F312" s="5"/>
+      <c r="G312" s="6" t="s">
+        <v>1539</v>
+      </c>
+      <c r="H312" s="7"/>
+      <c r="I312" s="8"/>
+      <c r="J312" s="8"/>
+      <c r="K312" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="L312" s="8"/>
+      <c r="M312" s="8"/>
+      <c r="N312" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="O312" s="7"/>
+    </row>
+    <row r="313" spans="1:15" s="9" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A313" s="3">
+        <v>42736</v>
+      </c>
+      <c r="B313" s="3"/>
+      <c r="C313" s="4" t="s">
+        <v>1537</v>
+      </c>
+      <c r="D313" s="4" t="s">
+        <v>1543</v>
+      </c>
+      <c r="E313" s="4" t="s">
+        <v>1543</v>
+      </c>
+      <c r="F313" s="5"/>
+      <c r="G313" s="6" t="s">
+        <v>1539</v>
+      </c>
+      <c r="H313" s="7"/>
+      <c r="I313" s="8"/>
+      <c r="J313" s="8"/>
+      <c r="K313" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="L313" s="8"/>
+      <c r="M313" s="8"/>
+      <c r="N313" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="O313" s="7"/>
+    </row>
+    <row r="314" spans="1:15" s="9" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A314" s="3">
+        <v>42736</v>
+      </c>
+      <c r="B314" s="3"/>
+      <c r="C314" s="4" t="s">
+        <v>1537</v>
+      </c>
+      <c r="D314" s="4" t="s">
+        <v>1544</v>
+      </c>
+      <c r="E314" s="4" t="s">
+        <v>1544</v>
+      </c>
+      <c r="F314" s="5"/>
+      <c r="G314" s="6" t="s">
+        <v>1539</v>
+      </c>
+      <c r="H314" s="7"/>
+      <c r="I314" s="8"/>
+      <c r="J314" s="8"/>
+      <c r="K314" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="L314" s="8"/>
+      <c r="M314" s="8"/>
+      <c r="N314" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="O314" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
CCD-7005: updated tab ordering
</commit_message>
<xml_diff>
--- a/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_Master_Definition.xlsx
+++ b/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_Master_Definition.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jen/IdeaProjects/test-defs-jen/ccd-test-definitions/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A45AA9F-5695-2D42-A9D1-0BA5D3C226EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{766FBB92-6CFF-1E46-9EC9-4E8F58A01D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" firstSheet="8" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10755,7 +10755,7 @@
         <v>1538</v>
       </c>
       <c r="G115">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H115" t="s">
         <v>1538</v>
@@ -10781,7 +10781,7 @@
         <v>1539</v>
       </c>
       <c r="G116">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H116" t="s">
         <v>1539</v>
@@ -10807,7 +10807,7 @@
         <v>1540</v>
       </c>
       <c r="G117">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H117" t="s">
         <v>1540</v>
@@ -10833,7 +10833,7 @@
         <v>1541</v>
       </c>
       <c r="G118">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H118" t="s">
         <v>1541</v>

</xml_diff>

<commit_message>
CCD-8066: Updating with Staff User basic type
</commit_message>
<xml_diff>
--- a/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_Master_Definition.xlsx
+++ b/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_Master_Definition.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jen/IdeaProjects/test-defs-jen/ccd-test-definitions/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{292B7B28-3B2C-3142-854C-3C64141921F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{491EB25B-AFB2-A642-A9E7-25A443DDA749}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18020" firstSheet="14" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" firstSheet="14" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SearchInputFields" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16031" uniqueCount="1537">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16058" uniqueCount="1542">
   <si>
     <t>SearchInputFields</t>
   </si>
@@ -4660,13 +4660,28 @@
   </si>
   <si>
     <t>${MCA_API_BASE_URL:http://aac-manage-case-assignment-aat.service.core-compute-aat.internal}/noc/apply-decision</t>
+  </si>
+  <si>
+    <t>StaffUser</t>
+  </si>
+  <si>
+    <t>Staff User</t>
+  </si>
+  <si>
+    <t>StaffUser Fields</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#ARGUMENT(CATEGORY-LEGAL-OPS,CATEGORY-ADMIN,REGION-1235) </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> #ARGUMENT(CATEGORY-LEGAL-OPS,CATEGORY-ADMIN,REGION-1235) </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -4681,6 +4696,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF172B4D"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -4704,10 +4725,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -31057,8 +31079,13 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
-  <dimension ref="A1:F477"/>
+  <dimension ref="A1:F478"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="27.33203125" customWidth="1"/>
+    <col min="4" max="4" width="22.1640625" customWidth="1"/>
+    <col min="5" max="5" width="34.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -37125,13 +37152,13 @@
         <v>42736</v>
       </c>
       <c r="C359" t="s">
-        <v>138</v>
+        <v>114</v>
       </c>
       <c r="D359" t="s">
-        <v>47</v>
+        <v>1537</v>
       </c>
       <c r="E359" t="s">
-        <v>644</v>
+        <v>727</v>
       </c>
       <c r="F359" t="s">
         <v>643</v>
@@ -37142,7 +37169,7 @@
         <v>42736</v>
       </c>
       <c r="C360" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D360" t="s">
         <v>47</v>
@@ -37159,13 +37186,13 @@
         <v>42736</v>
       </c>
       <c r="C361" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D361" t="s">
-        <v>239</v>
+        <v>47</v>
       </c>
       <c r="E361" t="s">
-        <v>735</v>
+        <v>644</v>
       </c>
       <c r="F361" t="s">
         <v>643</v>
@@ -37179,7 +37206,7 @@
         <v>140</v>
       </c>
       <c r="D362" t="s">
-        <v>141</v>
+        <v>239</v>
       </c>
       <c r="E362" t="s">
         <v>735</v>
@@ -37196,7 +37223,7 @@
         <v>140</v>
       </c>
       <c r="D363" t="s">
-        <v>436</v>
+        <v>141</v>
       </c>
       <c r="E363" t="s">
         <v>735</v>
@@ -37213,7 +37240,7 @@
         <v>140</v>
       </c>
       <c r="D364" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E364" t="s">
         <v>735</v>
@@ -37230,7 +37257,7 @@
         <v>140</v>
       </c>
       <c r="D365" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E365" t="s">
         <v>735</v>
@@ -37247,7 +37274,7 @@
         <v>140</v>
       </c>
       <c r="D366" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E366" t="s">
         <v>735</v>
@@ -37264,7 +37291,7 @@
         <v>140</v>
       </c>
       <c r="D367" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E367" t="s">
         <v>735</v>
@@ -37281,7 +37308,7 @@
         <v>140</v>
       </c>
       <c r="D368" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E368" t="s">
         <v>735</v>
@@ -37298,10 +37325,10 @@
         <v>140</v>
       </c>
       <c r="D369" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
       <c r="E369" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="F369" t="s">
         <v>643</v>
@@ -37315,7 +37342,7 @@
         <v>140</v>
       </c>
       <c r="D370" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E370" t="s">
         <v>736</v>
@@ -37332,7 +37359,7 @@
         <v>140</v>
       </c>
       <c r="D371" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E371" t="s">
         <v>736</v>
@@ -37349,7 +37376,7 @@
         <v>140</v>
       </c>
       <c r="D372" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E372" t="s">
         <v>736</v>
@@ -37366,10 +37393,10 @@
         <v>140</v>
       </c>
       <c r="D373" t="s">
-        <v>239</v>
+        <v>446</v>
       </c>
       <c r="E373" t="s">
-        <v>644</v>
+        <v>736</v>
       </c>
       <c r="F373" t="s">
         <v>643</v>
@@ -37383,7 +37410,7 @@
         <v>140</v>
       </c>
       <c r="D374" t="s">
-        <v>141</v>
+        <v>239</v>
       </c>
       <c r="E374" t="s">
         <v>644</v>
@@ -37400,7 +37427,7 @@
         <v>140</v>
       </c>
       <c r="D375" t="s">
-        <v>436</v>
+        <v>141</v>
       </c>
       <c r="E375" t="s">
         <v>644</v>
@@ -37417,7 +37444,7 @@
         <v>140</v>
       </c>
       <c r="D376" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E376" t="s">
         <v>644</v>
@@ -37434,7 +37461,7 @@
         <v>140</v>
       </c>
       <c r="D377" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E377" t="s">
         <v>644</v>
@@ -37451,7 +37478,7 @@
         <v>140</v>
       </c>
       <c r="D378" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E378" t="s">
         <v>644</v>
@@ -37468,7 +37495,7 @@
         <v>140</v>
       </c>
       <c r="D379" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E379" t="s">
         <v>644</v>
@@ -37485,7 +37512,7 @@
         <v>140</v>
       </c>
       <c r="D380" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E380" t="s">
         <v>644</v>
@@ -37499,10 +37526,10 @@
         <v>42736</v>
       </c>
       <c r="C381" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="D381" t="s">
-        <v>239</v>
+        <v>446</v>
       </c>
       <c r="E381" t="s">
         <v>644</v>
@@ -37519,7 +37546,7 @@
         <v>149</v>
       </c>
       <c r="D382" t="s">
-        <v>51</v>
+        <v>239</v>
       </c>
       <c r="E382" t="s">
         <v>644</v>
@@ -37539,7 +37566,7 @@
         <v>51</v>
       </c>
       <c r="E383" t="s">
-        <v>718</v>
+        <v>644</v>
       </c>
       <c r="F383" t="s">
         <v>643</v>
@@ -37550,13 +37577,13 @@
         <v>42736</v>
       </c>
       <c r="C384" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D384" t="s">
-        <v>239</v>
+        <v>51</v>
       </c>
       <c r="E384" t="s">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="F384" t="s">
         <v>643</v>
@@ -37570,7 +37597,7 @@
         <v>150</v>
       </c>
       <c r="D385" t="s">
-        <v>141</v>
+        <v>239</v>
       </c>
       <c r="E385" t="s">
         <v>710</v>
@@ -37587,7 +37614,7 @@
         <v>150</v>
       </c>
       <c r="D386" t="s">
-        <v>436</v>
+        <v>141</v>
       </c>
       <c r="E386" t="s">
         <v>710</v>
@@ -37604,7 +37631,7 @@
         <v>150</v>
       </c>
       <c r="D387" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E387" t="s">
         <v>710</v>
@@ -37621,7 +37648,7 @@
         <v>150</v>
       </c>
       <c r="D388" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E388" t="s">
         <v>710</v>
@@ -37638,7 +37665,7 @@
         <v>150</v>
       </c>
       <c r="D389" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E389" t="s">
         <v>710</v>
@@ -37655,7 +37682,7 @@
         <v>150</v>
       </c>
       <c r="D390" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E390" t="s">
         <v>710</v>
@@ -37672,7 +37699,7 @@
         <v>150</v>
       </c>
       <c r="D391" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E391" t="s">
         <v>710</v>
@@ -37689,10 +37716,10 @@
         <v>150</v>
       </c>
       <c r="D392" t="s">
-        <v>239</v>
+        <v>446</v>
       </c>
       <c r="E392" t="s">
-        <v>735</v>
+        <v>710</v>
       </c>
       <c r="F392" t="s">
         <v>643</v>
@@ -37706,7 +37733,7 @@
         <v>150</v>
       </c>
       <c r="D393" t="s">
-        <v>141</v>
+        <v>239</v>
       </c>
       <c r="E393" t="s">
         <v>735</v>
@@ -37723,7 +37750,7 @@
         <v>150</v>
       </c>
       <c r="D394" t="s">
-        <v>436</v>
+        <v>141</v>
       </c>
       <c r="E394" t="s">
         <v>735</v>
@@ -37740,7 +37767,7 @@
         <v>150</v>
       </c>
       <c r="D395" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E395" t="s">
         <v>735</v>
@@ -37757,7 +37784,7 @@
         <v>150</v>
       </c>
       <c r="D396" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E396" t="s">
         <v>735</v>
@@ -37774,7 +37801,7 @@
         <v>150</v>
       </c>
       <c r="D397" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E397" t="s">
         <v>735</v>
@@ -37791,7 +37818,7 @@
         <v>150</v>
       </c>
       <c r="D398" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E398" t="s">
         <v>735</v>
@@ -37808,7 +37835,7 @@
         <v>150</v>
       </c>
       <c r="D399" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E399" t="s">
         <v>735</v>
@@ -37825,10 +37852,10 @@
         <v>150</v>
       </c>
       <c r="D400" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
       <c r="E400" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="F400" t="s">
         <v>643</v>
@@ -37842,7 +37869,7 @@
         <v>150</v>
       </c>
       <c r="D401" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E401" t="s">
         <v>736</v>
@@ -37859,7 +37886,7 @@
         <v>150</v>
       </c>
       <c r="D402" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E402" t="s">
         <v>736</v>
@@ -37876,7 +37903,7 @@
         <v>150</v>
       </c>
       <c r="D403" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E403" t="s">
         <v>736</v>
@@ -37893,10 +37920,10 @@
         <v>150</v>
       </c>
       <c r="D404" t="s">
-        <v>239</v>
+        <v>446</v>
       </c>
       <c r="E404" t="s">
-        <v>644</v>
+        <v>736</v>
       </c>
       <c r="F404" t="s">
         <v>643</v>
@@ -37910,7 +37937,7 @@
         <v>150</v>
       </c>
       <c r="D405" t="s">
-        <v>141</v>
+        <v>239</v>
       </c>
       <c r="E405" t="s">
         <v>644</v>
@@ -37927,7 +37954,7 @@
         <v>150</v>
       </c>
       <c r="D406" t="s">
-        <v>436</v>
+        <v>141</v>
       </c>
       <c r="E406" t="s">
         <v>644</v>
@@ -37944,7 +37971,7 @@
         <v>150</v>
       </c>
       <c r="D407" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E407" t="s">
         <v>644</v>
@@ -37961,7 +37988,7 @@
         <v>150</v>
       </c>
       <c r="D408" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E408" t="s">
         <v>644</v>
@@ -37978,7 +38005,7 @@
         <v>150</v>
       </c>
       <c r="D409" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E409" t="s">
         <v>644</v>
@@ -37995,7 +38022,7 @@
         <v>150</v>
       </c>
       <c r="D410" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E410" t="s">
         <v>644</v>
@@ -38012,7 +38039,7 @@
         <v>150</v>
       </c>
       <c r="D411" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E411" t="s">
         <v>644</v>
@@ -38026,13 +38053,13 @@
         <v>42736</v>
       </c>
       <c r="C412" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D412" t="s">
-        <v>239</v>
+        <v>446</v>
       </c>
       <c r="E412" t="s">
-        <v>710</v>
+        <v>644</v>
       </c>
       <c r="F412" t="s">
         <v>643</v>
@@ -38046,7 +38073,7 @@
         <v>151</v>
       </c>
       <c r="D413" t="s">
-        <v>141</v>
+        <v>239</v>
       </c>
       <c r="E413" t="s">
         <v>710</v>
@@ -38063,7 +38090,7 @@
         <v>151</v>
       </c>
       <c r="D414" t="s">
-        <v>436</v>
+        <v>141</v>
       </c>
       <c r="E414" t="s">
         <v>710</v>
@@ -38080,7 +38107,7 @@
         <v>151</v>
       </c>
       <c r="D415" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E415" t="s">
         <v>710</v>
@@ -38097,7 +38124,7 @@
         <v>151</v>
       </c>
       <c r="D416" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E416" t="s">
         <v>710</v>
@@ -38114,7 +38141,7 @@
         <v>151</v>
       </c>
       <c r="D417" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E417" t="s">
         <v>710</v>
@@ -38131,7 +38158,7 @@
         <v>151</v>
       </c>
       <c r="D418" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E418" t="s">
         <v>710</v>
@@ -38148,7 +38175,7 @@
         <v>151</v>
       </c>
       <c r="D419" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E419" t="s">
         <v>710</v>
@@ -38165,10 +38192,10 @@
         <v>151</v>
       </c>
       <c r="D420" t="s">
-        <v>239</v>
+        <v>446</v>
       </c>
       <c r="E420" t="s">
-        <v>735</v>
+        <v>710</v>
       </c>
       <c r="F420" t="s">
         <v>643</v>
@@ -38182,7 +38209,7 @@
         <v>151</v>
       </c>
       <c r="D421" t="s">
-        <v>141</v>
+        <v>239</v>
       </c>
       <c r="E421" t="s">
         <v>735</v>
@@ -38199,7 +38226,7 @@
         <v>151</v>
       </c>
       <c r="D422" t="s">
-        <v>436</v>
+        <v>141</v>
       </c>
       <c r="E422" t="s">
         <v>735</v>
@@ -38216,7 +38243,7 @@
         <v>151</v>
       </c>
       <c r="D423" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E423" t="s">
         <v>735</v>
@@ -38233,7 +38260,7 @@
         <v>151</v>
       </c>
       <c r="D424" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E424" t="s">
         <v>735</v>
@@ -38250,7 +38277,7 @@
         <v>151</v>
       </c>
       <c r="D425" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E425" t="s">
         <v>735</v>
@@ -38267,7 +38294,7 @@
         <v>151</v>
       </c>
       <c r="D426" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E426" t="s">
         <v>735</v>
@@ -38284,7 +38311,7 @@
         <v>151</v>
       </c>
       <c r="D427" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E427" t="s">
         <v>735</v>
@@ -38301,10 +38328,10 @@
         <v>151</v>
       </c>
       <c r="D428" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
       <c r="E428" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="F428" t="s">
         <v>643</v>
@@ -38318,7 +38345,7 @@
         <v>151</v>
       </c>
       <c r="D429" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E429" t="s">
         <v>736</v>
@@ -38335,7 +38362,7 @@
         <v>151</v>
       </c>
       <c r="D430" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E430" t="s">
         <v>736</v>
@@ -38352,7 +38379,7 @@
         <v>151</v>
       </c>
       <c r="D431" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E431" t="s">
         <v>736</v>
@@ -38369,10 +38396,10 @@
         <v>151</v>
       </c>
       <c r="D432" t="s">
-        <v>239</v>
+        <v>446</v>
       </c>
       <c r="E432" t="s">
-        <v>644</v>
+        <v>736</v>
       </c>
       <c r="F432" t="s">
         <v>643</v>
@@ -38386,7 +38413,7 @@
         <v>151</v>
       </c>
       <c r="D433" t="s">
-        <v>141</v>
+        <v>239</v>
       </c>
       <c r="E433" t="s">
         <v>644</v>
@@ -38403,7 +38430,7 @@
         <v>151</v>
       </c>
       <c r="D434" t="s">
-        <v>436</v>
+        <v>141</v>
       </c>
       <c r="E434" t="s">
         <v>644</v>
@@ -38420,7 +38447,7 @@
         <v>151</v>
       </c>
       <c r="D435" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E435" t="s">
         <v>644</v>
@@ -38437,7 +38464,7 @@
         <v>151</v>
       </c>
       <c r="D436" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E436" t="s">
         <v>644</v>
@@ -38454,7 +38481,7 @@
         <v>151</v>
       </c>
       <c r="D437" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E437" t="s">
         <v>644</v>
@@ -38471,7 +38498,7 @@
         <v>151</v>
       </c>
       <c r="D438" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E438" t="s">
         <v>644</v>
@@ -38488,7 +38515,7 @@
         <v>151</v>
       </c>
       <c r="D439" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E439" t="s">
         <v>644</v>
@@ -38502,10 +38529,10 @@
         <v>42736</v>
       </c>
       <c r="C440" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D440" t="s">
-        <v>47</v>
+        <v>446</v>
       </c>
       <c r="E440" t="s">
         <v>644</v>
@@ -38525,7 +38552,7 @@
         <v>47</v>
       </c>
       <c r="E441" t="s">
-        <v>735</v>
+        <v>644</v>
       </c>
       <c r="F441" t="s">
         <v>643</v>
@@ -38536,13 +38563,13 @@
         <v>42736</v>
       </c>
       <c r="C442" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D442" t="s">
         <v>47</v>
       </c>
       <c r="E442" t="s">
-        <v>644</v>
+        <v>735</v>
       </c>
       <c r="F442" t="s">
         <v>643</v>
@@ -38553,10 +38580,10 @@
         <v>42736</v>
       </c>
       <c r="C443" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D443" t="s">
-        <v>239</v>
+        <v>47</v>
       </c>
       <c r="E443" t="s">
         <v>644</v>
@@ -38573,7 +38600,7 @@
         <v>154</v>
       </c>
       <c r="D444" t="s">
-        <v>51</v>
+        <v>239</v>
       </c>
       <c r="E444" t="s">
         <v>644</v>
@@ -38593,7 +38620,7 @@
         <v>51</v>
       </c>
       <c r="E445" t="s">
-        <v>718</v>
+        <v>644</v>
       </c>
       <c r="F445" t="s">
         <v>643</v>
@@ -38604,13 +38631,13 @@
         <v>42736</v>
       </c>
       <c r="C446" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D446" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E446" t="s">
-        <v>644</v>
+        <v>718</v>
       </c>
       <c r="F446" t="s">
         <v>643</v>
@@ -38621,7 +38648,7 @@
         <v>42736</v>
       </c>
       <c r="C447" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D447" t="s">
         <v>47</v>
@@ -38641,7 +38668,7 @@
         <v>156</v>
       </c>
       <c r="D448" t="s">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="E448" t="s">
         <v>644</v>
@@ -38655,13 +38682,13 @@
         <v>42736</v>
       </c>
       <c r="C449" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D449" t="s">
-        <v>450</v>
+        <v>13</v>
       </c>
       <c r="E449" t="s">
-        <v>665</v>
+        <v>644</v>
       </c>
       <c r="F449" t="s">
         <v>643</v>
@@ -38678,10 +38705,10 @@
         <v>450</v>
       </c>
       <c r="E450" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="F450" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
     </row>
     <row r="451" spans="1:6" x14ac:dyDescent="0.2">
@@ -38692,13 +38719,13 @@
         <v>157</v>
       </c>
       <c r="D451" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="E451" t="s">
         <v>667</v>
       </c>
       <c r="F451" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
     </row>
     <row r="452" spans="1:6" x14ac:dyDescent="0.2">
@@ -38709,7 +38736,7 @@
         <v>157</v>
       </c>
       <c r="D452" t="s">
-        <v>158</v>
+        <v>447</v>
       </c>
       <c r="E452" t="s">
         <v>667</v>
@@ -38726,10 +38753,10 @@
         <v>157</v>
       </c>
       <c r="D453" t="s">
-        <v>447</v>
+        <v>158</v>
       </c>
       <c r="E453" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="F453" t="s">
         <v>643</v>
@@ -38743,7 +38770,7 @@
         <v>157</v>
       </c>
       <c r="D454" t="s">
-        <v>158</v>
+        <v>447</v>
       </c>
       <c r="E454" t="s">
         <v>665</v>
@@ -38757,13 +38784,13 @@
         <v>42736</v>
       </c>
       <c r="C455" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D455" t="s">
-        <v>47</v>
+        <v>158</v>
       </c>
       <c r="E455" t="s">
-        <v>710</v>
+        <v>665</v>
       </c>
       <c r="F455" t="s">
         <v>643</v>
@@ -38780,10 +38807,10 @@
         <v>47</v>
       </c>
       <c r="E456" t="s">
-        <v>714</v>
+        <v>710</v>
       </c>
       <c r="F456" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
     </row>
     <row r="457" spans="1:6" x14ac:dyDescent="0.2">
@@ -38791,16 +38818,16 @@
         <v>42736</v>
       </c>
       <c r="C457" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D457" t="s">
         <v>47</v>
       </c>
       <c r="E457" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="F457" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
     </row>
     <row r="458" spans="1:6" x14ac:dyDescent="0.2">
@@ -38814,10 +38841,10 @@
         <v>47</v>
       </c>
       <c r="E458" t="s">
-        <v>714</v>
+        <v>710</v>
       </c>
       <c r="F458" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
     </row>
     <row r="459" spans="1:6" x14ac:dyDescent="0.2">
@@ -38825,16 +38852,16 @@
         <v>42736</v>
       </c>
       <c r="C459" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D459" t="s">
-        <v>239</v>
+        <v>47</v>
       </c>
       <c r="E459" t="s">
-        <v>644</v>
+        <v>714</v>
       </c>
       <c r="F459" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
     </row>
     <row r="460" spans="1:6" x14ac:dyDescent="0.2">
@@ -38845,7 +38872,7 @@
         <v>161</v>
       </c>
       <c r="D460" t="s">
-        <v>51</v>
+        <v>239</v>
       </c>
       <c r="E460" t="s">
         <v>644</v>
@@ -38865,7 +38892,7 @@
         <v>51</v>
       </c>
       <c r="E461" t="s">
-        <v>718</v>
+        <v>644</v>
       </c>
       <c r="F461" t="s">
         <v>643</v>
@@ -38873,16 +38900,16 @@
     </row>
     <row r="462" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A462" s="1">
-        <v>42741</v>
+        <v>42736</v>
       </c>
       <c r="C462" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D462" t="s">
-        <v>163</v>
+        <v>51</v>
       </c>
       <c r="E462" t="s">
-        <v>644</v>
+        <v>718</v>
       </c>
       <c r="F462" t="s">
         <v>643</v>
@@ -38890,13 +38917,13 @@
     </row>
     <row r="463" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A463" s="1">
-        <v>42742</v>
+        <v>42741</v>
       </c>
       <c r="C463" t="s">
         <v>162</v>
       </c>
       <c r="D463" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E463" t="s">
         <v>644</v>
@@ -38907,13 +38934,13 @@
     </row>
     <row r="464" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A464" s="1">
-        <v>42743</v>
+        <v>42742</v>
       </c>
       <c r="C464" t="s">
         <v>162</v>
       </c>
       <c r="D464" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="E464" t="s">
         <v>644</v>
@@ -38924,13 +38951,13 @@
     </row>
     <row r="465" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A465" s="1">
-        <v>42744</v>
+        <v>42743</v>
       </c>
       <c r="C465" t="s">
         <v>162</v>
       </c>
       <c r="D465" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E465" t="s">
         <v>644</v>
@@ -38941,13 +38968,13 @@
     </row>
     <row r="466" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A466" s="1">
-        <v>42745</v>
+        <v>42744</v>
       </c>
       <c r="C466" t="s">
         <v>162</v>
       </c>
       <c r="D466" t="s">
-        <v>456</v>
+        <v>169</v>
       </c>
       <c r="E466" t="s">
         <v>644</v>
@@ -38958,13 +38985,13 @@
     </row>
     <row r="467" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A467" s="1">
-        <v>42741</v>
+        <v>42745</v>
       </c>
       <c r="C467" t="s">
         <v>162</v>
       </c>
       <c r="D467" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="E467" t="s">
         <v>644</v>
@@ -38975,13 +39002,13 @@
     </row>
     <row r="468" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A468" s="1">
-        <v>42742</v>
+        <v>42741</v>
       </c>
       <c r="C468" t="s">
         <v>162</v>
       </c>
       <c r="D468" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="E468" t="s">
         <v>644</v>
@@ -38992,13 +39019,13 @@
     </row>
     <row r="469" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A469" s="1">
-        <v>42743</v>
+        <v>42742</v>
       </c>
       <c r="C469" t="s">
         <v>162</v>
       </c>
       <c r="D469" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="E469" t="s">
         <v>644</v>
@@ -39009,64 +39036,64 @@
     </row>
     <row r="470" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A470" s="1">
-        <v>42746</v>
+        <v>42743</v>
       </c>
       <c r="C470" t="s">
         <v>162</v>
       </c>
       <c r="D470" t="s">
-        <v>163</v>
+        <v>463</v>
       </c>
       <c r="E470" t="s">
-        <v>727</v>
+        <v>644</v>
       </c>
       <c r="F470" t="s">
-        <v>716</v>
+        <v>643</v>
       </c>
     </row>
     <row r="471" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A471" s="1">
-        <v>42747</v>
+        <v>42746</v>
       </c>
       <c r="C471" t="s">
         <v>162</v>
       </c>
       <c r="D471" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E471" t="s">
         <v>727</v>
       </c>
       <c r="F471" t="s">
-        <v>663</v>
+        <v>716</v>
       </c>
     </row>
     <row r="472" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A472" s="1">
-        <v>42748</v>
+        <v>42747</v>
       </c>
       <c r="C472" t="s">
         <v>162</v>
       </c>
       <c r="D472" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="E472" t="s">
         <v>727</v>
       </c>
       <c r="F472" t="s">
-        <v>716</v>
+        <v>663</v>
       </c>
     </row>
     <row r="473" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A473" s="1">
-        <v>42749</v>
+        <v>42748</v>
       </c>
       <c r="C473" t="s">
         <v>162</v>
       </c>
       <c r="D473" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E473" t="s">
         <v>727</v>
@@ -39077,13 +39104,13 @@
     </row>
     <row r="474" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A474" s="1">
-        <v>42750</v>
+        <v>42749</v>
       </c>
       <c r="C474" t="s">
         <v>162</v>
       </c>
       <c r="D474" t="s">
-        <v>456</v>
+        <v>169</v>
       </c>
       <c r="E474" t="s">
         <v>727</v>
@@ -39094,13 +39121,13 @@
     </row>
     <row r="475" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A475" s="1">
-        <v>42741</v>
+        <v>42750</v>
       </c>
       <c r="C475" t="s">
         <v>162</v>
       </c>
       <c r="D475" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="E475" t="s">
         <v>727</v>
@@ -39111,13 +39138,13 @@
     </row>
     <row r="476" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A476" s="1">
-        <v>42742</v>
+        <v>42741</v>
       </c>
       <c r="C476" t="s">
         <v>162</v>
       </c>
       <c r="D476" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="E476" t="s">
         <v>727</v>
@@ -39128,18 +39155,35 @@
     </row>
     <row r="477" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A477" s="1">
-        <v>42743</v>
+        <v>42742</v>
       </c>
       <c r="C477" t="s">
         <v>162</v>
       </c>
       <c r="D477" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="E477" t="s">
         <v>727</v>
       </c>
       <c r="F477" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="478" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A478" s="1">
+        <v>42743</v>
+      </c>
+      <c r="C478" t="s">
+        <v>162</v>
+      </c>
+      <c r="D478" t="s">
+        <v>463</v>
+      </c>
+      <c r="E478" t="s">
+        <v>727</v>
+      </c>
+      <c r="F478" t="s">
         <v>716</v>
       </c>
     </row>
@@ -39150,10 +39194,16 @@
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
-  <dimension ref="A1:V361"/>
+  <dimension ref="A1:V363"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="26.1640625" customWidth="1"/>
+    <col min="5" max="5" width="30.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="19.33203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="15" max="15" width="20.1640625" customWidth="1"/>
+    <col min="16" max="16" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.2">
@@ -49206,68 +49256,68 @@
         <v>700</v>
       </c>
     </row>
-    <row r="311" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:16" ht="18" x14ac:dyDescent="0.25">
       <c r="A311" s="1">
-        <v>42736</v>
+        <v>42746</v>
       </c>
       <c r="C311" t="s">
-        <v>138</v>
+        <v>114</v>
       </c>
       <c r="D311" t="s">
         <v>748</v>
       </c>
       <c r="E311" t="s">
-        <v>47</v>
+        <v>1537</v>
       </c>
       <c r="F311">
         <v>1</v>
       </c>
       <c r="G311" t="s">
-        <v>1252</v>
+        <v>1178</v>
       </c>
       <c r="H311" t="s">
         <v>1253</v>
       </c>
       <c r="I311" t="s">
-        <v>1314</v>
-      </c>
-      <c r="J311">
-        <v>1</v>
+        <v>1539</v>
+      </c>
+      <c r="O311" s="3" t="s">
+        <v>1540</v>
       </c>
       <c r="P311" t="s">
-        <v>405</v>
+        <v>700</v>
       </c>
     </row>
     <row r="312" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A312" s="1">
-        <v>42736</v>
+        <v>42746</v>
       </c>
       <c r="C312" t="s">
-        <v>139</v>
+        <v>114</v>
       </c>
       <c r="D312" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="E312" t="s">
-        <v>47</v>
+        <v>1537</v>
       </c>
       <c r="F312">
         <v>1</v>
       </c>
       <c r="G312" t="s">
-        <v>1252</v>
+        <v>1178</v>
       </c>
       <c r="H312" t="s">
         <v>1253</v>
       </c>
       <c r="I312" t="s">
-        <v>1314</v>
-      </c>
-      <c r="J312">
-        <v>1</v>
+        <v>1539</v>
+      </c>
+      <c r="O312" t="s">
+        <v>1541</v>
       </c>
       <c r="P312" t="s">
-        <v>405</v>
+        <v>700</v>
       </c>
     </row>
     <row r="313" spans="1:16" x14ac:dyDescent="0.2">
@@ -49275,10 +49325,10 @@
         <v>42736</v>
       </c>
       <c r="C313" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D313" t="s">
-        <v>782</v>
+        <v>748</v>
       </c>
       <c r="E313" t="s">
         <v>47</v>
@@ -49307,25 +49357,25 @@
         <v>42736</v>
       </c>
       <c r="C314" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D314" t="s">
         <v>748</v>
       </c>
       <c r="E314" t="s">
-        <v>141</v>
+        <v>47</v>
       </c>
       <c r="F314">
         <v>1</v>
       </c>
       <c r="G314" t="s">
-        <v>1178</v>
+        <v>1252</v>
       </c>
       <c r="H314" t="s">
         <v>1253</v>
       </c>
       <c r="I314" t="s">
-        <v>1254</v>
+        <v>1314</v>
       </c>
       <c r="J314">
         <v>1</v>
@@ -49339,25 +49389,25 @@
         <v>42736</v>
       </c>
       <c r="C315" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D315" t="s">
-        <v>748</v>
+        <v>782</v>
       </c>
       <c r="E315" t="s">
-        <v>436</v>
+        <v>47</v>
       </c>
       <c r="F315">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G315" t="s">
-        <v>1178</v>
+        <v>1252</v>
       </c>
       <c r="H315" t="s">
         <v>1253</v>
       </c>
       <c r="I315" t="s">
-        <v>1254</v>
+        <v>1314</v>
       </c>
       <c r="J315">
         <v>1</v>
@@ -49377,10 +49427,10 @@
         <v>748</v>
       </c>
       <c r="E316" t="s">
-        <v>438</v>
+        <v>141</v>
       </c>
       <c r="F316">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G316" t="s">
         <v>1178</v>
@@ -49403,16 +49453,16 @@
         <v>42736</v>
       </c>
       <c r="C317" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="D317" t="s">
-        <v>740</v>
+        <v>748</v>
       </c>
       <c r="E317" t="s">
-        <v>51</v>
+        <v>436</v>
       </c>
       <c r="F317">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G317" t="s">
         <v>1178</v>
@@ -49435,16 +49485,16 @@
         <v>42736</v>
       </c>
       <c r="C318" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="D318" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="E318" t="s">
-        <v>51</v>
+        <v>438</v>
       </c>
       <c r="F318">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G318" t="s">
         <v>1178</v>
@@ -49467,13 +49517,13 @@
         <v>42736</v>
       </c>
       <c r="C319" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D319" t="s">
-        <v>748</v>
+        <v>740</v>
       </c>
       <c r="E319" t="s">
-        <v>141</v>
+        <v>51</v>
       </c>
       <c r="F319">
         <v>1</v>
@@ -49499,16 +49549,16 @@
         <v>42736</v>
       </c>
       <c r="C320" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D320" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
       <c r="E320" t="s">
-        <v>436</v>
+        <v>51</v>
       </c>
       <c r="F320">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G320" t="s">
         <v>1178</v>
@@ -49537,10 +49587,10 @@
         <v>748</v>
       </c>
       <c r="E321" t="s">
-        <v>438</v>
+        <v>141</v>
       </c>
       <c r="F321">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G321" t="s">
         <v>1178</v>
@@ -49560,25 +49610,25 @@
     </row>
     <row r="322" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A322" s="1">
-        <v>42756</v>
+        <v>42736</v>
       </c>
       <c r="C322" t="s">
         <v>150</v>
       </c>
       <c r="D322" t="s">
-        <v>827</v>
+        <v>748</v>
       </c>
       <c r="E322" t="s">
-        <v>442</v>
+        <v>436</v>
       </c>
       <c r="F322">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G322" t="s">
-        <v>1258</v>
+        <v>1178</v>
       </c>
       <c r="H322" t="s">
-        <v>1322</v>
+        <v>1253</v>
       </c>
       <c r="I322" t="s">
         <v>1254</v>
@@ -49592,25 +49642,25 @@
     </row>
     <row r="323" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A323" s="1">
-        <v>42756</v>
+        <v>42736</v>
       </c>
       <c r="C323" t="s">
         <v>150</v>
       </c>
       <c r="D323" t="s">
-        <v>827</v>
+        <v>748</v>
       </c>
       <c r="E323" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="F323">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G323" t="s">
-        <v>1258</v>
+        <v>1178</v>
       </c>
       <c r="H323" t="s">
-        <v>1322</v>
+        <v>1253</v>
       </c>
       <c r="I323" t="s">
         <v>1254</v>
@@ -49633,10 +49683,10 @@
         <v>827</v>
       </c>
       <c r="E324" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="F324">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G324" t="s">
         <v>1258</v>
@@ -49656,28 +49706,28 @@
     </row>
     <row r="325" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A325" s="1">
-        <v>42736</v>
+        <v>42756</v>
       </c>
       <c r="C325" t="s">
         <v>150</v>
       </c>
       <c r="D325" t="s">
-        <v>825</v>
+        <v>827</v>
       </c>
       <c r="E325" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
       <c r="F325">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G325" t="s">
         <v>1258</v>
       </c>
       <c r="H325" t="s">
-        <v>1272</v>
+        <v>1322</v>
       </c>
       <c r="I325" t="s">
-        <v>293</v>
+        <v>1254</v>
       </c>
       <c r="J325">
         <v>1</v>
@@ -49688,28 +49738,28 @@
     </row>
     <row r="326" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A326" s="1">
-        <v>42736</v>
+        <v>42756</v>
       </c>
       <c r="C326" t="s">
         <v>150</v>
       </c>
       <c r="D326" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="E326" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="F326">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G326" t="s">
         <v>1258</v>
       </c>
       <c r="H326" t="s">
-        <v>1272</v>
+        <v>1322</v>
       </c>
       <c r="I326" t="s">
-        <v>293</v>
+        <v>1254</v>
       </c>
       <c r="J326">
         <v>1</v>
@@ -49726,13 +49776,13 @@
         <v>150</v>
       </c>
       <c r="D327" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="E327" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="F327">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G327" t="s">
         <v>1258</v>
@@ -49761,10 +49811,10 @@
         <v>826</v>
       </c>
       <c r="E328" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="F328">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G328" t="s">
         <v>1258</v>
@@ -49793,10 +49843,10 @@
         <v>826</v>
       </c>
       <c r="E329" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="F329">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G329" t="s">
         <v>1258</v>
@@ -49819,25 +49869,25 @@
         <v>42736</v>
       </c>
       <c r="C330" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D330" t="s">
-        <v>748</v>
+        <v>826</v>
       </c>
       <c r="E330" t="s">
-        <v>141</v>
+        <v>444</v>
       </c>
       <c r="F330">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G330" t="s">
-        <v>1178</v>
+        <v>1258</v>
       </c>
       <c r="H330" t="s">
-        <v>1253</v>
+        <v>1272</v>
       </c>
       <c r="I330" t="s">
-        <v>1254</v>
+        <v>293</v>
       </c>
       <c r="J330">
         <v>1</v>
@@ -49851,25 +49901,25 @@
         <v>42736</v>
       </c>
       <c r="C331" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D331" t="s">
-        <v>748</v>
+        <v>826</v>
       </c>
       <c r="E331" t="s">
-        <v>436</v>
+        <v>446</v>
       </c>
       <c r="F331">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G331" t="s">
-        <v>1178</v>
+        <v>1258</v>
       </c>
       <c r="H331" t="s">
-        <v>1253</v>
+        <v>1272</v>
       </c>
       <c r="I331" t="s">
-        <v>1254</v>
+        <v>293</v>
       </c>
       <c r="J331">
         <v>1</v>
@@ -49889,10 +49939,10 @@
         <v>748</v>
       </c>
       <c r="E332" t="s">
-        <v>438</v>
+        <v>141</v>
       </c>
       <c r="F332">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G332" t="s">
         <v>1178</v>
@@ -49918,22 +49968,22 @@
         <v>151</v>
       </c>
       <c r="D333" t="s">
-        <v>828</v>
+        <v>748</v>
       </c>
       <c r="E333" t="s">
-        <v>446</v>
+        <v>436</v>
       </c>
       <c r="F333">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G333" t="s">
-        <v>1258</v>
+        <v>1178</v>
       </c>
       <c r="H333" t="s">
-        <v>1272</v>
+        <v>1253</v>
       </c>
       <c r="I333" t="s">
-        <v>293</v>
+        <v>1254</v>
       </c>
       <c r="J333">
         <v>1</v>
@@ -49950,22 +50000,22 @@
         <v>151</v>
       </c>
       <c r="D334" t="s">
-        <v>826</v>
+        <v>748</v>
       </c>
       <c r="E334" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="F334">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G334" t="s">
-        <v>1258</v>
+        <v>1178</v>
       </c>
       <c r="H334" t="s">
-        <v>1272</v>
+        <v>1253</v>
       </c>
       <c r="I334" t="s">
-        <v>293</v>
+        <v>1254</v>
       </c>
       <c r="J334">
         <v>1</v>
@@ -49982,13 +50032,13 @@
         <v>151</v>
       </c>
       <c r="D335" t="s">
-        <v>826</v>
+        <v>828</v>
       </c>
       <c r="E335" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="F335">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G335" t="s">
         <v>1258</v>
@@ -50017,10 +50067,10 @@
         <v>826</v>
       </c>
       <c r="E336" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="F336">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G336" t="s">
         <v>1258</v>
@@ -50049,10 +50099,10 @@
         <v>826</v>
       </c>
       <c r="E337" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="F337">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G337" t="s">
         <v>1258</v>
@@ -50075,25 +50125,25 @@
         <v>42736</v>
       </c>
       <c r="C338" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D338" t="s">
-        <v>748</v>
+        <v>826</v>
       </c>
       <c r="E338" t="s">
-        <v>47</v>
+        <v>444</v>
       </c>
       <c r="F338">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G338" t="s">
-        <v>1252</v>
+        <v>1258</v>
       </c>
       <c r="H338" t="s">
-        <v>1253</v>
+        <v>1272</v>
       </c>
       <c r="I338" t="s">
-        <v>1314</v>
+        <v>293</v>
       </c>
       <c r="J338">
         <v>1</v>
@@ -50107,25 +50157,25 @@
         <v>42736</v>
       </c>
       <c r="C339" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D339" t="s">
-        <v>748</v>
+        <v>826</v>
       </c>
       <c r="E339" t="s">
-        <v>47</v>
+        <v>446</v>
       </c>
       <c r="F339">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G339" t="s">
-        <v>1252</v>
+        <v>1258</v>
       </c>
       <c r="H339" t="s">
-        <v>1253</v>
+        <v>1272</v>
       </c>
       <c r="I339" t="s">
-        <v>1314</v>
+        <v>293</v>
       </c>
       <c r="J339">
         <v>1</v>
@@ -50139,25 +50189,25 @@
         <v>42736</v>
       </c>
       <c r="C340" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D340" t="s">
-        <v>740</v>
+        <v>748</v>
       </c>
       <c r="E340" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F340">
         <v>1</v>
       </c>
       <c r="G340" t="s">
-        <v>1178</v>
+        <v>1252</v>
       </c>
       <c r="H340" t="s">
         <v>1253</v>
       </c>
       <c r="I340" t="s">
-        <v>1254</v>
+        <v>1314</v>
       </c>
       <c r="J340">
         <v>1</v>
@@ -50171,25 +50221,25 @@
         <v>42736</v>
       </c>
       <c r="C341" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D341" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="E341" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F341">
         <v>1</v>
       </c>
       <c r="G341" t="s">
-        <v>1178</v>
+        <v>1252</v>
       </c>
       <c r="H341" t="s">
         <v>1253</v>
       </c>
       <c r="I341" t="s">
-        <v>1254</v>
+        <v>1314</v>
       </c>
       <c r="J341">
         <v>1</v>
@@ -50203,13 +50253,13 @@
         <v>42736</v>
       </c>
       <c r="C342" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D342" t="s">
         <v>740</v>
       </c>
       <c r="E342" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F342">
         <v>1</v>
@@ -50235,13 +50285,13 @@
         <v>42736</v>
       </c>
       <c r="C343" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D343" t="s">
-        <v>829</v>
+        <v>744</v>
       </c>
       <c r="E343" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F343">
         <v>1</v>
@@ -50270,7 +50320,7 @@
         <v>155</v>
       </c>
       <c r="D344" t="s">
-        <v>830</v>
+        <v>740</v>
       </c>
       <c r="E344" t="s">
         <v>47</v>
@@ -50299,10 +50349,10 @@
         <v>42736</v>
       </c>
       <c r="C345" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D345" t="s">
-        <v>748</v>
+        <v>829</v>
       </c>
       <c r="E345" t="s">
         <v>47</v>
@@ -50311,7 +50361,7 @@
         <v>1</v>
       </c>
       <c r="G345" t="s">
-        <v>1252</v>
+        <v>1178</v>
       </c>
       <c r="H345" t="s">
         <v>1253</v>
@@ -50331,19 +50381,19 @@
         <v>42736</v>
       </c>
       <c r="C346" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D346" t="s">
-        <v>748</v>
+        <v>830</v>
       </c>
       <c r="E346" t="s">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="F346">
         <v>1</v>
       </c>
       <c r="G346" t="s">
-        <v>1252</v>
+        <v>1178</v>
       </c>
       <c r="H346" t="s">
         <v>1253</v>
@@ -50363,19 +50413,19 @@
         <v>42736</v>
       </c>
       <c r="C347" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D347" t="s">
         <v>748</v>
       </c>
       <c r="E347" t="s">
-        <v>447</v>
+        <v>47</v>
       </c>
       <c r="F347">
         <v>1</v>
       </c>
       <c r="G347" t="s">
-        <v>1258</v>
+        <v>1252</v>
       </c>
       <c r="H347" t="s">
         <v>1253</v>
@@ -50395,19 +50445,19 @@
         <v>42736</v>
       </c>
       <c r="C348" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D348" t="s">
         <v>748</v>
       </c>
       <c r="E348" t="s">
-        <v>450</v>
+        <v>13</v>
       </c>
       <c r="F348">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G348" t="s">
-        <v>1258</v>
+        <v>1252</v>
       </c>
       <c r="H348" t="s">
         <v>1253</v>
@@ -50416,7 +50466,7 @@
         <v>1254</v>
       </c>
       <c r="J348">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P348" t="s">
         <v>405</v>
@@ -50430,7 +50480,7 @@
         <v>157</v>
       </c>
       <c r="D349" t="s">
-        <v>831</v>
+        <v>748</v>
       </c>
       <c r="E349" t="s">
         <v>447</v>
@@ -50462,7 +50512,7 @@
         <v>157</v>
       </c>
       <c r="D350" t="s">
-        <v>831</v>
+        <v>748</v>
       </c>
       <c r="E350" t="s">
         <v>450</v>
@@ -50494,7 +50544,7 @@
         <v>157</v>
       </c>
       <c r="D351" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E351" t="s">
         <v>447</v>
@@ -50523,19 +50573,19 @@
         <v>42736</v>
       </c>
       <c r="C352" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="D352" t="s">
-        <v>740</v>
+        <v>831</v>
       </c>
       <c r="E352" t="s">
-        <v>51</v>
+        <v>450</v>
       </c>
       <c r="F352">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G352" t="s">
-        <v>1178</v>
+        <v>1258</v>
       </c>
       <c r="H352" t="s">
         <v>1253</v>
@@ -50544,7 +50594,7 @@
         <v>1254</v>
       </c>
       <c r="J352">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P352" t="s">
         <v>405</v>
@@ -50555,19 +50605,19 @@
         <v>42736</v>
       </c>
       <c r="C353" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="D353" t="s">
-        <v>744</v>
+        <v>832</v>
       </c>
       <c r="E353" t="s">
-        <v>51</v>
+        <v>447</v>
       </c>
       <c r="F353">
         <v>1</v>
       </c>
       <c r="G353" t="s">
-        <v>1178</v>
+        <v>1258</v>
       </c>
       <c r="H353" t="s">
         <v>1253</v>
@@ -50590,7 +50640,7 @@
         <v>161</v>
       </c>
       <c r="D354" t="s">
-        <v>833</v>
+        <v>740</v>
       </c>
       <c r="E354" t="s">
         <v>51</v>
@@ -50616,22 +50666,22 @@
     </row>
     <row r="355" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A355" s="1">
-        <v>42741</v>
+        <v>42736</v>
       </c>
       <c r="C355" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D355" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="E355" t="s">
-        <v>163</v>
+        <v>51</v>
       </c>
       <c r="F355">
         <v>1</v>
       </c>
       <c r="G355" t="s">
-        <v>1252</v>
+        <v>1178</v>
       </c>
       <c r="H355" t="s">
         <v>1253</v>
@@ -50648,22 +50698,22 @@
     </row>
     <row r="356" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A356" s="1">
-        <v>42742</v>
+        <v>42736</v>
       </c>
       <c r="C356" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D356" t="s">
-        <v>740</v>
+        <v>833</v>
       </c>
       <c r="E356" t="s">
-        <v>165</v>
+        <v>51</v>
       </c>
       <c r="F356">
         <v>1</v>
       </c>
       <c r="G356" t="s">
-        <v>1252</v>
+        <v>1178</v>
       </c>
       <c r="H356" t="s">
         <v>1253</v>
@@ -50680,7 +50730,7 @@
     </row>
     <row r="357" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A357" s="1">
-        <v>42743</v>
+        <v>42741</v>
       </c>
       <c r="C357" t="s">
         <v>162</v>
@@ -50689,7 +50739,7 @@
         <v>740</v>
       </c>
       <c r="E357" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="F357">
         <v>1</v>
@@ -50712,7 +50762,7 @@
     </row>
     <row r="358" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A358" s="1">
-        <v>42744</v>
+        <v>42742</v>
       </c>
       <c r="C358" t="s">
         <v>162</v>
@@ -50721,7 +50771,7 @@
         <v>740</v>
       </c>
       <c r="E358" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="F358">
         <v>1</v>
@@ -50744,7 +50794,7 @@
     </row>
     <row r="359" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A359" s="1">
-        <v>42741</v>
+        <v>42743</v>
       </c>
       <c r="C359" t="s">
         <v>162</v>
@@ -50753,7 +50803,7 @@
         <v>740</v>
       </c>
       <c r="E359" t="s">
-        <v>458</v>
+        <v>167</v>
       </c>
       <c r="F359">
         <v>1</v>
@@ -50776,7 +50826,7 @@
     </row>
     <row r="360" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A360" s="1">
-        <v>42742</v>
+        <v>42744</v>
       </c>
       <c r="C360" t="s">
         <v>162</v>
@@ -50785,7 +50835,7 @@
         <v>740</v>
       </c>
       <c r="E360" t="s">
-        <v>460</v>
+        <v>169</v>
       </c>
       <c r="F360">
         <v>1</v>
@@ -50808,7 +50858,7 @@
     </row>
     <row r="361" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A361" s="1">
-        <v>42743</v>
+        <v>42741</v>
       </c>
       <c r="C361" t="s">
         <v>162</v>
@@ -50817,7 +50867,7 @@
         <v>740</v>
       </c>
       <c r="E361" t="s">
-        <v>463</v>
+        <v>458</v>
       </c>
       <c r="F361">
         <v>1</v>
@@ -50835,6 +50885,70 @@
         <v>1</v>
       </c>
       <c r="P361" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="362" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A362" s="1">
+        <v>42742</v>
+      </c>
+      <c r="C362" t="s">
+        <v>162</v>
+      </c>
+      <c r="D362" t="s">
+        <v>740</v>
+      </c>
+      <c r="E362" t="s">
+        <v>460</v>
+      </c>
+      <c r="F362">
+        <v>1</v>
+      </c>
+      <c r="G362" t="s">
+        <v>1252</v>
+      </c>
+      <c r="H362" t="s">
+        <v>1253</v>
+      </c>
+      <c r="I362" t="s">
+        <v>1254</v>
+      </c>
+      <c r="J362">
+        <v>1</v>
+      </c>
+      <c r="P362" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="363" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A363" s="1">
+        <v>42743</v>
+      </c>
+      <c r="C363" t="s">
+        <v>162</v>
+      </c>
+      <c r="D363" t="s">
+        <v>740</v>
+      </c>
+      <c r="E363" t="s">
+        <v>463</v>
+      </c>
+      <c r="F363">
+        <v>1</v>
+      </c>
+      <c r="G363" t="s">
+        <v>1252</v>
+      </c>
+      <c r="H363" t="s">
+        <v>1253</v>
+      </c>
+      <c r="I363" t="s">
+        <v>1254</v>
+      </c>
+      <c r="J363">
+        <v>1</v>
+      </c>
+      <c r="P363" t="s">
         <v>405</v>
       </c>
     </row>
@@ -56503,8 +56617,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Q310"/>
+  <dimension ref="A1:Q311"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="27.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -62539,7 +62658,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="257" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A257" s="1">
         <v>42738</v>
       </c>
@@ -62562,7 +62681,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="258" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A258" s="1">
         <v>42738</v>
       </c>
@@ -62585,7 +62704,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="259" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A259" s="1">
         <v>42736</v>
       </c>
@@ -62611,18 +62730,18 @@
         <v>197</v>
       </c>
     </row>
-    <row r="260" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A260" s="1">
-        <v>42736</v>
+        <v>42738</v>
       </c>
       <c r="C260" t="s">
-        <v>138</v>
+        <v>114</v>
       </c>
       <c r="D260" t="s">
-        <v>47</v>
+        <v>1537</v>
       </c>
       <c r="E260" t="s">
-        <v>47</v>
+        <v>1538</v>
       </c>
       <c r="G260" t="s">
         <v>224</v>
@@ -62633,13 +62752,16 @@
       <c r="N260" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="261" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O260" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="261" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A261" s="1">
         <v>42736</v>
       </c>
       <c r="C261" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D261" t="s">
         <v>47</v>
@@ -62657,21 +62779,21 @@
         <v>197</v>
       </c>
     </row>
-    <row r="262" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A262" s="1">
         <v>42736</v>
       </c>
       <c r="C262" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D262" t="s">
-        <v>239</v>
+        <v>47</v>
       </c>
       <c r="E262" t="s">
-        <v>240</v>
+        <v>47</v>
       </c>
       <c r="G262" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="K262" t="s">
         <v>218</v>
@@ -62680,7 +62802,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="263" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A263" s="1">
         <v>42736</v>
       </c>
@@ -62688,13 +62810,13 @@
         <v>140</v>
       </c>
       <c r="D263" t="s">
-        <v>141</v>
+        <v>239</v>
       </c>
       <c r="E263" t="s">
-        <v>434</v>
+        <v>240</v>
       </c>
       <c r="G263" t="s">
-        <v>435</v>
+        <v>214</v>
       </c>
       <c r="K263" t="s">
         <v>218</v>
@@ -62703,7 +62825,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="264" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A264" s="1">
         <v>42736</v>
       </c>
@@ -62711,10 +62833,10 @@
         <v>140</v>
       </c>
       <c r="D264" t="s">
-        <v>436</v>
+        <v>141</v>
       </c>
       <c r="E264" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="G264" t="s">
         <v>435</v>
@@ -62726,7 +62848,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="265" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A265" s="1">
         <v>42736</v>
       </c>
@@ -62734,10 +62856,10 @@
         <v>140</v>
       </c>
       <c r="D265" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E265" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="G265" t="s">
         <v>435</v>
@@ -62749,7 +62871,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="266" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A266" s="1">
         <v>42736</v>
       </c>
@@ -62757,13 +62879,13 @@
         <v>140</v>
       </c>
       <c r="D266" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E266" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="G266" t="s">
-        <v>291</v>
+        <v>435</v>
       </c>
       <c r="K266" t="s">
         <v>218</v>
@@ -62772,7 +62894,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="267" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A267" s="1">
         <v>42736</v>
       </c>
@@ -62780,10 +62902,10 @@
         <v>140</v>
       </c>
       <c r="D267" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E267" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="G267" t="s">
         <v>291</v>
@@ -62795,7 +62917,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="268" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A268" s="1">
         <v>42736</v>
       </c>
@@ -62803,10 +62925,10 @@
         <v>140</v>
       </c>
       <c r="D268" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E268" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="G268" t="s">
         <v>291</v>
@@ -62818,7 +62940,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="269" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A269" s="1">
         <v>42736</v>
       </c>
@@ -62826,13 +62948,13 @@
         <v>140</v>
       </c>
       <c r="D269" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E269" t="s">
-        <v>293</v>
+        <v>445</v>
       </c>
       <c r="G269" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="K269" t="s">
         <v>218</v>
@@ -62841,21 +62963,21 @@
         <v>197</v>
       </c>
     </row>
-    <row r="270" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A270" s="1">
         <v>42736</v>
       </c>
       <c r="C270" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="D270" t="s">
-        <v>51</v>
+        <v>446</v>
       </c>
       <c r="E270" t="s">
-        <v>52</v>
+        <v>293</v>
       </c>
       <c r="G270" t="s">
-        <v>51</v>
+        <v>294</v>
       </c>
       <c r="K270" t="s">
         <v>218</v>
@@ -62864,7 +62986,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="271" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A271" s="1">
         <v>42736</v>
       </c>
@@ -62872,13 +62994,13 @@
         <v>149</v>
       </c>
       <c r="D271" t="s">
-        <v>239</v>
+        <v>51</v>
       </c>
       <c r="E271" t="s">
-        <v>240</v>
+        <v>52</v>
       </c>
       <c r="G271" t="s">
-        <v>214</v>
+        <v>51</v>
       </c>
       <c r="K271" t="s">
         <v>218</v>
@@ -62887,12 +63009,12 @@
         <v>197</v>
       </c>
     </row>
-    <row r="272" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A272" s="1">
         <v>42736</v>
       </c>
       <c r="C272" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D272" t="s">
         <v>239</v>
@@ -62918,13 +63040,13 @@
         <v>150</v>
       </c>
       <c r="D273" t="s">
-        <v>141</v>
+        <v>239</v>
       </c>
       <c r="E273" t="s">
-        <v>434</v>
+        <v>240</v>
       </c>
       <c r="G273" t="s">
-        <v>435</v>
+        <v>214</v>
       </c>
       <c r="K273" t="s">
         <v>218</v>
@@ -62941,10 +63063,10 @@
         <v>150</v>
       </c>
       <c r="D274" t="s">
-        <v>436</v>
+        <v>141</v>
       </c>
       <c r="E274" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="G274" t="s">
         <v>435</v>
@@ -62964,10 +63086,10 @@
         <v>150</v>
       </c>
       <c r="D275" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E275" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="G275" t="s">
         <v>435</v>
@@ -62987,13 +63109,13 @@
         <v>150</v>
       </c>
       <c r="D276" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E276" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="G276" t="s">
-        <v>291</v>
+        <v>435</v>
       </c>
       <c r="K276" t="s">
         <v>218</v>
@@ -63010,10 +63132,10 @@
         <v>150</v>
       </c>
       <c r="D277" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E277" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="G277" t="s">
         <v>291</v>
@@ -63033,10 +63155,10 @@
         <v>150</v>
       </c>
       <c r="D278" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E278" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="G278" t="s">
         <v>291</v>
@@ -63056,13 +63178,13 @@
         <v>150</v>
       </c>
       <c r="D279" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E279" t="s">
-        <v>293</v>
+        <v>445</v>
       </c>
       <c r="G279" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="K279" t="s">
         <v>218</v>
@@ -63076,16 +63198,16 @@
         <v>42736</v>
       </c>
       <c r="C280" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D280" t="s">
-        <v>239</v>
+        <v>446</v>
       </c>
       <c r="E280" t="s">
-        <v>240</v>
+        <v>293</v>
       </c>
       <c r="G280" t="s">
-        <v>214</v>
+        <v>294</v>
       </c>
       <c r="K280" t="s">
         <v>218</v>
@@ -63102,13 +63224,13 @@
         <v>151</v>
       </c>
       <c r="D281" t="s">
-        <v>141</v>
+        <v>239</v>
       </c>
       <c r="E281" t="s">
-        <v>434</v>
+        <v>240</v>
       </c>
       <c r="G281" t="s">
-        <v>435</v>
+        <v>214</v>
       </c>
       <c r="K281" t="s">
         <v>218</v>
@@ -63125,10 +63247,10 @@
         <v>151</v>
       </c>
       <c r="D282" t="s">
-        <v>436</v>
+        <v>141</v>
       </c>
       <c r="E282" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="G282" t="s">
         <v>435</v>
@@ -63148,10 +63270,10 @@
         <v>151</v>
       </c>
       <c r="D283" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E283" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="G283" t="s">
         <v>435</v>
@@ -63171,13 +63293,13 @@
         <v>151</v>
       </c>
       <c r="D284" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E284" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="G284" t="s">
-        <v>291</v>
+        <v>435</v>
       </c>
       <c r="K284" t="s">
         <v>218</v>
@@ -63194,10 +63316,10 @@
         <v>151</v>
       </c>
       <c r="D285" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E285" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="G285" t="s">
         <v>291</v>
@@ -63217,10 +63339,10 @@
         <v>151</v>
       </c>
       <c r="D286" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E286" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="G286" t="s">
         <v>291</v>
@@ -63240,13 +63362,13 @@
         <v>151</v>
       </c>
       <c r="D287" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E287" t="s">
-        <v>293</v>
+        <v>445</v>
       </c>
       <c r="G287" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="K287" t="s">
         <v>218</v>
@@ -63260,16 +63382,16 @@
         <v>42736</v>
       </c>
       <c r="C288" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D288" t="s">
-        <v>47</v>
+        <v>446</v>
       </c>
       <c r="E288" t="s">
-        <v>47</v>
+        <v>293</v>
       </c>
       <c r="G288" t="s">
-        <v>224</v>
+        <v>294</v>
       </c>
       <c r="K288" t="s">
         <v>218</v>
@@ -63283,7 +63405,7 @@
         <v>42736</v>
       </c>
       <c r="C289" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D289" t="s">
         <v>47</v>
@@ -63306,16 +63428,16 @@
         <v>42736</v>
       </c>
       <c r="C290" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D290" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E290" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G290" t="s">
-        <v>51</v>
+        <v>224</v>
       </c>
       <c r="K290" t="s">
         <v>218</v>
@@ -63332,13 +63454,13 @@
         <v>154</v>
       </c>
       <c r="D291" t="s">
-        <v>239</v>
+        <v>51</v>
       </c>
       <c r="E291" t="s">
-        <v>240</v>
+        <v>52</v>
       </c>
       <c r="G291" t="s">
-        <v>214</v>
+        <v>51</v>
       </c>
       <c r="K291" t="s">
         <v>218</v>
@@ -63352,16 +63474,16 @@
         <v>42736</v>
       </c>
       <c r="C292" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D292" t="s">
-        <v>47</v>
+        <v>239</v>
       </c>
       <c r="E292" t="s">
-        <v>47</v>
+        <v>240</v>
       </c>
       <c r="G292" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="K292" t="s">
         <v>218</v>
@@ -63375,13 +63497,13 @@
         <v>42736</v>
       </c>
       <c r="C293" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D293" t="s">
         <v>47</v>
       </c>
       <c r="E293" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G293" t="s">
         <v>224</v>
@@ -63401,13 +63523,13 @@
         <v>156</v>
       </c>
       <c r="D294" t="s">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="E294" t="s">
-        <v>117</v>
+        <v>48</v>
       </c>
       <c r="G294" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="K294" t="s">
         <v>218</v>
@@ -63424,13 +63546,13 @@
         <v>156</v>
       </c>
       <c r="D295" t="s">
-        <v>239</v>
+        <v>13</v>
       </c>
       <c r="E295" t="s">
-        <v>240</v>
+        <v>117</v>
       </c>
       <c r="G295" t="s">
-        <v>214</v>
+        <v>199</v>
       </c>
       <c r="K295" t="s">
         <v>218</v>
@@ -63444,19 +63566,16 @@
         <v>42736</v>
       </c>
       <c r="C296" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D296" t="s">
-        <v>447</v>
+        <v>239</v>
       </c>
       <c r="E296" t="s">
-        <v>448</v>
+        <v>240</v>
       </c>
       <c r="G296" t="s">
-        <v>206</v>
-      </c>
-      <c r="I296" t="s">
-        <v>449</v>
+        <v>214</v>
       </c>
       <c r="K296" t="s">
         <v>218</v>
@@ -63473,13 +63592,16 @@
         <v>157</v>
       </c>
       <c r="D297" t="s">
-        <v>158</v>
+        <v>447</v>
       </c>
       <c r="E297" t="s">
-        <v>158</v>
+        <v>448</v>
       </c>
       <c r="G297" t="s">
-        <v>224</v>
+        <v>206</v>
+      </c>
+      <c r="I297" t="s">
+        <v>449</v>
       </c>
       <c r="K297" t="s">
         <v>218</v>
@@ -63496,16 +63618,13 @@
         <v>157</v>
       </c>
       <c r="D298" t="s">
-        <v>450</v>
+        <v>158</v>
       </c>
       <c r="E298" t="s">
-        <v>451</v>
+        <v>158</v>
       </c>
       <c r="G298" t="s">
-        <v>206</v>
-      </c>
-      <c r="I298" t="s">
-        <v>452</v>
+        <v>224</v>
       </c>
       <c r="K298" t="s">
         <v>218</v>
@@ -63519,16 +63638,19 @@
         <v>42736</v>
       </c>
       <c r="C299" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D299" t="s">
-        <v>47</v>
+        <v>450</v>
       </c>
       <c r="E299" t="s">
-        <v>47</v>
+        <v>451</v>
       </c>
       <c r="G299" t="s">
-        <v>224</v>
+        <v>206</v>
+      </c>
+      <c r="I299" t="s">
+        <v>452</v>
       </c>
       <c r="K299" t="s">
         <v>218</v>
@@ -63542,7 +63664,7 @@
         <v>42736</v>
       </c>
       <c r="C300" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D300" t="s">
         <v>47</v>
@@ -63565,16 +63687,16 @@
         <v>42736</v>
       </c>
       <c r="C301" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D301" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E301" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G301" t="s">
-        <v>51</v>
+        <v>224</v>
       </c>
       <c r="K301" t="s">
         <v>218</v>
@@ -63591,13 +63713,13 @@
         <v>161</v>
       </c>
       <c r="D302" t="s">
-        <v>239</v>
+        <v>51</v>
       </c>
       <c r="E302" t="s">
-        <v>240</v>
+        <v>52</v>
       </c>
       <c r="G302" t="s">
-        <v>214</v>
+        <v>51</v>
       </c>
       <c r="K302" t="s">
         <v>218</v>
@@ -63611,19 +63733,16 @@
         <v>42736</v>
       </c>
       <c r="C303" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D303" t="s">
-        <v>163</v>
+        <v>239</v>
       </c>
       <c r="E303" t="s">
-        <v>164</v>
+        <v>240</v>
       </c>
       <c r="G303" t="s">
-        <v>216</v>
-      </c>
-      <c r="H303" t="s">
-        <v>453</v>
+        <v>214</v>
       </c>
       <c r="K303" t="s">
         <v>218</v>
@@ -63640,16 +63759,16 @@
         <v>162</v>
       </c>
       <c r="D304" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E304" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="G304" t="s">
         <v>216</v>
       </c>
       <c r="H304" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="K304" t="s">
         <v>218</v>
@@ -63666,14 +63785,17 @@
         <v>162</v>
       </c>
       <c r="D305" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="E305" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="G305" t="s">
         <v>216</v>
       </c>
+      <c r="H305" t="s">
+        <v>454</v>
+      </c>
       <c r="K305" t="s">
         <v>218</v>
       </c>
@@ -63689,13 +63811,13 @@
         <v>162</v>
       </c>
       <c r="D306" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E306" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="G306" t="s">
-        <v>455</v>
+        <v>216</v>
       </c>
       <c r="K306" t="s">
         <v>218</v>
@@ -63712,13 +63834,13 @@
         <v>162</v>
       </c>
       <c r="D307" t="s">
-        <v>456</v>
+        <v>169</v>
       </c>
       <c r="E307" t="s">
-        <v>457</v>
+        <v>170</v>
       </c>
       <c r="G307" t="s">
-        <v>224</v>
+        <v>455</v>
       </c>
       <c r="K307" t="s">
         <v>218</v>
@@ -63735,19 +63857,13 @@
         <v>162</v>
       </c>
       <c r="D308" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="E308" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="G308" t="s">
-        <v>206</v>
-      </c>
-      <c r="H308" t="s">
-        <v>453</v>
-      </c>
-      <c r="I308" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="K308" t="s">
         <v>218</v>
@@ -63764,16 +63880,19 @@
         <v>162</v>
       </c>
       <c r="D309" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="E309" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="G309" t="s">
         <v>206</v>
       </c>
+      <c r="H309" t="s">
+        <v>453</v>
+      </c>
       <c r="I309" t="s">
-        <v>462</v>
+        <v>216</v>
       </c>
       <c r="K309" t="s">
         <v>218</v>
@@ -63790,21 +63909,47 @@
         <v>162</v>
       </c>
       <c r="D310" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="E310" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="G310" t="s">
         <v>206</v>
       </c>
       <c r="I310" t="s">
-        <v>216</v>
+        <v>462</v>
       </c>
       <c r="K310" t="s">
         <v>218</v>
       </c>
       <c r="N310" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="311" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A311" s="1">
+        <v>42736</v>
+      </c>
+      <c r="C311" t="s">
+        <v>162</v>
+      </c>
+      <c r="D311" t="s">
+        <v>463</v>
+      </c>
+      <c r="E311" t="s">
+        <v>464</v>
+      </c>
+      <c r="G311" t="s">
+        <v>206</v>
+      </c>
+      <c r="I311" t="s">
+        <v>216</v>
+      </c>
+      <c r="K311" t="s">
+        <v>218</v>
+      </c>
+      <c r="N311" t="s">
         <v>197</v>
       </c>
     </row>

</xml_diff>

<commit_message>
CCD-8066: Updating with master
</commit_message>
<xml_diff>
--- a/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_Master_Definition.xlsx
+++ b/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_Master_Definition.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jen/IdeaProjects/test-defs-jen/ccd-test-definitions/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{491EB25B-AFB2-A642-A9E7-25A443DDA749}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{292B7B28-3B2C-3142-854C-3C64141921F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" firstSheet="14" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18020" firstSheet="14" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SearchInputFields" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16058" uniqueCount="1542">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16031" uniqueCount="1537">
   <si>
     <t>SearchInputFields</t>
   </si>
@@ -4660,28 +4660,13 @@
   </si>
   <si>
     <t>${MCA_API_BASE_URL:http://aac-manage-case-assignment-aat.service.core-compute-aat.internal}/noc/apply-decision</t>
-  </si>
-  <si>
-    <t>StaffUser</t>
-  </si>
-  <si>
-    <t>Staff User</t>
-  </si>
-  <si>
-    <t>StaffUser Fields</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#ARGUMENT(CATEGORY-LEGAL-OPS,CATEGORY-ADMIN,REGION-1235) </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> #ARGUMENT(CATEGORY-LEGAL-OPS,CATEGORY-ADMIN,REGION-1235) </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -4696,12 +4681,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF172B4D"/>
-      <name val="Arial Unicode MS"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -4725,11 +4704,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -31079,13 +31057,8 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
-  <dimension ref="A1:F478"/>
+  <dimension ref="A1:F477"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="3" max="3" width="27.33203125" customWidth="1"/>
-    <col min="4" max="4" width="22.1640625" customWidth="1"/>
-    <col min="5" max="5" width="34.33203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -37152,13 +37125,13 @@
         <v>42736</v>
       </c>
       <c r="C359" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="D359" t="s">
-        <v>1537</v>
+        <v>47</v>
       </c>
       <c r="E359" t="s">
-        <v>727</v>
+        <v>644</v>
       </c>
       <c r="F359" t="s">
         <v>643</v>
@@ -37169,7 +37142,7 @@
         <v>42736</v>
       </c>
       <c r="C360" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D360" t="s">
         <v>47</v>
@@ -37186,13 +37159,13 @@
         <v>42736</v>
       </c>
       <c r="C361" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D361" t="s">
-        <v>47</v>
+        <v>239</v>
       </c>
       <c r="E361" t="s">
-        <v>644</v>
+        <v>735</v>
       </c>
       <c r="F361" t="s">
         <v>643</v>
@@ -37206,7 +37179,7 @@
         <v>140</v>
       </c>
       <c r="D362" t="s">
-        <v>239</v>
+        <v>141</v>
       </c>
       <c r="E362" t="s">
         <v>735</v>
@@ -37223,7 +37196,7 @@
         <v>140</v>
       </c>
       <c r="D363" t="s">
-        <v>141</v>
+        <v>436</v>
       </c>
       <c r="E363" t="s">
         <v>735</v>
@@ -37240,7 +37213,7 @@
         <v>140</v>
       </c>
       <c r="D364" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="E364" t="s">
         <v>735</v>
@@ -37257,7 +37230,7 @@
         <v>140</v>
       </c>
       <c r="D365" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E365" t="s">
         <v>735</v>
@@ -37274,7 +37247,7 @@
         <v>140</v>
       </c>
       <c r="D366" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E366" t="s">
         <v>735</v>
@@ -37291,7 +37264,7 @@
         <v>140</v>
       </c>
       <c r="D367" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="E367" t="s">
         <v>735</v>
@@ -37308,7 +37281,7 @@
         <v>140</v>
       </c>
       <c r="D368" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E368" t="s">
         <v>735</v>
@@ -37325,10 +37298,10 @@
         <v>140</v>
       </c>
       <c r="D369" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
       <c r="E369" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="F369" t="s">
         <v>643</v>
@@ -37342,7 +37315,7 @@
         <v>140</v>
       </c>
       <c r="D370" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E370" t="s">
         <v>736</v>
@@ -37359,7 +37332,7 @@
         <v>140</v>
       </c>
       <c r="D371" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="E371" t="s">
         <v>736</v>
@@ -37376,7 +37349,7 @@
         <v>140</v>
       </c>
       <c r="D372" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E372" t="s">
         <v>736</v>
@@ -37393,10 +37366,10 @@
         <v>140</v>
       </c>
       <c r="D373" t="s">
-        <v>446</v>
+        <v>239</v>
       </c>
       <c r="E373" t="s">
-        <v>736</v>
+        <v>644</v>
       </c>
       <c r="F373" t="s">
         <v>643</v>
@@ -37410,7 +37383,7 @@
         <v>140</v>
       </c>
       <c r="D374" t="s">
-        <v>239</v>
+        <v>141</v>
       </c>
       <c r="E374" t="s">
         <v>644</v>
@@ -37427,7 +37400,7 @@
         <v>140</v>
       </c>
       <c r="D375" t="s">
-        <v>141</v>
+        <v>436</v>
       </c>
       <c r="E375" t="s">
         <v>644</v>
@@ -37444,7 +37417,7 @@
         <v>140</v>
       </c>
       <c r="D376" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="E376" t="s">
         <v>644</v>
@@ -37461,7 +37434,7 @@
         <v>140</v>
       </c>
       <c r="D377" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E377" t="s">
         <v>644</v>
@@ -37478,7 +37451,7 @@
         <v>140</v>
       </c>
       <c r="D378" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E378" t="s">
         <v>644</v>
@@ -37495,7 +37468,7 @@
         <v>140</v>
       </c>
       <c r="D379" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="E379" t="s">
         <v>644</v>
@@ -37512,7 +37485,7 @@
         <v>140</v>
       </c>
       <c r="D380" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E380" t="s">
         <v>644</v>
@@ -37526,10 +37499,10 @@
         <v>42736</v>
       </c>
       <c r="C381" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="D381" t="s">
-        <v>446</v>
+        <v>239</v>
       </c>
       <c r="E381" t="s">
         <v>644</v>
@@ -37546,7 +37519,7 @@
         <v>149</v>
       </c>
       <c r="D382" t="s">
-        <v>239</v>
+        <v>51</v>
       </c>
       <c r="E382" t="s">
         <v>644</v>
@@ -37566,7 +37539,7 @@
         <v>51</v>
       </c>
       <c r="E383" t="s">
-        <v>644</v>
+        <v>718</v>
       </c>
       <c r="F383" t="s">
         <v>643</v>
@@ -37577,13 +37550,13 @@
         <v>42736</v>
       </c>
       <c r="C384" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D384" t="s">
-        <v>51</v>
+        <v>239</v>
       </c>
       <c r="E384" t="s">
-        <v>718</v>
+        <v>710</v>
       </c>
       <c r="F384" t="s">
         <v>643</v>
@@ -37597,7 +37570,7 @@
         <v>150</v>
       </c>
       <c r="D385" t="s">
-        <v>239</v>
+        <v>141</v>
       </c>
       <c r="E385" t="s">
         <v>710</v>
@@ -37614,7 +37587,7 @@
         <v>150</v>
       </c>
       <c r="D386" t="s">
-        <v>141</v>
+        <v>436</v>
       </c>
       <c r="E386" t="s">
         <v>710</v>
@@ -37631,7 +37604,7 @@
         <v>150</v>
       </c>
       <c r="D387" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="E387" t="s">
         <v>710</v>
@@ -37648,7 +37621,7 @@
         <v>150</v>
       </c>
       <c r="D388" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E388" t="s">
         <v>710</v>
@@ -37665,7 +37638,7 @@
         <v>150</v>
       </c>
       <c r="D389" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E389" t="s">
         <v>710</v>
@@ -37682,7 +37655,7 @@
         <v>150</v>
       </c>
       <c r="D390" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="E390" t="s">
         <v>710</v>
@@ -37699,7 +37672,7 @@
         <v>150</v>
       </c>
       <c r="D391" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E391" t="s">
         <v>710</v>
@@ -37716,10 +37689,10 @@
         <v>150</v>
       </c>
       <c r="D392" t="s">
-        <v>446</v>
+        <v>239</v>
       </c>
       <c r="E392" t="s">
-        <v>710</v>
+        <v>735</v>
       </c>
       <c r="F392" t="s">
         <v>643</v>
@@ -37733,7 +37706,7 @@
         <v>150</v>
       </c>
       <c r="D393" t="s">
-        <v>239</v>
+        <v>141</v>
       </c>
       <c r="E393" t="s">
         <v>735</v>
@@ -37750,7 +37723,7 @@
         <v>150</v>
       </c>
       <c r="D394" t="s">
-        <v>141</v>
+        <v>436</v>
       </c>
       <c r="E394" t="s">
         <v>735</v>
@@ -37767,7 +37740,7 @@
         <v>150</v>
       </c>
       <c r="D395" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="E395" t="s">
         <v>735</v>
@@ -37784,7 +37757,7 @@
         <v>150</v>
       </c>
       <c r="D396" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E396" t="s">
         <v>735</v>
@@ -37801,7 +37774,7 @@
         <v>150</v>
       </c>
       <c r="D397" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E397" t="s">
         <v>735</v>
@@ -37818,7 +37791,7 @@
         <v>150</v>
       </c>
       <c r="D398" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="E398" t="s">
         <v>735</v>
@@ -37835,7 +37808,7 @@
         <v>150</v>
       </c>
       <c r="D399" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E399" t="s">
         <v>735</v>
@@ -37852,10 +37825,10 @@
         <v>150</v>
       </c>
       <c r="D400" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
       <c r="E400" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="F400" t="s">
         <v>643</v>
@@ -37869,7 +37842,7 @@
         <v>150</v>
       </c>
       <c r="D401" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E401" t="s">
         <v>736</v>
@@ -37886,7 +37859,7 @@
         <v>150</v>
       </c>
       <c r="D402" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="E402" t="s">
         <v>736</v>
@@ -37903,7 +37876,7 @@
         <v>150</v>
       </c>
       <c r="D403" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E403" t="s">
         <v>736</v>
@@ -37920,10 +37893,10 @@
         <v>150</v>
       </c>
       <c r="D404" t="s">
-        <v>446</v>
+        <v>239</v>
       </c>
       <c r="E404" t="s">
-        <v>736</v>
+        <v>644</v>
       </c>
       <c r="F404" t="s">
         <v>643</v>
@@ -37937,7 +37910,7 @@
         <v>150</v>
       </c>
       <c r="D405" t="s">
-        <v>239</v>
+        <v>141</v>
       </c>
       <c r="E405" t="s">
         <v>644</v>
@@ -37954,7 +37927,7 @@
         <v>150</v>
       </c>
       <c r="D406" t="s">
-        <v>141</v>
+        <v>436</v>
       </c>
       <c r="E406" t="s">
         <v>644</v>
@@ -37971,7 +37944,7 @@
         <v>150</v>
       </c>
       <c r="D407" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="E407" t="s">
         <v>644</v>
@@ -37988,7 +37961,7 @@
         <v>150</v>
       </c>
       <c r="D408" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E408" t="s">
         <v>644</v>
@@ -38005,7 +37978,7 @@
         <v>150</v>
       </c>
       <c r="D409" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E409" t="s">
         <v>644</v>
@@ -38022,7 +37995,7 @@
         <v>150</v>
       </c>
       <c r="D410" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="E410" t="s">
         <v>644</v>
@@ -38039,7 +38012,7 @@
         <v>150</v>
       </c>
       <c r="D411" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E411" t="s">
         <v>644</v>
@@ -38053,13 +38026,13 @@
         <v>42736</v>
       </c>
       <c r="C412" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D412" t="s">
-        <v>446</v>
+        <v>239</v>
       </c>
       <c r="E412" t="s">
-        <v>644</v>
+        <v>710</v>
       </c>
       <c r="F412" t="s">
         <v>643</v>
@@ -38073,7 +38046,7 @@
         <v>151</v>
       </c>
       <c r="D413" t="s">
-        <v>239</v>
+        <v>141</v>
       </c>
       <c r="E413" t="s">
         <v>710</v>
@@ -38090,7 +38063,7 @@
         <v>151</v>
       </c>
       <c r="D414" t="s">
-        <v>141</v>
+        <v>436</v>
       </c>
       <c r="E414" t="s">
         <v>710</v>
@@ -38107,7 +38080,7 @@
         <v>151</v>
       </c>
       <c r="D415" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="E415" t="s">
         <v>710</v>
@@ -38124,7 +38097,7 @@
         <v>151</v>
       </c>
       <c r="D416" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E416" t="s">
         <v>710</v>
@@ -38141,7 +38114,7 @@
         <v>151</v>
       </c>
       <c r="D417" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E417" t="s">
         <v>710</v>
@@ -38158,7 +38131,7 @@
         <v>151</v>
       </c>
       <c r="D418" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="E418" t="s">
         <v>710</v>
@@ -38175,7 +38148,7 @@
         <v>151</v>
       </c>
       <c r="D419" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E419" t="s">
         <v>710</v>
@@ -38192,10 +38165,10 @@
         <v>151</v>
       </c>
       <c r="D420" t="s">
-        <v>446</v>
+        <v>239</v>
       </c>
       <c r="E420" t="s">
-        <v>710</v>
+        <v>735</v>
       </c>
       <c r="F420" t="s">
         <v>643</v>
@@ -38209,7 +38182,7 @@
         <v>151</v>
       </c>
       <c r="D421" t="s">
-        <v>239</v>
+        <v>141</v>
       </c>
       <c r="E421" t="s">
         <v>735</v>
@@ -38226,7 +38199,7 @@
         <v>151</v>
       </c>
       <c r="D422" t="s">
-        <v>141</v>
+        <v>436</v>
       </c>
       <c r="E422" t="s">
         <v>735</v>
@@ -38243,7 +38216,7 @@
         <v>151</v>
       </c>
       <c r="D423" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="E423" t="s">
         <v>735</v>
@@ -38260,7 +38233,7 @@
         <v>151</v>
       </c>
       <c r="D424" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E424" t="s">
         <v>735</v>
@@ -38277,7 +38250,7 @@
         <v>151</v>
       </c>
       <c r="D425" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E425" t="s">
         <v>735</v>
@@ -38294,7 +38267,7 @@
         <v>151</v>
       </c>
       <c r="D426" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="E426" t="s">
         <v>735</v>
@@ -38311,7 +38284,7 @@
         <v>151</v>
       </c>
       <c r="D427" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E427" t="s">
         <v>735</v>
@@ -38328,10 +38301,10 @@
         <v>151</v>
       </c>
       <c r="D428" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
       <c r="E428" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="F428" t="s">
         <v>643</v>
@@ -38345,7 +38318,7 @@
         <v>151</v>
       </c>
       <c r="D429" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E429" t="s">
         <v>736</v>
@@ -38362,7 +38335,7 @@
         <v>151</v>
       </c>
       <c r="D430" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="E430" t="s">
         <v>736</v>
@@ -38379,7 +38352,7 @@
         <v>151</v>
       </c>
       <c r="D431" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E431" t="s">
         <v>736</v>
@@ -38396,10 +38369,10 @@
         <v>151</v>
       </c>
       <c r="D432" t="s">
-        <v>446</v>
+        <v>239</v>
       </c>
       <c r="E432" t="s">
-        <v>736</v>
+        <v>644</v>
       </c>
       <c r="F432" t="s">
         <v>643</v>
@@ -38413,7 +38386,7 @@
         <v>151</v>
       </c>
       <c r="D433" t="s">
-        <v>239</v>
+        <v>141</v>
       </c>
       <c r="E433" t="s">
         <v>644</v>
@@ -38430,7 +38403,7 @@
         <v>151</v>
       </c>
       <c r="D434" t="s">
-        <v>141</v>
+        <v>436</v>
       </c>
       <c r="E434" t="s">
         <v>644</v>
@@ -38447,7 +38420,7 @@
         <v>151</v>
       </c>
       <c r="D435" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="E435" t="s">
         <v>644</v>
@@ -38464,7 +38437,7 @@
         <v>151</v>
       </c>
       <c r="D436" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E436" t="s">
         <v>644</v>
@@ -38481,7 +38454,7 @@
         <v>151</v>
       </c>
       <c r="D437" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E437" t="s">
         <v>644</v>
@@ -38498,7 +38471,7 @@
         <v>151</v>
       </c>
       <c r="D438" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="E438" t="s">
         <v>644</v>
@@ -38515,7 +38488,7 @@
         <v>151</v>
       </c>
       <c r="D439" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E439" t="s">
         <v>644</v>
@@ -38529,10 +38502,10 @@
         <v>42736</v>
       </c>
       <c r="C440" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D440" t="s">
-        <v>446</v>
+        <v>47</v>
       </c>
       <c r="E440" t="s">
         <v>644</v>
@@ -38552,7 +38525,7 @@
         <v>47</v>
       </c>
       <c r="E441" t="s">
-        <v>644</v>
+        <v>735</v>
       </c>
       <c r="F441" t="s">
         <v>643</v>
@@ -38563,13 +38536,13 @@
         <v>42736</v>
       </c>
       <c r="C442" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D442" t="s">
         <v>47</v>
       </c>
       <c r="E442" t="s">
-        <v>735</v>
+        <v>644</v>
       </c>
       <c r="F442" t="s">
         <v>643</v>
@@ -38580,10 +38553,10 @@
         <v>42736</v>
       </c>
       <c r="C443" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D443" t="s">
-        <v>47</v>
+        <v>239</v>
       </c>
       <c r="E443" t="s">
         <v>644</v>
@@ -38600,7 +38573,7 @@
         <v>154</v>
       </c>
       <c r="D444" t="s">
-        <v>239</v>
+        <v>51</v>
       </c>
       <c r="E444" t="s">
         <v>644</v>
@@ -38620,7 +38593,7 @@
         <v>51</v>
       </c>
       <c r="E445" t="s">
-        <v>644</v>
+        <v>718</v>
       </c>
       <c r="F445" t="s">
         <v>643</v>
@@ -38631,13 +38604,13 @@
         <v>42736</v>
       </c>
       <c r="C446" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D446" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E446" t="s">
-        <v>718</v>
+        <v>644</v>
       </c>
       <c r="F446" t="s">
         <v>643</v>
@@ -38648,7 +38621,7 @@
         <v>42736</v>
       </c>
       <c r="C447" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D447" t="s">
         <v>47</v>
@@ -38668,7 +38641,7 @@
         <v>156</v>
       </c>
       <c r="D448" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="E448" t="s">
         <v>644</v>
@@ -38682,13 +38655,13 @@
         <v>42736</v>
       </c>
       <c r="C449" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D449" t="s">
-        <v>13</v>
+        <v>450</v>
       </c>
       <c r="E449" t="s">
-        <v>644</v>
+        <v>665</v>
       </c>
       <c r="F449" t="s">
         <v>643</v>
@@ -38705,10 +38678,10 @@
         <v>450</v>
       </c>
       <c r="E450" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="F450" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
     </row>
     <row r="451" spans="1:6" x14ac:dyDescent="0.2">
@@ -38719,13 +38692,13 @@
         <v>157</v>
       </c>
       <c r="D451" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="E451" t="s">
         <v>667</v>
       </c>
       <c r="F451" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
     </row>
     <row r="452" spans="1:6" x14ac:dyDescent="0.2">
@@ -38736,7 +38709,7 @@
         <v>157</v>
       </c>
       <c r="D452" t="s">
-        <v>447</v>
+        <v>158</v>
       </c>
       <c r="E452" t="s">
         <v>667</v>
@@ -38753,10 +38726,10 @@
         <v>157</v>
       </c>
       <c r="D453" t="s">
-        <v>158</v>
+        <v>447</v>
       </c>
       <c r="E453" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="F453" t="s">
         <v>643</v>
@@ -38770,7 +38743,7 @@
         <v>157</v>
       </c>
       <c r="D454" t="s">
-        <v>447</v>
+        <v>158</v>
       </c>
       <c r="E454" t="s">
         <v>665</v>
@@ -38784,13 +38757,13 @@
         <v>42736</v>
       </c>
       <c r="C455" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D455" t="s">
-        <v>158</v>
+        <v>47</v>
       </c>
       <c r="E455" t="s">
-        <v>665</v>
+        <v>710</v>
       </c>
       <c r="F455" t="s">
         <v>643</v>
@@ -38807,10 +38780,10 @@
         <v>47</v>
       </c>
       <c r="E456" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="F456" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
     </row>
     <row r="457" spans="1:6" x14ac:dyDescent="0.2">
@@ -38818,16 +38791,16 @@
         <v>42736</v>
       </c>
       <c r="C457" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D457" t="s">
         <v>47</v>
       </c>
       <c r="E457" t="s">
-        <v>714</v>
+        <v>710</v>
       </c>
       <c r="F457" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
     </row>
     <row r="458" spans="1:6" x14ac:dyDescent="0.2">
@@ -38841,10 +38814,10 @@
         <v>47</v>
       </c>
       <c r="E458" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="F458" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
     </row>
     <row r="459" spans="1:6" x14ac:dyDescent="0.2">
@@ -38852,16 +38825,16 @@
         <v>42736</v>
       </c>
       <c r="C459" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D459" t="s">
-        <v>47</v>
+        <v>239</v>
       </c>
       <c r="E459" t="s">
-        <v>714</v>
+        <v>644</v>
       </c>
       <c r="F459" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
     </row>
     <row r="460" spans="1:6" x14ac:dyDescent="0.2">
@@ -38872,7 +38845,7 @@
         <v>161</v>
       </c>
       <c r="D460" t="s">
-        <v>239</v>
+        <v>51</v>
       </c>
       <c r="E460" t="s">
         <v>644</v>
@@ -38892,7 +38865,7 @@
         <v>51</v>
       </c>
       <c r="E461" t="s">
-        <v>644</v>
+        <v>718</v>
       </c>
       <c r="F461" t="s">
         <v>643</v>
@@ -38900,16 +38873,16 @@
     </row>
     <row r="462" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A462" s="1">
-        <v>42736</v>
+        <v>42741</v>
       </c>
       <c r="C462" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D462" t="s">
-        <v>51</v>
+        <v>163</v>
       </c>
       <c r="E462" t="s">
-        <v>718</v>
+        <v>644</v>
       </c>
       <c r="F462" t="s">
         <v>643</v>
@@ -38917,13 +38890,13 @@
     </row>
     <row r="463" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A463" s="1">
-        <v>42741</v>
+        <v>42742</v>
       </c>
       <c r="C463" t="s">
         <v>162</v>
       </c>
       <c r="D463" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="E463" t="s">
         <v>644</v>
@@ -38934,13 +38907,13 @@
     </row>
     <row r="464" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A464" s="1">
-        <v>42742</v>
+        <v>42743</v>
       </c>
       <c r="C464" t="s">
         <v>162</v>
       </c>
       <c r="D464" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E464" t="s">
         <v>644</v>
@@ -38951,13 +38924,13 @@
     </row>
     <row r="465" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A465" s="1">
-        <v>42743</v>
+        <v>42744</v>
       </c>
       <c r="C465" t="s">
         <v>162</v>
       </c>
       <c r="D465" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="E465" t="s">
         <v>644</v>
@@ -38968,13 +38941,13 @@
     </row>
     <row r="466" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A466" s="1">
-        <v>42744</v>
+        <v>42745</v>
       </c>
       <c r="C466" t="s">
         <v>162</v>
       </c>
       <c r="D466" t="s">
-        <v>169</v>
+        <v>456</v>
       </c>
       <c r="E466" t="s">
         <v>644</v>
@@ -38985,13 +38958,13 @@
     </row>
     <row r="467" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A467" s="1">
-        <v>42745</v>
+        <v>42741</v>
       </c>
       <c r="C467" t="s">
         <v>162</v>
       </c>
       <c r="D467" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="E467" t="s">
         <v>644</v>
@@ -39002,13 +38975,13 @@
     </row>
     <row r="468" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A468" s="1">
-        <v>42741</v>
+        <v>42742</v>
       </c>
       <c r="C468" t="s">
         <v>162</v>
       </c>
       <c r="D468" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="E468" t="s">
         <v>644</v>
@@ -39019,13 +38992,13 @@
     </row>
     <row r="469" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A469" s="1">
-        <v>42742</v>
+        <v>42743</v>
       </c>
       <c r="C469" t="s">
         <v>162</v>
       </c>
       <c r="D469" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="E469" t="s">
         <v>644</v>
@@ -39036,64 +39009,64 @@
     </row>
     <row r="470" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A470" s="1">
-        <v>42743</v>
+        <v>42746</v>
       </c>
       <c r="C470" t="s">
         <v>162</v>
       </c>
       <c r="D470" t="s">
-        <v>463</v>
+        <v>163</v>
       </c>
       <c r="E470" t="s">
-        <v>644</v>
+        <v>727</v>
       </c>
       <c r="F470" t="s">
-        <v>643</v>
+        <v>716</v>
       </c>
     </row>
     <row r="471" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A471" s="1">
-        <v>42746</v>
+        <v>42747</v>
       </c>
       <c r="C471" t="s">
         <v>162</v>
       </c>
       <c r="D471" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="E471" t="s">
         <v>727</v>
       </c>
       <c r="F471" t="s">
-        <v>716</v>
+        <v>663</v>
       </c>
     </row>
     <row r="472" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A472" s="1">
-        <v>42747</v>
+        <v>42748</v>
       </c>
       <c r="C472" t="s">
         <v>162</v>
       </c>
       <c r="D472" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E472" t="s">
         <v>727</v>
       </c>
       <c r="F472" t="s">
-        <v>663</v>
+        <v>716</v>
       </c>
     </row>
     <row r="473" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A473" s="1">
-        <v>42748</v>
+        <v>42749</v>
       </c>
       <c r="C473" t="s">
         <v>162</v>
       </c>
       <c r="D473" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="E473" t="s">
         <v>727</v>
@@ -39104,13 +39077,13 @@
     </row>
     <row r="474" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A474" s="1">
-        <v>42749</v>
+        <v>42750</v>
       </c>
       <c r="C474" t="s">
         <v>162</v>
       </c>
       <c r="D474" t="s">
-        <v>169</v>
+        <v>456</v>
       </c>
       <c r="E474" t="s">
         <v>727</v>
@@ -39121,13 +39094,13 @@
     </row>
     <row r="475" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A475" s="1">
-        <v>42750</v>
+        <v>42741</v>
       </c>
       <c r="C475" t="s">
         <v>162</v>
       </c>
       <c r="D475" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="E475" t="s">
         <v>727</v>
@@ -39138,13 +39111,13 @@
     </row>
     <row r="476" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A476" s="1">
-        <v>42741</v>
+        <v>42742</v>
       </c>
       <c r="C476" t="s">
         <v>162</v>
       </c>
       <c r="D476" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="E476" t="s">
         <v>727</v>
@@ -39155,35 +39128,18 @@
     </row>
     <row r="477" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A477" s="1">
-        <v>42742</v>
+        <v>42743</v>
       </c>
       <c r="C477" t="s">
         <v>162</v>
       </c>
       <c r="D477" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="E477" t="s">
         <v>727</v>
       </c>
       <c r="F477" t="s">
-        <v>716</v>
-      </c>
-    </row>
-    <row r="478" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A478" s="1">
-        <v>42743</v>
-      </c>
-      <c r="C478" t="s">
-        <v>162</v>
-      </c>
-      <c r="D478" t="s">
-        <v>463</v>
-      </c>
-      <c r="E478" t="s">
-        <v>727</v>
-      </c>
-      <c r="F478" t="s">
         <v>716</v>
       </c>
     </row>
@@ -39194,16 +39150,10 @@
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
-  <dimension ref="A1:V363"/>
+  <dimension ref="A1:V361"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="26.1640625" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="19.33203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="15" max="15" width="20.1640625" customWidth="1"/>
-    <col min="16" max="16" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.2">
@@ -49256,68 +49206,68 @@
         <v>700</v>
       </c>
     </row>
-    <row r="311" spans="1:16" ht="18" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A311" s="1">
-        <v>42746</v>
+        <v>42736</v>
       </c>
       <c r="C311" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="D311" t="s">
         <v>748</v>
       </c>
       <c r="E311" t="s">
-        <v>1537</v>
+        <v>47</v>
       </c>
       <c r="F311">
         <v>1</v>
       </c>
       <c r="G311" t="s">
-        <v>1178</v>
+        <v>1252</v>
       </c>
       <c r="H311" t="s">
         <v>1253</v>
       </c>
       <c r="I311" t="s">
-        <v>1539</v>
-      </c>
-      <c r="O311" s="3" t="s">
-        <v>1540</v>
+        <v>1314</v>
+      </c>
+      <c r="J311">
+        <v>1</v>
       </c>
       <c r="P311" t="s">
-        <v>700</v>
+        <v>405</v>
       </c>
     </row>
     <row r="312" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A312" s="1">
-        <v>42746</v>
+        <v>42736</v>
       </c>
       <c r="C312" t="s">
-        <v>114</v>
+        <v>139</v>
       </c>
       <c r="D312" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="E312" t="s">
-        <v>1537</v>
+        <v>47</v>
       </c>
       <c r="F312">
         <v>1</v>
       </c>
       <c r="G312" t="s">
-        <v>1178</v>
+        <v>1252</v>
       </c>
       <c r="H312" t="s">
         <v>1253</v>
       </c>
       <c r="I312" t="s">
-        <v>1539</v>
-      </c>
-      <c r="O312" t="s">
-        <v>1541</v>
+        <v>1314</v>
+      </c>
+      <c r="J312">
+        <v>1</v>
       </c>
       <c r="P312" t="s">
-        <v>700</v>
+        <v>405</v>
       </c>
     </row>
     <row r="313" spans="1:16" x14ac:dyDescent="0.2">
@@ -49325,10 +49275,10 @@
         <v>42736</v>
       </c>
       <c r="C313" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D313" t="s">
-        <v>748</v>
+        <v>782</v>
       </c>
       <c r="E313" t="s">
         <v>47</v>
@@ -49357,25 +49307,25 @@
         <v>42736</v>
       </c>
       <c r="C314" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D314" t="s">
         <v>748</v>
       </c>
       <c r="E314" t="s">
-        <v>47</v>
+        <v>141</v>
       </c>
       <c r="F314">
         <v>1</v>
       </c>
       <c r="G314" t="s">
-        <v>1252</v>
+        <v>1178</v>
       </c>
       <c r="H314" t="s">
         <v>1253</v>
       </c>
       <c r="I314" t="s">
-        <v>1314</v>
+        <v>1254</v>
       </c>
       <c r="J314">
         <v>1</v>
@@ -49389,25 +49339,25 @@
         <v>42736</v>
       </c>
       <c r="C315" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D315" t="s">
-        <v>782</v>
+        <v>748</v>
       </c>
       <c r="E315" t="s">
-        <v>47</v>
+        <v>436</v>
       </c>
       <c r="F315">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G315" t="s">
-        <v>1252</v>
+        <v>1178</v>
       </c>
       <c r="H315" t="s">
         <v>1253</v>
       </c>
       <c r="I315" t="s">
-        <v>1314</v>
+        <v>1254</v>
       </c>
       <c r="J315">
         <v>1</v>
@@ -49427,10 +49377,10 @@
         <v>748</v>
       </c>
       <c r="E316" t="s">
-        <v>141</v>
+        <v>438</v>
       </c>
       <c r="F316">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G316" t="s">
         <v>1178</v>
@@ -49453,16 +49403,16 @@
         <v>42736</v>
       </c>
       <c r="C317" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="D317" t="s">
-        <v>748</v>
+        <v>740</v>
       </c>
       <c r="E317" t="s">
-        <v>436</v>
+        <v>51</v>
       </c>
       <c r="F317">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G317" t="s">
         <v>1178</v>
@@ -49485,16 +49435,16 @@
         <v>42736</v>
       </c>
       <c r="C318" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="D318" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
       <c r="E318" t="s">
-        <v>438</v>
+        <v>51</v>
       </c>
       <c r="F318">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G318" t="s">
         <v>1178</v>
@@ -49517,13 +49467,13 @@
         <v>42736</v>
       </c>
       <c r="C319" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D319" t="s">
-        <v>740</v>
+        <v>748</v>
       </c>
       <c r="E319" t="s">
-        <v>51</v>
+        <v>141</v>
       </c>
       <c r="F319">
         <v>1</v>
@@ -49549,16 +49499,16 @@
         <v>42736</v>
       </c>
       <c r="C320" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D320" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="E320" t="s">
-        <v>51</v>
+        <v>436</v>
       </c>
       <c r="F320">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G320" t="s">
         <v>1178</v>
@@ -49587,10 +49537,10 @@
         <v>748</v>
       </c>
       <c r="E321" t="s">
-        <v>141</v>
+        <v>438</v>
       </c>
       <c r="F321">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G321" t="s">
         <v>1178</v>
@@ -49610,25 +49560,25 @@
     </row>
     <row r="322" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A322" s="1">
-        <v>42736</v>
+        <v>42756</v>
       </c>
       <c r="C322" t="s">
         <v>150</v>
       </c>
       <c r="D322" t="s">
-        <v>748</v>
+        <v>827</v>
       </c>
       <c r="E322" t="s">
-        <v>436</v>
+        <v>442</v>
       </c>
       <c r="F322">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G322" t="s">
-        <v>1178</v>
+        <v>1258</v>
       </c>
       <c r="H322" t="s">
-        <v>1253</v>
+        <v>1322</v>
       </c>
       <c r="I322" t="s">
         <v>1254</v>
@@ -49642,25 +49592,25 @@
     </row>
     <row r="323" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A323" s="1">
-        <v>42736</v>
+        <v>42756</v>
       </c>
       <c r="C323" t="s">
         <v>150</v>
       </c>
       <c r="D323" t="s">
-        <v>748</v>
+        <v>827</v>
       </c>
       <c r="E323" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="F323">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G323" t="s">
-        <v>1178</v>
+        <v>1258</v>
       </c>
       <c r="H323" t="s">
-        <v>1253</v>
+        <v>1322</v>
       </c>
       <c r="I323" t="s">
         <v>1254</v>
@@ -49683,10 +49633,10 @@
         <v>827</v>
       </c>
       <c r="E324" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="F324">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G324" t="s">
         <v>1258</v>
@@ -49706,28 +49656,28 @@
     </row>
     <row r="325" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A325" s="1">
-        <v>42756</v>
+        <v>42736</v>
       </c>
       <c r="C325" t="s">
         <v>150</v>
       </c>
       <c r="D325" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
       <c r="E325" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
       <c r="F325">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G325" t="s">
         <v>1258</v>
       </c>
       <c r="H325" t="s">
-        <v>1322</v>
+        <v>1272</v>
       </c>
       <c r="I325" t="s">
-        <v>1254</v>
+        <v>293</v>
       </c>
       <c r="J325">
         <v>1</v>
@@ -49738,28 +49688,28 @@
     </row>
     <row r="326" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A326" s="1">
-        <v>42756</v>
+        <v>42736</v>
       </c>
       <c r="C326" t="s">
         <v>150</v>
       </c>
       <c r="D326" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="E326" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="F326">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G326" t="s">
         <v>1258</v>
       </c>
       <c r="H326" t="s">
-        <v>1322</v>
+        <v>1272</v>
       </c>
       <c r="I326" t="s">
-        <v>1254</v>
+        <v>293</v>
       </c>
       <c r="J326">
         <v>1</v>
@@ -49776,13 +49726,13 @@
         <v>150</v>
       </c>
       <c r="D327" t="s">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="E327" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="F327">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G327" t="s">
         <v>1258</v>
@@ -49811,10 +49761,10 @@
         <v>826</v>
       </c>
       <c r="E328" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="F328">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G328" t="s">
         <v>1258</v>
@@ -49843,10 +49793,10 @@
         <v>826</v>
       </c>
       <c r="E329" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="F329">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G329" t="s">
         <v>1258</v>
@@ -49869,25 +49819,25 @@
         <v>42736</v>
       </c>
       <c r="C330" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D330" t="s">
-        <v>826</v>
+        <v>748</v>
       </c>
       <c r="E330" t="s">
-        <v>444</v>
+        <v>141</v>
       </c>
       <c r="F330">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G330" t="s">
-        <v>1258</v>
+        <v>1178</v>
       </c>
       <c r="H330" t="s">
-        <v>1272</v>
+        <v>1253</v>
       </c>
       <c r="I330" t="s">
-        <v>293</v>
+        <v>1254</v>
       </c>
       <c r="J330">
         <v>1</v>
@@ -49901,25 +49851,25 @@
         <v>42736</v>
       </c>
       <c r="C331" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D331" t="s">
-        <v>826</v>
+        <v>748</v>
       </c>
       <c r="E331" t="s">
-        <v>446</v>
+        <v>436</v>
       </c>
       <c r="F331">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G331" t="s">
-        <v>1258</v>
+        <v>1178</v>
       </c>
       <c r="H331" t="s">
-        <v>1272</v>
+        <v>1253</v>
       </c>
       <c r="I331" t="s">
-        <v>293</v>
+        <v>1254</v>
       </c>
       <c r="J331">
         <v>1</v>
@@ -49939,10 +49889,10 @@
         <v>748</v>
       </c>
       <c r="E332" t="s">
-        <v>141</v>
+        <v>438</v>
       </c>
       <c r="F332">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G332" t="s">
         <v>1178</v>
@@ -49968,22 +49918,22 @@
         <v>151</v>
       </c>
       <c r="D333" t="s">
-        <v>748</v>
+        <v>828</v>
       </c>
       <c r="E333" t="s">
-        <v>436</v>
+        <v>446</v>
       </c>
       <c r="F333">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G333" t="s">
-        <v>1178</v>
+        <v>1258</v>
       </c>
       <c r="H333" t="s">
-        <v>1253</v>
+        <v>1272</v>
       </c>
       <c r="I333" t="s">
-        <v>1254</v>
+        <v>293</v>
       </c>
       <c r="J333">
         <v>1</v>
@@ -50000,22 +49950,22 @@
         <v>151</v>
       </c>
       <c r="D334" t="s">
-        <v>748</v>
+        <v>826</v>
       </c>
       <c r="E334" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="F334">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G334" t="s">
-        <v>1178</v>
+        <v>1258</v>
       </c>
       <c r="H334" t="s">
-        <v>1253</v>
+        <v>1272</v>
       </c>
       <c r="I334" t="s">
-        <v>1254</v>
+        <v>293</v>
       </c>
       <c r="J334">
         <v>1</v>
@@ -50032,13 +49982,13 @@
         <v>151</v>
       </c>
       <c r="D335" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
       <c r="E335" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="F335">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G335" t="s">
         <v>1258</v>
@@ -50067,10 +50017,10 @@
         <v>826</v>
       </c>
       <c r="E336" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="F336">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G336" t="s">
         <v>1258</v>
@@ -50099,10 +50049,10 @@
         <v>826</v>
       </c>
       <c r="E337" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="F337">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G337" t="s">
         <v>1258</v>
@@ -50125,25 +50075,25 @@
         <v>42736</v>
       </c>
       <c r="C338" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D338" t="s">
-        <v>826</v>
+        <v>748</v>
       </c>
       <c r="E338" t="s">
-        <v>444</v>
+        <v>47</v>
       </c>
       <c r="F338">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G338" t="s">
-        <v>1258</v>
+        <v>1252</v>
       </c>
       <c r="H338" t="s">
-        <v>1272</v>
+        <v>1253</v>
       </c>
       <c r="I338" t="s">
-        <v>293</v>
+        <v>1314</v>
       </c>
       <c r="J338">
         <v>1</v>
@@ -50157,25 +50107,25 @@
         <v>42736</v>
       </c>
       <c r="C339" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D339" t="s">
-        <v>826</v>
+        <v>748</v>
       </c>
       <c r="E339" t="s">
-        <v>446</v>
+        <v>47</v>
       </c>
       <c r="F339">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G339" t="s">
-        <v>1258</v>
+        <v>1252</v>
       </c>
       <c r="H339" t="s">
-        <v>1272</v>
+        <v>1253</v>
       </c>
       <c r="I339" t="s">
-        <v>293</v>
+        <v>1314</v>
       </c>
       <c r="J339">
         <v>1</v>
@@ -50189,25 +50139,25 @@
         <v>42736</v>
       </c>
       <c r="C340" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D340" t="s">
-        <v>748</v>
+        <v>740</v>
       </c>
       <c r="E340" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F340">
         <v>1</v>
       </c>
       <c r="G340" t="s">
-        <v>1252</v>
+        <v>1178</v>
       </c>
       <c r="H340" t="s">
         <v>1253</v>
       </c>
       <c r="I340" t="s">
-        <v>1314</v>
+        <v>1254</v>
       </c>
       <c r="J340">
         <v>1</v>
@@ -50221,25 +50171,25 @@
         <v>42736</v>
       </c>
       <c r="C341" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D341" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
       <c r="E341" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F341">
         <v>1</v>
       </c>
       <c r="G341" t="s">
-        <v>1252</v>
+        <v>1178</v>
       </c>
       <c r="H341" t="s">
         <v>1253</v>
       </c>
       <c r="I341" t="s">
-        <v>1314</v>
+        <v>1254</v>
       </c>
       <c r="J341">
         <v>1</v>
@@ -50253,13 +50203,13 @@
         <v>42736</v>
       </c>
       <c r="C342" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D342" t="s">
         <v>740</v>
       </c>
       <c r="E342" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F342">
         <v>1</v>
@@ -50285,13 +50235,13 @@
         <v>42736</v>
       </c>
       <c r="C343" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D343" t="s">
-        <v>744</v>
+        <v>829</v>
       </c>
       <c r="E343" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F343">
         <v>1</v>
@@ -50320,7 +50270,7 @@
         <v>155</v>
       </c>
       <c r="D344" t="s">
-        <v>740</v>
+        <v>830</v>
       </c>
       <c r="E344" t="s">
         <v>47</v>
@@ -50349,10 +50299,10 @@
         <v>42736</v>
       </c>
       <c r="C345" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D345" t="s">
-        <v>829</v>
+        <v>748</v>
       </c>
       <c r="E345" t="s">
         <v>47</v>
@@ -50361,7 +50311,7 @@
         <v>1</v>
       </c>
       <c r="G345" t="s">
-        <v>1178</v>
+        <v>1252</v>
       </c>
       <c r="H345" t="s">
         <v>1253</v>
@@ -50381,19 +50331,19 @@
         <v>42736</v>
       </c>
       <c r="C346" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D346" t="s">
-        <v>830</v>
+        <v>748</v>
       </c>
       <c r="E346" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="F346">
         <v>1</v>
       </c>
       <c r="G346" t="s">
-        <v>1178</v>
+        <v>1252</v>
       </c>
       <c r="H346" t="s">
         <v>1253</v>
@@ -50413,19 +50363,19 @@
         <v>42736</v>
       </c>
       <c r="C347" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D347" t="s">
         <v>748</v>
       </c>
       <c r="E347" t="s">
-        <v>47</v>
+        <v>447</v>
       </c>
       <c r="F347">
         <v>1</v>
       </c>
       <c r="G347" t="s">
-        <v>1252</v>
+        <v>1258</v>
       </c>
       <c r="H347" t="s">
         <v>1253</v>
@@ -50445,19 +50395,19 @@
         <v>42736</v>
       </c>
       <c r="C348" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D348" t="s">
         <v>748</v>
       </c>
       <c r="E348" t="s">
-        <v>13</v>
+        <v>450</v>
       </c>
       <c r="F348">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G348" t="s">
-        <v>1252</v>
+        <v>1258</v>
       </c>
       <c r="H348" t="s">
         <v>1253</v>
@@ -50466,7 +50416,7 @@
         <v>1254</v>
       </c>
       <c r="J348">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P348" t="s">
         <v>405</v>
@@ -50480,7 +50430,7 @@
         <v>157</v>
       </c>
       <c r="D349" t="s">
-        <v>748</v>
+        <v>831</v>
       </c>
       <c r="E349" t="s">
         <v>447</v>
@@ -50512,7 +50462,7 @@
         <v>157</v>
       </c>
       <c r="D350" t="s">
-        <v>748</v>
+        <v>831</v>
       </c>
       <c r="E350" t="s">
         <v>450</v>
@@ -50544,7 +50494,7 @@
         <v>157</v>
       </c>
       <c r="D351" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="E351" t="s">
         <v>447</v>
@@ -50573,19 +50523,19 @@
         <v>42736</v>
       </c>
       <c r="C352" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D352" t="s">
-        <v>831</v>
+        <v>740</v>
       </c>
       <c r="E352" t="s">
-        <v>450</v>
+        <v>51</v>
       </c>
       <c r="F352">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G352" t="s">
-        <v>1258</v>
+        <v>1178</v>
       </c>
       <c r="H352" t="s">
         <v>1253</v>
@@ -50594,7 +50544,7 @@
         <v>1254</v>
       </c>
       <c r="J352">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P352" t="s">
         <v>405</v>
@@ -50605,19 +50555,19 @@
         <v>42736</v>
       </c>
       <c r="C353" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D353" t="s">
-        <v>832</v>
+        <v>744</v>
       </c>
       <c r="E353" t="s">
-        <v>447</v>
+        <v>51</v>
       </c>
       <c r="F353">
         <v>1</v>
       </c>
       <c r="G353" t="s">
-        <v>1258</v>
+        <v>1178</v>
       </c>
       <c r="H353" t="s">
         <v>1253</v>
@@ -50640,7 +50590,7 @@
         <v>161</v>
       </c>
       <c r="D354" t="s">
-        <v>740</v>
+        <v>833</v>
       </c>
       <c r="E354" t="s">
         <v>51</v>
@@ -50666,22 +50616,22 @@
     </row>
     <row r="355" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A355" s="1">
-        <v>42736</v>
+        <v>42741</v>
       </c>
       <c r="C355" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D355" t="s">
-        <v>744</v>
+        <v>740</v>
       </c>
       <c r="E355" t="s">
-        <v>51</v>
+        <v>163</v>
       </c>
       <c r="F355">
         <v>1</v>
       </c>
       <c r="G355" t="s">
-        <v>1178</v>
+        <v>1252</v>
       </c>
       <c r="H355" t="s">
         <v>1253</v>
@@ -50698,22 +50648,22 @@
     </row>
     <row r="356" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A356" s="1">
-        <v>42736</v>
+        <v>42742</v>
       </c>
       <c r="C356" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D356" t="s">
-        <v>833</v>
+        <v>740</v>
       </c>
       <c r="E356" t="s">
-        <v>51</v>
+        <v>165</v>
       </c>
       <c r="F356">
         <v>1</v>
       </c>
       <c r="G356" t="s">
-        <v>1178</v>
+        <v>1252</v>
       </c>
       <c r="H356" t="s">
         <v>1253</v>
@@ -50730,7 +50680,7 @@
     </row>
     <row r="357" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A357" s="1">
-        <v>42741</v>
+        <v>42743</v>
       </c>
       <c r="C357" t="s">
         <v>162</v>
@@ -50739,7 +50689,7 @@
         <v>740</v>
       </c>
       <c r="E357" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="F357">
         <v>1</v>
@@ -50762,7 +50712,7 @@
     </row>
     <row r="358" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A358" s="1">
-        <v>42742</v>
+        <v>42744</v>
       </c>
       <c r="C358" t="s">
         <v>162</v>
@@ -50771,7 +50721,7 @@
         <v>740</v>
       </c>
       <c r="E358" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="F358">
         <v>1</v>
@@ -50794,7 +50744,7 @@
     </row>
     <row r="359" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A359" s="1">
-        <v>42743</v>
+        <v>42741</v>
       </c>
       <c r="C359" t="s">
         <v>162</v>
@@ -50803,7 +50753,7 @@
         <v>740</v>
       </c>
       <c r="E359" t="s">
-        <v>167</v>
+        <v>458</v>
       </c>
       <c r="F359">
         <v>1</v>
@@ -50826,7 +50776,7 @@
     </row>
     <row r="360" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A360" s="1">
-        <v>42744</v>
+        <v>42742</v>
       </c>
       <c r="C360" t="s">
         <v>162</v>
@@ -50835,7 +50785,7 @@
         <v>740</v>
       </c>
       <c r="E360" t="s">
-        <v>169</v>
+        <v>460</v>
       </c>
       <c r="F360">
         <v>1</v>
@@ -50858,7 +50808,7 @@
     </row>
     <row r="361" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A361" s="1">
-        <v>42741</v>
+        <v>42743</v>
       </c>
       <c r="C361" t="s">
         <v>162</v>
@@ -50867,7 +50817,7 @@
         <v>740</v>
       </c>
       <c r="E361" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="F361">
         <v>1</v>
@@ -50885,70 +50835,6 @@
         <v>1</v>
       </c>
       <c r="P361" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="362" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A362" s="1">
-        <v>42742</v>
-      </c>
-      <c r="C362" t="s">
-        <v>162</v>
-      </c>
-      <c r="D362" t="s">
-        <v>740</v>
-      </c>
-      <c r="E362" t="s">
-        <v>460</v>
-      </c>
-      <c r="F362">
-        <v>1</v>
-      </c>
-      <c r="G362" t="s">
-        <v>1252</v>
-      </c>
-      <c r="H362" t="s">
-        <v>1253</v>
-      </c>
-      <c r="I362" t="s">
-        <v>1254</v>
-      </c>
-      <c r="J362">
-        <v>1</v>
-      </c>
-      <c r="P362" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="363" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A363" s="1">
-        <v>42743</v>
-      </c>
-      <c r="C363" t="s">
-        <v>162</v>
-      </c>
-      <c r="D363" t="s">
-        <v>740</v>
-      </c>
-      <c r="E363" t="s">
-        <v>463</v>
-      </c>
-      <c r="F363">
-        <v>1</v>
-      </c>
-      <c r="G363" t="s">
-        <v>1252</v>
-      </c>
-      <c r="H363" t="s">
-        <v>1253</v>
-      </c>
-      <c r="I363" t="s">
-        <v>1254</v>
-      </c>
-      <c r="J363">
-        <v>1</v>
-      </c>
-      <c r="P363" t="s">
         <v>405</v>
       </c>
     </row>
@@ -56617,13 +56503,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Q311"/>
+  <dimension ref="A1:Q310"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="3" max="3" width="24" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="27.33203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -62658,7 +62539,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="257" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A257" s="1">
         <v>42738</v>
       </c>
@@ -62681,7 +62562,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="258" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A258" s="1">
         <v>42738</v>
       </c>
@@ -62704,7 +62585,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="259" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A259" s="1">
         <v>42736</v>
       </c>
@@ -62730,18 +62611,18 @@
         <v>197</v>
       </c>
     </row>
-    <row r="260" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A260" s="1">
-        <v>42738</v>
+        <v>42736</v>
       </c>
       <c r="C260" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="D260" t="s">
-        <v>1537</v>
+        <v>47</v>
       </c>
       <c r="E260" t="s">
-        <v>1538</v>
+        <v>47</v>
       </c>
       <c r="G260" t="s">
         <v>224</v>
@@ -62752,16 +62633,13 @@
       <c r="N260" t="s">
         <v>197</v>
       </c>
-      <c r="O260" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="261" spans="1:15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="261" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A261" s="1">
         <v>42736</v>
       </c>
       <c r="C261" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D261" t="s">
         <v>47</v>
@@ -62779,21 +62657,21 @@
         <v>197</v>
       </c>
     </row>
-    <row r="262" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A262" s="1">
         <v>42736</v>
       </c>
       <c r="C262" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D262" t="s">
-        <v>47</v>
+        <v>239</v>
       </c>
       <c r="E262" t="s">
-        <v>47</v>
+        <v>240</v>
       </c>
       <c r="G262" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="K262" t="s">
         <v>218</v>
@@ -62802,7 +62680,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="263" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A263" s="1">
         <v>42736</v>
       </c>
@@ -62810,13 +62688,13 @@
         <v>140</v>
       </c>
       <c r="D263" t="s">
-        <v>239</v>
+        <v>141</v>
       </c>
       <c r="E263" t="s">
-        <v>240</v>
+        <v>434</v>
       </c>
       <c r="G263" t="s">
-        <v>214</v>
+        <v>435</v>
       </c>
       <c r="K263" t="s">
         <v>218</v>
@@ -62825,7 +62703,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="264" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A264" s="1">
         <v>42736</v>
       </c>
@@ -62833,10 +62711,10 @@
         <v>140</v>
       </c>
       <c r="D264" t="s">
-        <v>141</v>
+        <v>436</v>
       </c>
       <c r="E264" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="G264" t="s">
         <v>435</v>
@@ -62848,7 +62726,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="265" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A265" s="1">
         <v>42736</v>
       </c>
@@ -62856,10 +62734,10 @@
         <v>140</v>
       </c>
       <c r="D265" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="E265" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="G265" t="s">
         <v>435</v>
@@ -62871,7 +62749,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="266" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A266" s="1">
         <v>42736</v>
       </c>
@@ -62879,13 +62757,13 @@
         <v>140</v>
       </c>
       <c r="D266" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E266" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="G266" t="s">
-        <v>435</v>
+        <v>291</v>
       </c>
       <c r="K266" t="s">
         <v>218</v>
@@ -62894,7 +62772,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="267" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A267" s="1">
         <v>42736</v>
       </c>
@@ -62902,10 +62780,10 @@
         <v>140</v>
       </c>
       <c r="D267" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E267" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="G267" t="s">
         <v>291</v>
@@ -62917,7 +62795,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="268" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A268" s="1">
         <v>42736</v>
       </c>
@@ -62925,10 +62803,10 @@
         <v>140</v>
       </c>
       <c r="D268" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="E268" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="G268" t="s">
         <v>291</v>
@@ -62940,7 +62818,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="269" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A269" s="1">
         <v>42736</v>
       </c>
@@ -62948,13 +62826,13 @@
         <v>140</v>
       </c>
       <c r="D269" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E269" t="s">
-        <v>445</v>
+        <v>293</v>
       </c>
       <c r="G269" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="K269" t="s">
         <v>218</v>
@@ -62963,21 +62841,21 @@
         <v>197</v>
       </c>
     </row>
-    <row r="270" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A270" s="1">
         <v>42736</v>
       </c>
       <c r="C270" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="D270" t="s">
-        <v>446</v>
+        <v>51</v>
       </c>
       <c r="E270" t="s">
-        <v>293</v>
+        <v>52</v>
       </c>
       <c r="G270" t="s">
-        <v>294</v>
+        <v>51</v>
       </c>
       <c r="K270" t="s">
         <v>218</v>
@@ -62986,7 +62864,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="271" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A271" s="1">
         <v>42736</v>
       </c>
@@ -62994,13 +62872,13 @@
         <v>149</v>
       </c>
       <c r="D271" t="s">
-        <v>51</v>
+        <v>239</v>
       </c>
       <c r="E271" t="s">
-        <v>52</v>
+        <v>240</v>
       </c>
       <c r="G271" t="s">
-        <v>51</v>
+        <v>214</v>
       </c>
       <c r="K271" t="s">
         <v>218</v>
@@ -63009,12 +62887,12 @@
         <v>197</v>
       </c>
     </row>
-    <row r="272" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A272" s="1">
         <v>42736</v>
       </c>
       <c r="C272" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D272" t="s">
         <v>239</v>
@@ -63040,13 +62918,13 @@
         <v>150</v>
       </c>
       <c r="D273" t="s">
-        <v>239</v>
+        <v>141</v>
       </c>
       <c r="E273" t="s">
-        <v>240</v>
+        <v>434</v>
       </c>
       <c r="G273" t="s">
-        <v>214</v>
+        <v>435</v>
       </c>
       <c r="K273" t="s">
         <v>218</v>
@@ -63063,10 +62941,10 @@
         <v>150</v>
       </c>
       <c r="D274" t="s">
-        <v>141</v>
+        <v>436</v>
       </c>
       <c r="E274" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="G274" t="s">
         <v>435</v>
@@ -63086,10 +62964,10 @@
         <v>150</v>
       </c>
       <c r="D275" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="E275" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="G275" t="s">
         <v>435</v>
@@ -63109,13 +62987,13 @@
         <v>150</v>
       </c>
       <c r="D276" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E276" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="G276" t="s">
-        <v>435</v>
+        <v>291</v>
       </c>
       <c r="K276" t="s">
         <v>218</v>
@@ -63132,10 +63010,10 @@
         <v>150</v>
       </c>
       <c r="D277" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E277" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="G277" t="s">
         <v>291</v>
@@ -63155,10 +63033,10 @@
         <v>150</v>
       </c>
       <c r="D278" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="E278" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="G278" t="s">
         <v>291</v>
@@ -63178,13 +63056,13 @@
         <v>150</v>
       </c>
       <c r="D279" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E279" t="s">
-        <v>445</v>
+        <v>293</v>
       </c>
       <c r="G279" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="K279" t="s">
         <v>218</v>
@@ -63198,16 +63076,16 @@
         <v>42736</v>
       </c>
       <c r="C280" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D280" t="s">
-        <v>446</v>
+        <v>239</v>
       </c>
       <c r="E280" t="s">
-        <v>293</v>
+        <v>240</v>
       </c>
       <c r="G280" t="s">
-        <v>294</v>
+        <v>214</v>
       </c>
       <c r="K280" t="s">
         <v>218</v>
@@ -63224,13 +63102,13 @@
         <v>151</v>
       </c>
       <c r="D281" t="s">
-        <v>239</v>
+        <v>141</v>
       </c>
       <c r="E281" t="s">
-        <v>240</v>
+        <v>434</v>
       </c>
       <c r="G281" t="s">
-        <v>214</v>
+        <v>435</v>
       </c>
       <c r="K281" t="s">
         <v>218</v>
@@ -63247,10 +63125,10 @@
         <v>151</v>
       </c>
       <c r="D282" t="s">
-        <v>141</v>
+        <v>436</v>
       </c>
       <c r="E282" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="G282" t="s">
         <v>435</v>
@@ -63270,10 +63148,10 @@
         <v>151</v>
       </c>
       <c r="D283" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="E283" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="G283" t="s">
         <v>435</v>
@@ -63293,13 +63171,13 @@
         <v>151</v>
       </c>
       <c r="D284" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E284" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="G284" t="s">
-        <v>435</v>
+        <v>291</v>
       </c>
       <c r="K284" t="s">
         <v>218</v>
@@ -63316,10 +63194,10 @@
         <v>151</v>
       </c>
       <c r="D285" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="E285" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="G285" t="s">
         <v>291</v>
@@ -63339,10 +63217,10 @@
         <v>151</v>
       </c>
       <c r="D286" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="E286" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="G286" t="s">
         <v>291</v>
@@ -63362,13 +63240,13 @@
         <v>151</v>
       </c>
       <c r="D287" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="E287" t="s">
-        <v>445</v>
+        <v>293</v>
       </c>
       <c r="G287" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="K287" t="s">
         <v>218</v>
@@ -63382,16 +63260,16 @@
         <v>42736</v>
       </c>
       <c r="C288" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D288" t="s">
-        <v>446</v>
+        <v>47</v>
       </c>
       <c r="E288" t="s">
-        <v>293</v>
+        <v>47</v>
       </c>
       <c r="G288" t="s">
-        <v>294</v>
+        <v>224</v>
       </c>
       <c r="K288" t="s">
         <v>218</v>
@@ -63405,7 +63283,7 @@
         <v>42736</v>
       </c>
       <c r="C289" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D289" t="s">
         <v>47</v>
@@ -63428,16 +63306,16 @@
         <v>42736</v>
       </c>
       <c r="C290" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D290" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E290" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="G290" t="s">
-        <v>224</v>
+        <v>51</v>
       </c>
       <c r="K290" t="s">
         <v>218</v>
@@ -63454,13 +63332,13 @@
         <v>154</v>
       </c>
       <c r="D291" t="s">
-        <v>51</v>
+        <v>239</v>
       </c>
       <c r="E291" t="s">
-        <v>52</v>
+        <v>240</v>
       </c>
       <c r="G291" t="s">
-        <v>51</v>
+        <v>214</v>
       </c>
       <c r="K291" t="s">
         <v>218</v>
@@ -63474,16 +63352,16 @@
         <v>42736</v>
       </c>
       <c r="C292" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D292" t="s">
-        <v>239</v>
+        <v>47</v>
       </c>
       <c r="E292" t="s">
-        <v>240</v>
+        <v>47</v>
       </c>
       <c r="G292" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="K292" t="s">
         <v>218</v>
@@ -63497,13 +63375,13 @@
         <v>42736</v>
       </c>
       <c r="C293" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D293" t="s">
         <v>47</v>
       </c>
       <c r="E293" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G293" t="s">
         <v>224</v>
@@ -63523,13 +63401,13 @@
         <v>156</v>
       </c>
       <c r="D294" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="E294" t="s">
-        <v>48</v>
+        <v>117</v>
       </c>
       <c r="G294" t="s">
-        <v>224</v>
+        <v>199</v>
       </c>
       <c r="K294" t="s">
         <v>218</v>
@@ -63546,13 +63424,13 @@
         <v>156</v>
       </c>
       <c r="D295" t="s">
-        <v>13</v>
+        <v>239</v>
       </c>
       <c r="E295" t="s">
-        <v>117</v>
+        <v>240</v>
       </c>
       <c r="G295" t="s">
-        <v>199</v>
+        <v>214</v>
       </c>
       <c r="K295" t="s">
         <v>218</v>
@@ -63566,16 +63444,19 @@
         <v>42736</v>
       </c>
       <c r="C296" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D296" t="s">
-        <v>239</v>
+        <v>447</v>
       </c>
       <c r="E296" t="s">
-        <v>240</v>
+        <v>448</v>
       </c>
       <c r="G296" t="s">
-        <v>214</v>
+        <v>206</v>
+      </c>
+      <c r="I296" t="s">
+        <v>449</v>
       </c>
       <c r="K296" t="s">
         <v>218</v>
@@ -63592,16 +63473,13 @@
         <v>157</v>
       </c>
       <c r="D297" t="s">
-        <v>447</v>
+        <v>158</v>
       </c>
       <c r="E297" t="s">
-        <v>448</v>
+        <v>158</v>
       </c>
       <c r="G297" t="s">
-        <v>206</v>
-      </c>
-      <c r="I297" t="s">
-        <v>449</v>
+        <v>224</v>
       </c>
       <c r="K297" t="s">
         <v>218</v>
@@ -63618,13 +63496,16 @@
         <v>157</v>
       </c>
       <c r="D298" t="s">
-        <v>158</v>
+        <v>450</v>
       </c>
       <c r="E298" t="s">
-        <v>158</v>
+        <v>451</v>
       </c>
       <c r="G298" t="s">
-        <v>224</v>
+        <v>206</v>
+      </c>
+      <c r="I298" t="s">
+        <v>452</v>
       </c>
       <c r="K298" t="s">
         <v>218</v>
@@ -63638,19 +63519,16 @@
         <v>42736</v>
       </c>
       <c r="C299" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D299" t="s">
-        <v>450</v>
+        <v>47</v>
       </c>
       <c r="E299" t="s">
-        <v>451</v>
+        <v>47</v>
       </c>
       <c r="G299" t="s">
-        <v>206</v>
-      </c>
-      <c r="I299" t="s">
-        <v>452</v>
+        <v>224</v>
       </c>
       <c r="K299" t="s">
         <v>218</v>
@@ -63664,7 +63542,7 @@
         <v>42736</v>
       </c>
       <c r="C300" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D300" t="s">
         <v>47</v>
@@ -63687,16 +63565,16 @@
         <v>42736</v>
       </c>
       <c r="C301" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D301" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E301" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="G301" t="s">
-        <v>224</v>
+        <v>51</v>
       </c>
       <c r="K301" t="s">
         <v>218</v>
@@ -63713,13 +63591,13 @@
         <v>161</v>
       </c>
       <c r="D302" t="s">
-        <v>51</v>
+        <v>239</v>
       </c>
       <c r="E302" t="s">
-        <v>52</v>
+        <v>240</v>
       </c>
       <c r="G302" t="s">
-        <v>51</v>
+        <v>214</v>
       </c>
       <c r="K302" t="s">
         <v>218</v>
@@ -63733,16 +63611,19 @@
         <v>42736</v>
       </c>
       <c r="C303" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D303" t="s">
-        <v>239</v>
+        <v>163</v>
       </c>
       <c r="E303" t="s">
-        <v>240</v>
+        <v>164</v>
       </c>
       <c r="G303" t="s">
-        <v>214</v>
+        <v>216</v>
+      </c>
+      <c r="H303" t="s">
+        <v>453</v>
       </c>
       <c r="K303" t="s">
         <v>218</v>
@@ -63759,16 +63640,16 @@
         <v>162</v>
       </c>
       <c r="D304" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="E304" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="G304" t="s">
         <v>216</v>
       </c>
       <c r="H304" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="K304" t="s">
         <v>218</v>
@@ -63785,17 +63666,14 @@
         <v>162</v>
       </c>
       <c r="D305" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E305" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="G305" t="s">
         <v>216</v>
       </c>
-      <c r="H305" t="s">
-        <v>454</v>
-      </c>
       <c r="K305" t="s">
         <v>218</v>
       </c>
@@ -63811,13 +63689,13 @@
         <v>162</v>
       </c>
       <c r="D306" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="E306" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="G306" t="s">
-        <v>216</v>
+        <v>455</v>
       </c>
       <c r="K306" t="s">
         <v>218</v>
@@ -63834,13 +63712,13 @@
         <v>162</v>
       </c>
       <c r="D307" t="s">
-        <v>169</v>
+        <v>456</v>
       </c>
       <c r="E307" t="s">
-        <v>170</v>
+        <v>457</v>
       </c>
       <c r="G307" t="s">
-        <v>455</v>
+        <v>224</v>
       </c>
       <c r="K307" t="s">
         <v>218</v>
@@ -63857,13 +63735,19 @@
         <v>162</v>
       </c>
       <c r="D308" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="E308" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="G308" t="s">
-        <v>224</v>
+        <v>206</v>
+      </c>
+      <c r="H308" t="s">
+        <v>453</v>
+      </c>
+      <c r="I308" t="s">
+        <v>216</v>
       </c>
       <c r="K308" t="s">
         <v>218</v>
@@ -63880,19 +63764,16 @@
         <v>162</v>
       </c>
       <c r="D309" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="E309" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="G309" t="s">
         <v>206</v>
       </c>
-      <c r="H309" t="s">
-        <v>453</v>
-      </c>
       <c r="I309" t="s">
-        <v>216</v>
+        <v>462</v>
       </c>
       <c r="K309" t="s">
         <v>218</v>
@@ -63909,47 +63790,21 @@
         <v>162</v>
       </c>
       <c r="D310" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="E310" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="G310" t="s">
         <v>206</v>
       </c>
       <c r="I310" t="s">
-        <v>462</v>
+        <v>216</v>
       </c>
       <c r="K310" t="s">
         <v>218</v>
       </c>
       <c r="N310" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="311" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A311" s="1">
-        <v>42736</v>
-      </c>
-      <c r="C311" t="s">
-        <v>162</v>
-      </c>
-      <c r="D311" t="s">
-        <v>463</v>
-      </c>
-      <c r="E311" t="s">
-        <v>464</v>
-      </c>
-      <c r="G311" t="s">
-        <v>206</v>
-      </c>
-      <c r="I311" t="s">
-        <v>216</v>
-      </c>
-      <c r="K311" t="s">
-        <v>218</v>
-      </c>
-      <c r="N311" t="s">
         <v>197</v>
       </c>
     </row>

</xml_diff>

<commit_message>
CCD-8066: updated with master
</commit_message>
<xml_diff>
--- a/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_Master_Definition.xlsx
+++ b/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/BEFTA_Master_Definition.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jen/IdeaProjects/test-defs-jen/ccd-test-definitions/src/main/resources/uk/gov/hmcts/ccd/test_definitions/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{292B7B28-3B2C-3142-854C-3C64141921F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE82AF4E-0597-364D-9EE1-7BC4A2A2EBC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18020" firstSheet="14" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17900" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SearchInputFields" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16031" uniqueCount="1537">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16061" uniqueCount="1540">
   <si>
     <t>SearchInputFields</t>
   </si>
@@ -4660,13 +4660,22 @@
   </si>
   <si>
     <t>${MCA_API_BASE_URL:http://aac-manage-case-assignment-aat.service.core-compute-aat.internal}/noc/apply-decision</t>
+  </si>
+  <si>
+    <t>StaffUser</t>
+  </si>
+  <si>
+    <t>Staff User Fields</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#ARGUMENT(CATEGORY-LEGAL-OPS,CATEGORY-ADMIN,REGION-1235) </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -4681,6 +4690,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF172B4D"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -4704,10 +4719,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -7737,6 +7753,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:L152"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="15.6640625" customWidth="1"/>
+    <col min="8" max="8" width="17.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -31057,8 +31077,13 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
-  <dimension ref="A1:F477"/>
+  <dimension ref="A1:F479"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="36.83203125" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" customWidth="1"/>
+    <col min="5" max="5" width="8.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -37125,10 +37150,10 @@
         <v>42736</v>
       </c>
       <c r="C359" t="s">
-        <v>138</v>
+        <v>114</v>
       </c>
       <c r="D359" t="s">
-        <v>47</v>
+        <v>1537</v>
       </c>
       <c r="E359" t="s">
         <v>644</v>
@@ -37142,13 +37167,13 @@
         <v>42736</v>
       </c>
       <c r="C360" t="s">
-        <v>139</v>
+        <v>114</v>
       </c>
       <c r="D360" t="s">
-        <v>47</v>
+        <v>1537</v>
       </c>
       <c r="E360" t="s">
-        <v>644</v>
+        <v>727</v>
       </c>
       <c r="F360" t="s">
         <v>643</v>
@@ -37159,13 +37184,13 @@
         <v>42736</v>
       </c>
       <c r="C361" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D361" t="s">
-        <v>239</v>
+        <v>47</v>
       </c>
       <c r="E361" t="s">
-        <v>735</v>
+        <v>644</v>
       </c>
       <c r="F361" t="s">
         <v>643</v>
@@ -37176,13 +37201,13 @@
         <v>42736</v>
       </c>
       <c r="C362" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D362" t="s">
-        <v>141</v>
+        <v>47</v>
       </c>
       <c r="E362" t="s">
-        <v>735</v>
+        <v>644</v>
       </c>
       <c r="F362" t="s">
         <v>643</v>
@@ -37196,7 +37221,7 @@
         <v>140</v>
       </c>
       <c r="D363" t="s">
-        <v>436</v>
+        <v>239</v>
       </c>
       <c r="E363" t="s">
         <v>735</v>
@@ -37213,7 +37238,7 @@
         <v>140</v>
       </c>
       <c r="D364" t="s">
-        <v>438</v>
+        <v>141</v>
       </c>
       <c r="E364" t="s">
         <v>735</v>
@@ -37230,7 +37255,7 @@
         <v>140</v>
       </c>
       <c r="D365" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="E365" t="s">
         <v>735</v>
@@ -37247,7 +37272,7 @@
         <v>140</v>
       </c>
       <c r="D366" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="E366" t="s">
         <v>735</v>
@@ -37264,7 +37289,7 @@
         <v>140</v>
       </c>
       <c r="D367" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="E367" t="s">
         <v>735</v>
@@ -37281,7 +37306,7 @@
         <v>140</v>
       </c>
       <c r="D368" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E368" t="s">
         <v>735</v>
@@ -37298,10 +37323,10 @@
         <v>140</v>
       </c>
       <c r="D369" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="E369" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="F369" t="s">
         <v>643</v>
@@ -37315,10 +37340,10 @@
         <v>140</v>
       </c>
       <c r="D370" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="E370" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="F370" t="s">
         <v>643</v>
@@ -37332,7 +37357,7 @@
         <v>140</v>
       </c>
       <c r="D371" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="E371" t="s">
         <v>736</v>
@@ -37349,7 +37374,7 @@
         <v>140</v>
       </c>
       <c r="D372" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E372" t="s">
         <v>736</v>
@@ -37366,10 +37391,10 @@
         <v>140</v>
       </c>
       <c r="D373" t="s">
-        <v>239</v>
+        <v>444</v>
       </c>
       <c r="E373" t="s">
-        <v>644</v>
+        <v>736</v>
       </c>
       <c r="F373" t="s">
         <v>643</v>
@@ -37383,10 +37408,10 @@
         <v>140</v>
       </c>
       <c r="D374" t="s">
-        <v>141</v>
+        <v>446</v>
       </c>
       <c r="E374" t="s">
-        <v>644</v>
+        <v>736</v>
       </c>
       <c r="F374" t="s">
         <v>643</v>
@@ -37400,7 +37425,7 @@
         <v>140</v>
       </c>
       <c r="D375" t="s">
-        <v>436</v>
+        <v>239</v>
       </c>
       <c r="E375" t="s">
         <v>644</v>
@@ -37417,7 +37442,7 @@
         <v>140</v>
       </c>
       <c r="D376" t="s">
-        <v>438</v>
+        <v>141</v>
       </c>
       <c r="E376" t="s">
         <v>644</v>
@@ -37434,7 +37459,7 @@
         <v>140</v>
       </c>
       <c r="D377" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="E377" t="s">
         <v>644</v>
@@ -37451,7 +37476,7 @@
         <v>140</v>
       </c>
       <c r="D378" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="E378" t="s">
         <v>644</v>
@@ -37468,7 +37493,7 @@
         <v>140</v>
       </c>
       <c r="D379" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="E379" t="s">
         <v>644</v>
@@ -37485,7 +37510,7 @@
         <v>140</v>
       </c>
       <c r="D380" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E380" t="s">
         <v>644</v>
@@ -37499,10 +37524,10 @@
         <v>42736</v>
       </c>
       <c r="C381" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="D381" t="s">
-        <v>239</v>
+        <v>444</v>
       </c>
       <c r="E381" t="s">
         <v>644</v>
@@ -37516,10 +37541,10 @@
         <v>42736</v>
       </c>
       <c r="C382" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="D382" t="s">
-        <v>51</v>
+        <v>446</v>
       </c>
       <c r="E382" t="s">
         <v>644</v>
@@ -37536,10 +37561,10 @@
         <v>149</v>
       </c>
       <c r="D383" t="s">
-        <v>51</v>
+        <v>239</v>
       </c>
       <c r="E383" t="s">
-        <v>718</v>
+        <v>644</v>
       </c>
       <c r="F383" t="s">
         <v>643</v>
@@ -37550,13 +37575,13 @@
         <v>42736</v>
       </c>
       <c r="C384" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D384" t="s">
-        <v>239</v>
+        <v>51</v>
       </c>
       <c r="E384" t="s">
-        <v>710</v>
+        <v>644</v>
       </c>
       <c r="F384" t="s">
         <v>643</v>
@@ -37567,13 +37592,13 @@
         <v>42736</v>
       </c>
       <c r="C385" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D385" t="s">
-        <v>141</v>
+        <v>51</v>
       </c>
       <c r="E385" t="s">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="F385" t="s">
         <v>643</v>
@@ -37587,7 +37612,7 @@
         <v>150</v>
       </c>
       <c r="D386" t="s">
-        <v>436</v>
+        <v>239</v>
       </c>
       <c r="E386" t="s">
         <v>710</v>
@@ -37604,7 +37629,7 @@
         <v>150</v>
       </c>
       <c r="D387" t="s">
-        <v>438</v>
+        <v>141</v>
       </c>
       <c r="E387" t="s">
         <v>710</v>
@@ -37621,7 +37646,7 @@
         <v>150</v>
       </c>
       <c r="D388" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="E388" t="s">
         <v>710</v>
@@ -37638,7 +37663,7 @@
         <v>150</v>
       </c>
       <c r="D389" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="E389" t="s">
         <v>710</v>
@@ -37655,7 +37680,7 @@
         <v>150</v>
       </c>
       <c r="D390" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="E390" t="s">
         <v>710</v>
@@ -37672,7 +37697,7 @@
         <v>150</v>
       </c>
       <c r="D391" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E391" t="s">
         <v>710</v>
@@ -37689,10 +37714,10 @@
         <v>150</v>
       </c>
       <c r="D392" t="s">
-        <v>239</v>
+        <v>444</v>
       </c>
       <c r="E392" t="s">
-        <v>735</v>
+        <v>710</v>
       </c>
       <c r="F392" t="s">
         <v>643</v>
@@ -37706,10 +37731,10 @@
         <v>150</v>
       </c>
       <c r="D393" t="s">
-        <v>141</v>
+        <v>446</v>
       </c>
       <c r="E393" t="s">
-        <v>735</v>
+        <v>710</v>
       </c>
       <c r="F393" t="s">
         <v>643</v>
@@ -37723,7 +37748,7 @@
         <v>150</v>
       </c>
       <c r="D394" t="s">
-        <v>436</v>
+        <v>239</v>
       </c>
       <c r="E394" t="s">
         <v>735</v>
@@ -37740,7 +37765,7 @@
         <v>150</v>
       </c>
       <c r="D395" t="s">
-        <v>438</v>
+        <v>141</v>
       </c>
       <c r="E395" t="s">
         <v>735</v>
@@ -37757,7 +37782,7 @@
         <v>150</v>
       </c>
       <c r="D396" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="E396" t="s">
         <v>735</v>
@@ -37774,7 +37799,7 @@
         <v>150</v>
       </c>
       <c r="D397" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="E397" t="s">
         <v>735</v>
@@ -37791,7 +37816,7 @@
         <v>150</v>
       </c>
       <c r="D398" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="E398" t="s">
         <v>735</v>
@@ -37808,7 +37833,7 @@
         <v>150</v>
       </c>
       <c r="D399" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E399" t="s">
         <v>735</v>
@@ -37825,10 +37850,10 @@
         <v>150</v>
       </c>
       <c r="D400" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="E400" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="F400" t="s">
         <v>643</v>
@@ -37842,10 +37867,10 @@
         <v>150</v>
       </c>
       <c r="D401" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="E401" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="F401" t="s">
         <v>643</v>
@@ -37859,7 +37884,7 @@
         <v>150</v>
       </c>
       <c r="D402" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="E402" t="s">
         <v>736</v>
@@ -37876,7 +37901,7 @@
         <v>150</v>
       </c>
       <c r="D403" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E403" t="s">
         <v>736</v>
@@ -37893,10 +37918,10 @@
         <v>150</v>
       </c>
       <c r="D404" t="s">
-        <v>239</v>
+        <v>444</v>
       </c>
       <c r="E404" t="s">
-        <v>644</v>
+        <v>736</v>
       </c>
       <c r="F404" t="s">
         <v>643</v>
@@ -37910,10 +37935,10 @@
         <v>150</v>
       </c>
       <c r="D405" t="s">
-        <v>141</v>
+        <v>446</v>
       </c>
       <c r="E405" t="s">
-        <v>644</v>
+        <v>736</v>
       </c>
       <c r="F405" t="s">
         <v>643</v>
@@ -37927,7 +37952,7 @@
         <v>150</v>
       </c>
       <c r="D406" t="s">
-        <v>436</v>
+        <v>239</v>
       </c>
       <c r="E406" t="s">
         <v>644</v>
@@ -37944,7 +37969,7 @@
         <v>150</v>
       </c>
       <c r="D407" t="s">
-        <v>438</v>
+        <v>141</v>
       </c>
       <c r="E407" t="s">
         <v>644</v>
@@ -37961,7 +37986,7 @@
         <v>150</v>
       </c>
       <c r="D408" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="E408" t="s">
         <v>644</v>
@@ -37978,7 +38003,7 @@
         <v>150</v>
       </c>
       <c r="D409" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="E409" t="s">
         <v>644</v>
@@ -37995,7 +38020,7 @@
         <v>150</v>
       </c>
       <c r="D410" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="E410" t="s">
         <v>644</v>
@@ -38012,7 +38037,7 @@
         <v>150</v>
       </c>
       <c r="D411" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E411" t="s">
         <v>644</v>
@@ -38026,13 +38051,13 @@
         <v>42736</v>
       </c>
       <c r="C412" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D412" t="s">
-        <v>239</v>
+        <v>444</v>
       </c>
       <c r="E412" t="s">
-        <v>710</v>
+        <v>644</v>
       </c>
       <c r="F412" t="s">
         <v>643</v>
@@ -38043,13 +38068,13 @@
         <v>42736</v>
       </c>
       <c r="C413" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D413" t="s">
-        <v>141</v>
+        <v>446</v>
       </c>
       <c r="E413" t="s">
-        <v>710</v>
+        <v>644</v>
       </c>
       <c r="F413" t="s">
         <v>643</v>
@@ -38063,7 +38088,7 @@
         <v>151</v>
       </c>
       <c r="D414" t="s">
-        <v>436</v>
+        <v>239</v>
       </c>
       <c r="E414" t="s">
         <v>710</v>
@@ -38080,7 +38105,7 @@
         <v>151</v>
       </c>
       <c r="D415" t="s">
-        <v>438</v>
+        <v>141</v>
       </c>
       <c r="E415" t="s">
         <v>710</v>
@@ -38097,7 +38122,7 @@
         <v>151</v>
       </c>
       <c r="D416" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="E416" t="s">
         <v>710</v>
@@ -38114,7 +38139,7 @@
         <v>151</v>
       </c>
       <c r="D417" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="E417" t="s">
         <v>710</v>
@@ -38131,7 +38156,7 @@
         <v>151</v>
       </c>
       <c r="D418" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="E418" t="s">
         <v>710</v>
@@ -38148,7 +38173,7 @@
         <v>151</v>
       </c>
       <c r="D419" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E419" t="s">
         <v>710</v>
@@ -38165,10 +38190,10 @@
         <v>151</v>
       </c>
       <c r="D420" t="s">
-        <v>239</v>
+        <v>444</v>
       </c>
       <c r="E420" t="s">
-        <v>735</v>
+        <v>710</v>
       </c>
       <c r="F420" t="s">
         <v>643</v>
@@ -38182,10 +38207,10 @@
         <v>151</v>
       </c>
       <c r="D421" t="s">
-        <v>141</v>
+        <v>446</v>
       </c>
       <c r="E421" t="s">
-        <v>735</v>
+        <v>710</v>
       </c>
       <c r="F421" t="s">
         <v>643</v>
@@ -38199,7 +38224,7 @@
         <v>151</v>
       </c>
       <c r="D422" t="s">
-        <v>436</v>
+        <v>239</v>
       </c>
       <c r="E422" t="s">
         <v>735</v>
@@ -38216,7 +38241,7 @@
         <v>151</v>
       </c>
       <c r="D423" t="s">
-        <v>438</v>
+        <v>141</v>
       </c>
       <c r="E423" t="s">
         <v>735</v>
@@ -38233,7 +38258,7 @@
         <v>151</v>
       </c>
       <c r="D424" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="E424" t="s">
         <v>735</v>
@@ -38250,7 +38275,7 @@
         <v>151</v>
       </c>
       <c r="D425" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="E425" t="s">
         <v>735</v>
@@ -38267,7 +38292,7 @@
         <v>151</v>
       </c>
       <c r="D426" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="E426" t="s">
         <v>735</v>
@@ -38284,7 +38309,7 @@
         <v>151</v>
       </c>
       <c r="D427" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E427" t="s">
         <v>735</v>
@@ -38301,10 +38326,10 @@
         <v>151</v>
       </c>
       <c r="D428" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="E428" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="F428" t="s">
         <v>643</v>
@@ -38318,10 +38343,10 @@
         <v>151</v>
       </c>
       <c r="D429" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="E429" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="F429" t="s">
         <v>643</v>
@@ -38335,7 +38360,7 @@
         <v>151</v>
       </c>
       <c r="D430" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="E430" t="s">
         <v>736</v>
@@ -38352,7 +38377,7 @@
         <v>151</v>
       </c>
       <c r="D431" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E431" t="s">
         <v>736</v>
@@ -38369,10 +38394,10 @@
         <v>151</v>
       </c>
       <c r="D432" t="s">
-        <v>239</v>
+        <v>444</v>
       </c>
       <c r="E432" t="s">
-        <v>644</v>
+        <v>736</v>
       </c>
       <c r="F432" t="s">
         <v>643</v>
@@ -38386,10 +38411,10 @@
         <v>151</v>
       </c>
       <c r="D433" t="s">
-        <v>141</v>
+        <v>446</v>
       </c>
       <c r="E433" t="s">
-        <v>644</v>
+        <v>736</v>
       </c>
       <c r="F433" t="s">
         <v>643</v>
@@ -38403,7 +38428,7 @@
         <v>151</v>
       </c>
       <c r="D434" t="s">
-        <v>436</v>
+        <v>239</v>
       </c>
       <c r="E434" t="s">
         <v>644</v>
@@ -38420,7 +38445,7 @@
         <v>151</v>
       </c>
       <c r="D435" t="s">
-        <v>438</v>
+        <v>141</v>
       </c>
       <c r="E435" t="s">
         <v>644</v>
@@ -38437,7 +38462,7 @@
         <v>151</v>
       </c>
       <c r="D436" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="E436" t="s">
         <v>644</v>
@@ -38454,7 +38479,7 @@
         <v>151</v>
       </c>
       <c r="D437" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="E437" t="s">
         <v>644</v>
@@ -38471,7 +38496,7 @@
         <v>151</v>
       </c>
       <c r="D438" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="E438" t="s">
         <v>644</v>
@@ -38488,7 +38513,7 @@
         <v>151</v>
       </c>
       <c r="D439" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="E439" t="s">
         <v>644</v>
@@ -38502,10 +38527,10 @@
         <v>42736</v>
       </c>
       <c r="C440" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D440" t="s">
-        <v>47</v>
+        <v>444</v>
       </c>
       <c r="E440" t="s">
         <v>644</v>
@@ -38519,13 +38544,13 @@
         <v>42736</v>
       </c>
       <c r="C441" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D441" t="s">
-        <v>47</v>
+        <v>446</v>
       </c>
       <c r="E441" t="s">
-        <v>735</v>
+        <v>644</v>
       </c>
       <c r="F441" t="s">
         <v>643</v>
@@ -38536,7 +38561,7 @@
         <v>42736</v>
       </c>
       <c r="C442" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D442" t="s">
         <v>47</v>
@@ -38553,13 +38578,13 @@
         <v>42736</v>
       </c>
       <c r="C443" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D443" t="s">
-        <v>239</v>
+        <v>47</v>
       </c>
       <c r="E443" t="s">
-        <v>644</v>
+        <v>735</v>
       </c>
       <c r="F443" t="s">
         <v>643</v>
@@ -38570,10 +38595,10 @@
         <v>42736</v>
       </c>
       <c r="C444" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D444" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E444" t="s">
         <v>644</v>
@@ -38590,10 +38615,10 @@
         <v>154</v>
       </c>
       <c r="D445" t="s">
-        <v>51</v>
+        <v>239</v>
       </c>
       <c r="E445" t="s">
-        <v>718</v>
+        <v>644</v>
       </c>
       <c r="F445" t="s">
         <v>643</v>
@@ -38604,10 +38629,10 @@
         <v>42736</v>
       </c>
       <c r="C446" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D446" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E446" t="s">
         <v>644</v>
@@ -38621,13 +38646,13 @@
         <v>42736</v>
       </c>
       <c r="C447" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D447" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E447" t="s">
-        <v>644</v>
+        <v>718</v>
       </c>
       <c r="F447" t="s">
         <v>643</v>
@@ -38638,10 +38663,10 @@
         <v>42736</v>
       </c>
       <c r="C448" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D448" t="s">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="E448" t="s">
         <v>644</v>
@@ -38655,13 +38680,13 @@
         <v>42736</v>
       </c>
       <c r="C449" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D449" t="s">
-        <v>450</v>
+        <v>47</v>
       </c>
       <c r="E449" t="s">
-        <v>665</v>
+        <v>644</v>
       </c>
       <c r="F449" t="s">
         <v>643</v>
@@ -38672,16 +38697,16 @@
         <v>42736</v>
       </c>
       <c r="C450" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D450" t="s">
-        <v>450</v>
+        <v>13</v>
       </c>
       <c r="E450" t="s">
-        <v>667</v>
+        <v>644</v>
       </c>
       <c r="F450" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
     </row>
     <row r="451" spans="1:6" x14ac:dyDescent="0.2">
@@ -38692,10 +38717,10 @@
         <v>157</v>
       </c>
       <c r="D451" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="E451" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="F451" t="s">
         <v>643</v>
@@ -38709,13 +38734,13 @@
         <v>157</v>
       </c>
       <c r="D452" t="s">
-        <v>158</v>
+        <v>450</v>
       </c>
       <c r="E452" t="s">
         <v>667</v>
       </c>
       <c r="F452" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
     </row>
     <row r="453" spans="1:6" x14ac:dyDescent="0.2">
@@ -38729,7 +38754,7 @@
         <v>447</v>
       </c>
       <c r="E453" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="F453" t="s">
         <v>643</v>
@@ -38746,7 +38771,7 @@
         <v>158</v>
       </c>
       <c r="E454" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="F454" t="s">
         <v>643</v>
@@ -38757,13 +38782,13 @@
         <v>42736</v>
       </c>
       <c r="C455" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D455" t="s">
-        <v>47</v>
+        <v>447</v>
       </c>
       <c r="E455" t="s">
-        <v>710</v>
+        <v>665</v>
       </c>
       <c r="F455" t="s">
         <v>643</v>
@@ -38774,16 +38799,16 @@
         <v>42736</v>
       </c>
       <c r="C456" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D456" t="s">
-        <v>47</v>
+        <v>158</v>
       </c>
       <c r="E456" t="s">
-        <v>714</v>
+        <v>665</v>
       </c>
       <c r="F456" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
     </row>
     <row r="457" spans="1:6" x14ac:dyDescent="0.2">
@@ -38791,7 +38816,7 @@
         <v>42736</v>
       </c>
       <c r="C457" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D457" t="s">
         <v>47</v>
@@ -38808,7 +38833,7 @@
         <v>42736</v>
       </c>
       <c r="C458" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D458" t="s">
         <v>47</v>
@@ -38825,13 +38850,13 @@
         <v>42736</v>
       </c>
       <c r="C459" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D459" t="s">
-        <v>239</v>
+        <v>47</v>
       </c>
       <c r="E459" t="s">
-        <v>644</v>
+        <v>710</v>
       </c>
       <c r="F459" t="s">
         <v>643</v>
@@ -38842,16 +38867,16 @@
         <v>42736</v>
       </c>
       <c r="C460" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D460" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E460" t="s">
-        <v>644</v>
+        <v>714</v>
       </c>
       <c r="F460" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
     </row>
     <row r="461" spans="1:6" x14ac:dyDescent="0.2">
@@ -38862,10 +38887,10 @@
         <v>161</v>
       </c>
       <c r="D461" t="s">
-        <v>51</v>
+        <v>239</v>
       </c>
       <c r="E461" t="s">
-        <v>718</v>
+        <v>644</v>
       </c>
       <c r="F461" t="s">
         <v>643</v>
@@ -38873,13 +38898,13 @@
     </row>
     <row r="462" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A462" s="1">
-        <v>42741</v>
+        <v>42736</v>
       </c>
       <c r="C462" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D462" t="s">
-        <v>163</v>
+        <v>51</v>
       </c>
       <c r="E462" t="s">
         <v>644</v>
@@ -38890,16 +38915,16 @@
     </row>
     <row r="463" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A463" s="1">
-        <v>42742</v>
+        <v>42736</v>
       </c>
       <c r="C463" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D463" t="s">
-        <v>165</v>
+        <v>51</v>
       </c>
       <c r="E463" t="s">
-        <v>644</v>
+        <v>718</v>
       </c>
       <c r="F463" t="s">
         <v>643</v>
@@ -38907,13 +38932,13 @@
     </row>
     <row r="464" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A464" s="1">
-        <v>42743</v>
+        <v>42741</v>
       </c>
       <c r="C464" t="s">
         <v>162</v>
       </c>
       <c r="D464" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="E464" t="s">
         <v>644</v>
@@ -38924,13 +38949,13 @@
     </row>
     <row r="465" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A465" s="1">
-        <v>42744</v>
+        <v>42742</v>
       </c>
       <c r="C465" t="s">
         <v>162</v>
       </c>
       <c r="D465" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E465" t="s">
         <v>644</v>
@@ -38941,13 +38966,13 @@
     </row>
     <row r="466" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A466" s="1">
-        <v>42745</v>
+        <v>42743</v>
       </c>
       <c r="C466" t="s">
         <v>162</v>
       </c>
       <c r="D466" t="s">
-        <v>456</v>
+        <v>167</v>
       </c>
       <c r="E466" t="s">
         <v>644</v>
@@ -38958,13 +38983,13 @@
     </row>
     <row r="467" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A467" s="1">
-        <v>42741</v>
+        <v>42744</v>
       </c>
       <c r="C467" t="s">
         <v>162</v>
       </c>
       <c r="D467" t="s">
-        <v>458</v>
+        <v>169</v>
       </c>
       <c r="E467" t="s">
         <v>644</v>
@@ -38975,13 +39000,13 @@
     </row>
     <row r="468" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A468" s="1">
-        <v>42742</v>
+        <v>42745</v>
       </c>
       <c r="C468" t="s">
         <v>162</v>
       </c>
       <c r="D468" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="E468" t="s">
         <v>644</v>
@@ -38992,13 +39017,13 @@
     </row>
     <row r="469" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A469" s="1">
-        <v>42743</v>
+        <v>42741</v>
       </c>
       <c r="C469" t="s">
         <v>162</v>
       </c>
       <c r="D469" t="s">
-        <v>463</v>
+        <v>458</v>
       </c>
       <c r="E469" t="s">
         <v>644</v>
@@ -39009,47 +39034,47 @@
     </row>
     <row r="470" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A470" s="1">
-        <v>42746</v>
+        <v>42742</v>
       </c>
       <c r="C470" t="s">
         <v>162</v>
       </c>
       <c r="D470" t="s">
-        <v>163</v>
+        <v>460</v>
       </c>
       <c r="E470" t="s">
-        <v>727</v>
+        <v>644</v>
       </c>
       <c r="F470" t="s">
-        <v>716</v>
+        <v>643</v>
       </c>
     </row>
     <row r="471" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A471" s="1">
-        <v>42747</v>
+        <v>42743</v>
       </c>
       <c r="C471" t="s">
         <v>162</v>
       </c>
       <c r="D471" t="s">
-        <v>165</v>
+        <v>463</v>
       </c>
       <c r="E471" t="s">
-        <v>727</v>
+        <v>644</v>
       </c>
       <c r="F471" t="s">
-        <v>663</v>
+        <v>643</v>
       </c>
     </row>
     <row r="472" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A472" s="1">
-        <v>42748</v>
+        <v>42746</v>
       </c>
       <c r="C472" t="s">
         <v>162</v>
       </c>
       <c r="D472" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="E472" t="s">
         <v>727</v>
@@ -39060,30 +39085,30 @@
     </row>
     <row r="473" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A473" s="1">
-        <v>42749</v>
+        <v>42747</v>
       </c>
       <c r="C473" t="s">
         <v>162</v>
       </c>
       <c r="D473" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E473" t="s">
         <v>727</v>
       </c>
       <c r="F473" t="s">
-        <v>716</v>
+        <v>663</v>
       </c>
     </row>
     <row r="474" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A474" s="1">
-        <v>42750</v>
+        <v>42748</v>
       </c>
       <c r="C474" t="s">
         <v>162</v>
       </c>
       <c r="D474" t="s">
-        <v>456</v>
+        <v>167</v>
       </c>
       <c r="E474" t="s">
         <v>727</v>
@@ -39094,13 +39119,13 @@
     </row>
     <row r="475" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A475" s="1">
-        <v>42741</v>
+        <v>42749</v>
       </c>
       <c r="C475" t="s">
         <v>162</v>
       </c>
       <c r="D475" t="s">
-        <v>458</v>
+        <v>169</v>
       </c>
       <c r="E475" t="s">
         <v>727</v>
@@ -39111,13 +39136,13 @@
     </row>
     <row r="476" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A476" s="1">
-        <v>42742</v>
+        <v>42750</v>
       </c>
       <c r="C476" t="s">
         <v>162</v>
       </c>
       <c r="D476" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="E476" t="s">
         <v>727</v>
@@ -39128,18 +39153,52 @@
     </row>
     <row r="477" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A477" s="1">
-        <v>42743</v>
+        <v>42741</v>
       </c>
       <c r="C477" t="s">
         <v>162</v>
       </c>
       <c r="D477" t="s">
-        <v>463</v>
+        <v>458</v>
       </c>
       <c r="E477" t="s">
         <v>727</v>
       </c>
       <c r="F477" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="478" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A478" s="1">
+        <v>42742</v>
+      </c>
+      <c r="C478" t="s">
+        <v>162</v>
+      </c>
+      <c r="D478" t="s">
+        <v>460</v>
+      </c>
+      <c r="E478" t="s">
+        <v>727</v>
+      </c>
+      <c r="F478" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="479" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A479" s="1">
+        <v>42743</v>
+      </c>
+      <c r="C479" t="s">
+        <v>162</v>
+      </c>
+      <c r="D479" t="s">
+        <v>463</v>
+      </c>
+      <c r="E479" t="s">
+        <v>727</v>
+      </c>
+      <c r="F479" t="s">
         <v>716</v>
       </c>
     </row>
@@ -39150,10 +39209,14 @@
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
-  <dimension ref="A1:V361"/>
+  <dimension ref="A1:V363"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="26.1640625" customWidth="1"/>
+    <col min="5" max="5" width="26.6640625" customWidth="1"/>
+    <col min="8" max="8" width="15.5" customWidth="1"/>
+    <col min="9" max="9" width="23.33203125" customWidth="1"/>
+    <col min="15" max="15" width="19.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.2">
@@ -49206,68 +49269,74 @@
         <v>700</v>
       </c>
     </row>
-    <row r="311" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:16" ht="18" x14ac:dyDescent="0.25">
       <c r="A311" s="1">
-        <v>42736</v>
+        <v>42746</v>
       </c>
       <c r="C311" t="s">
-        <v>138</v>
+        <v>114</v>
       </c>
       <c r="D311" t="s">
         <v>748</v>
       </c>
       <c r="E311" t="s">
-        <v>47</v>
+        <v>1537</v>
       </c>
       <c r="F311">
         <v>1</v>
       </c>
       <c r="G311" t="s">
-        <v>1252</v>
+        <v>1178</v>
       </c>
       <c r="H311" t="s">
         <v>1253</v>
       </c>
       <c r="I311" t="s">
-        <v>1314</v>
+        <v>1538</v>
       </c>
       <c r="J311">
         <v>1</v>
       </c>
+      <c r="O311" s="3" t="s">
+        <v>1539</v>
+      </c>
       <c r="P311" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="312" spans="1:16" x14ac:dyDescent="0.2">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="312" spans="1:16" ht="18" x14ac:dyDescent="0.25">
       <c r="A312" s="1">
-        <v>42736</v>
+        <v>42746</v>
       </c>
       <c r="C312" t="s">
-        <v>139</v>
+        <v>114</v>
       </c>
       <c r="D312" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="E312" t="s">
-        <v>47</v>
+        <v>1537</v>
       </c>
       <c r="F312">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G312" t="s">
-        <v>1252</v>
+        <v>1178</v>
       </c>
       <c r="H312" t="s">
         <v>1253</v>
       </c>
       <c r="I312" t="s">
-        <v>1314</v>
+        <v>1538</v>
       </c>
       <c r="J312">
         <v>1</v>
       </c>
+      <c r="O312" s="3" t="s">
+        <v>1539</v>
+      </c>
       <c r="P312" t="s">
-        <v>405</v>
+        <v>700</v>
       </c>
     </row>
     <row r="313" spans="1:16" x14ac:dyDescent="0.2">
@@ -49275,10 +49344,10 @@
         <v>42736</v>
       </c>
       <c r="C313" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D313" t="s">
-        <v>782</v>
+        <v>748</v>
       </c>
       <c r="E313" t="s">
         <v>47</v>
@@ -49307,25 +49376,25 @@
         <v>42736</v>
       </c>
       <c r="C314" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D314" t="s">
         <v>748</v>
       </c>
       <c r="E314" t="s">
-        <v>141</v>
+        <v>47</v>
       </c>
       <c r="F314">
         <v>1</v>
       </c>
       <c r="G314" t="s">
-        <v>1178</v>
+        <v>1252</v>
       </c>
       <c r="H314" t="s">
         <v>1253</v>
       </c>
       <c r="I314" t="s">
-        <v>1254</v>
+        <v>1314</v>
       </c>
       <c r="J314">
         <v>1</v>
@@ -49339,25 +49408,25 @@
         <v>42736</v>
       </c>
       <c r="C315" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D315" t="s">
-        <v>748</v>
+        <v>782</v>
       </c>
       <c r="E315" t="s">
-        <v>436</v>
+        <v>47</v>
       </c>
       <c r="F315">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G315" t="s">
-        <v>1178</v>
+        <v>1252</v>
       </c>
       <c r="H315" t="s">
         <v>1253</v>
       </c>
       <c r="I315" t="s">
-        <v>1254</v>
+        <v>1314</v>
       </c>
       <c r="J315">
         <v>1</v>
@@ -49377,10 +49446,10 @@
         <v>748</v>
       </c>
       <c r="E316" t="s">
-        <v>438</v>
+        <v>141</v>
       </c>
       <c r="F316">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G316" t="s">
         <v>1178</v>
@@ -49403,16 +49472,16 @@
         <v>42736</v>
       </c>
       <c r="C317" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="D317" t="s">
-        <v>740</v>
+        <v>748</v>
       </c>
       <c r="E317" t="s">
-        <v>51</v>
+        <v>436</v>
       </c>
       <c r="F317">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G317" t="s">
         <v>1178</v>
@@ -49435,16 +49504,16 @@
         <v>42736</v>
       </c>
       <c r="C318" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="D318" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="E318" t="s">
-        <v>51</v>
+        <v>438</v>
       </c>
       <c r="F318">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G318" t="s">
         <v>1178</v>
@@ -49467,13 +49536,13 @@
         <v>42736</v>
       </c>
       <c r="C319" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D319" t="s">
-        <v>748</v>
+        <v>740</v>
       </c>
       <c r="E319" t="s">
-        <v>141</v>
+        <v>51</v>
       </c>
       <c r="F319">
         <v>1</v>
@@ -49499,16 +49568,16 @@
         <v>42736</v>
       </c>
       <c r="C320" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D320" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
       <c r="E320" t="s">
-        <v>436</v>
+        <v>51</v>
       </c>
       <c r="F320">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G320" t="s">
         <v>1178</v>
@@ -49537,10 +49606,10 @@
         <v>748</v>
       </c>
       <c r="E321" t="s">
-        <v>438</v>
+        <v>141</v>
       </c>
       <c r="F321">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G321" t="s">
         <v>1178</v>
@@ -49560,25 +49629,25 @@
     </row>
     <row r="322" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A322" s="1">
-        <v>42756</v>
+        <v>42736</v>
       </c>
       <c r="C322" t="s">
         <v>150</v>
       </c>
       <c r="D322" t="s">
-        <v>827</v>
+        <v>748</v>
       </c>
       <c r="E322" t="s">
-        <v>442</v>
+        <v>436</v>
       </c>
       <c r="F322">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G322" t="s">
-        <v>1258</v>
+        <v>1178</v>
       </c>
       <c r="H322" t="s">
-        <v>1322</v>
+        <v>1253</v>
       </c>
       <c r="I322" t="s">
         <v>1254</v>
@@ -49592,25 +49661,25 @@
     </row>
     <row r="323" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A323" s="1">
-        <v>42756</v>
+        <v>42736</v>
       </c>
       <c r="C323" t="s">
         <v>150</v>
       </c>
       <c r="D323" t="s">
-        <v>827</v>
+        <v>748</v>
       </c>
       <c r="E323" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="F323">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G323" t="s">
-        <v>1258</v>
+        <v>1178</v>
       </c>
       <c r="H323" t="s">
-        <v>1322</v>
+        <v>1253</v>
       </c>
       <c r="I323" t="s">
         <v>1254</v>
@@ -49633,10 +49702,10 @@
         <v>827</v>
       </c>
       <c r="E324" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="F324">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G324" t="s">
         <v>1258</v>
@@ -49656,28 +49725,28 @@
     </row>
     <row r="325" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A325" s="1">
-        <v>42736</v>
+        <v>42756</v>
       </c>
       <c r="C325" t="s">
         <v>150</v>
       </c>
       <c r="D325" t="s">
-        <v>825</v>
+        <v>827</v>
       </c>
       <c r="E325" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
       <c r="F325">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G325" t="s">
         <v>1258</v>
       </c>
       <c r="H325" t="s">
-        <v>1272</v>
+        <v>1322</v>
       </c>
       <c r="I325" t="s">
-        <v>293</v>
+        <v>1254</v>
       </c>
       <c r="J325">
         <v>1</v>
@@ -49688,28 +49757,28 @@
     </row>
     <row r="326" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A326" s="1">
-        <v>42736</v>
+        <v>42756</v>
       </c>
       <c r="C326" t="s">
         <v>150</v>
       </c>
       <c r="D326" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="E326" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="F326">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G326" t="s">
         <v>1258</v>
       </c>
       <c r="H326" t="s">
-        <v>1272</v>
+        <v>1322</v>
       </c>
       <c r="I326" t="s">
-        <v>293</v>
+        <v>1254</v>
       </c>
       <c r="J326">
         <v>1</v>
@@ -49726,13 +49795,13 @@
         <v>150</v>
       </c>
       <c r="D327" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="E327" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="F327">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G327" t="s">
         <v>1258</v>
@@ -49761,10 +49830,10 @@
         <v>826</v>
       </c>
       <c r="E328" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="F328">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G328" t="s">
         <v>1258</v>
@@ -49793,10 +49862,10 @@
         <v>826</v>
       </c>
       <c r="E329" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="F329">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G329" t="s">
         <v>1258</v>
@@ -49819,25 +49888,25 @@
         <v>42736</v>
       </c>
       <c r="C330" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D330" t="s">
-        <v>748</v>
+        <v>826</v>
       </c>
       <c r="E330" t="s">
-        <v>141</v>
+        <v>444</v>
       </c>
       <c r="F330">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G330" t="s">
-        <v>1178</v>
+        <v>1258</v>
       </c>
       <c r="H330" t="s">
-        <v>1253</v>
+        <v>1272</v>
       </c>
       <c r="I330" t="s">
-        <v>1254</v>
+        <v>293</v>
       </c>
       <c r="J330">
         <v>1</v>
@@ -49851,25 +49920,25 @@
         <v>42736</v>
       </c>
       <c r="C331" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D331" t="s">
-        <v>748</v>
+        <v>826</v>
       </c>
       <c r="E331" t="s">
-        <v>436</v>
+        <v>446</v>
       </c>
       <c r="F331">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G331" t="s">
-        <v>1178</v>
+        <v>1258</v>
       </c>
       <c r="H331" t="s">
-        <v>1253</v>
+        <v>1272</v>
       </c>
       <c r="I331" t="s">
-        <v>1254</v>
+        <v>293</v>
       </c>
       <c r="J331">
         <v>1</v>
@@ -49889,10 +49958,10 @@
         <v>748</v>
       </c>
       <c r="E332" t="s">
-        <v>438</v>
+        <v>141</v>
       </c>
       <c r="F332">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G332" t="s">
         <v>1178</v>
@@ -49918,22 +49987,22 @@
         <v>151</v>
       </c>
       <c r="D333" t="s">
-        <v>828</v>
+        <v>748</v>
       </c>
       <c r="E333" t="s">
-        <v>446</v>
+        <v>436</v>
       </c>
       <c r="F333">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G333" t="s">
-        <v>1258</v>
+        <v>1178</v>
       </c>
       <c r="H333" t="s">
-        <v>1272</v>
+        <v>1253</v>
       </c>
       <c r="I333" t="s">
-        <v>293</v>
+        <v>1254</v>
       </c>
       <c r="J333">
         <v>1</v>
@@ -49950,22 +50019,22 @@
         <v>151</v>
       </c>
       <c r="D334" t="s">
-        <v>826</v>
+        <v>748</v>
       </c>
       <c r="E334" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="F334">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G334" t="s">
-        <v>1258</v>
+        <v>1178</v>
       </c>
       <c r="H334" t="s">
-        <v>1272</v>
+        <v>1253</v>
       </c>
       <c r="I334" t="s">
-        <v>293</v>
+        <v>1254</v>
       </c>
       <c r="J334">
         <v>1</v>
@@ -49982,13 +50051,13 @@
         <v>151</v>
       </c>
       <c r="D335" t="s">
-        <v>826</v>
+        <v>828</v>
       </c>
       <c r="E335" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="F335">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G335" t="s">
         <v>1258</v>
@@ -50017,10 +50086,10 @@
         <v>826</v>
       </c>
       <c r="E336" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="F336">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G336" t="s">
         <v>1258</v>
@@ -50049,10 +50118,10 @@
         <v>826</v>
       </c>
       <c r="E337" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="F337">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G337" t="s">
         <v>1258</v>
@@ -50075,25 +50144,25 @@
         <v>42736</v>
       </c>
       <c r="C338" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D338" t="s">
-        <v>748</v>
+        <v>826</v>
       </c>
       <c r="E338" t="s">
-        <v>47</v>
+        <v>444</v>
       </c>
       <c r="F338">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G338" t="s">
-        <v>1252</v>
+        <v>1258</v>
       </c>
       <c r="H338" t="s">
-        <v>1253</v>
+        <v>1272</v>
       </c>
       <c r="I338" t="s">
-        <v>1314</v>
+        <v>293</v>
       </c>
       <c r="J338">
         <v>1</v>
@@ -50107,25 +50176,25 @@
         <v>42736</v>
       </c>
       <c r="C339" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D339" t="s">
-        <v>748</v>
+        <v>826</v>
       </c>
       <c r="E339" t="s">
-        <v>47</v>
+        <v>446</v>
       </c>
       <c r="F339">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G339" t="s">
-        <v>1252</v>
+        <v>1258</v>
       </c>
       <c r="H339" t="s">
-        <v>1253</v>
+        <v>1272</v>
       </c>
       <c r="I339" t="s">
-        <v>1314</v>
+        <v>293</v>
       </c>
       <c r="J339">
         <v>1</v>
@@ -50139,25 +50208,25 @@
         <v>42736</v>
       </c>
       <c r="C340" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D340" t="s">
-        <v>740</v>
+        <v>748</v>
       </c>
       <c r="E340" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F340">
         <v>1</v>
       </c>
       <c r="G340" t="s">
-        <v>1178</v>
+        <v>1252</v>
       </c>
       <c r="H340" t="s">
         <v>1253</v>
       </c>
       <c r="I340" t="s">
-        <v>1254</v>
+        <v>1314</v>
       </c>
       <c r="J340">
         <v>1</v>
@@ -50171,25 +50240,25 @@
         <v>42736</v>
       </c>
       <c r="C341" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D341" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="E341" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F341">
         <v>1</v>
       </c>
       <c r="G341" t="s">
-        <v>1178</v>
+        <v>1252</v>
       </c>
       <c r="H341" t="s">
         <v>1253</v>
       </c>
       <c r="I341" t="s">
-        <v>1254</v>
+        <v>1314</v>
       </c>
       <c r="J341">
         <v>1</v>
@@ -50203,13 +50272,13 @@
         <v>42736</v>
       </c>
       <c r="C342" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D342" t="s">
         <v>740</v>
       </c>
       <c r="E342" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F342">
         <v>1</v>
@@ -50235,13 +50304,13 @@
         <v>42736</v>
       </c>
       <c r="C343" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D343" t="s">
-        <v>829</v>
+        <v>744</v>
       </c>
       <c r="E343" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F343">
         <v>1</v>
@@ -50270,7 +50339,7 @@
         <v>155</v>
       </c>
       <c r="D344" t="s">
-        <v>830</v>
+        <v>740</v>
       </c>
       <c r="E344" t="s">
         <v>47</v>
@@ -50299,10 +50368,10 @@
         <v>42736</v>
       </c>
       <c r="C345" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D345" t="s">
-        <v>748</v>
+        <v>829</v>
       </c>
       <c r="E345" t="s">
         <v>47</v>
@@ -50311,7 +50380,7 @@
         <v>1</v>
       </c>
       <c r="G345" t="s">
-        <v>1252</v>
+        <v>1178</v>
       </c>
       <c r="H345" t="s">
         <v>1253</v>
@@ -50331,19 +50400,19 @@
         <v>42736</v>
       </c>
       <c r="C346" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D346" t="s">
-        <v>748</v>
+        <v>830</v>
       </c>
       <c r="E346" t="s">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="F346">
         <v>1</v>
       </c>
       <c r="G346" t="s">
-        <v>1252</v>
+        <v>1178</v>
       </c>
       <c r="H346" t="s">
         <v>1253</v>
@@ -50363,19 +50432,19 @@
         <v>42736</v>
       </c>
       <c r="C347" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D347" t="s">
         <v>748</v>
       </c>
       <c r="E347" t="s">
-        <v>447</v>
+        <v>47</v>
       </c>
       <c r="F347">
         <v>1</v>
       </c>
       <c r="G347" t="s">
-        <v>1258</v>
+        <v>1252</v>
       </c>
       <c r="H347" t="s">
         <v>1253</v>
@@ -50395,19 +50464,19 @@
         <v>42736</v>
       </c>
       <c r="C348" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D348" t="s">
         <v>748</v>
       </c>
       <c r="E348" t="s">
-        <v>450</v>
+        <v>13</v>
       </c>
       <c r="F348">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G348" t="s">
-        <v>1258</v>
+        <v>1252</v>
       </c>
       <c r="H348" t="s">
         <v>1253</v>
@@ -50416,7 +50485,7 @@
         <v>1254</v>
       </c>
       <c r="J348">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P348" t="s">
         <v>405</v>
@@ -50430,7 +50499,7 @@
         <v>157</v>
       </c>
       <c r="D349" t="s">
-        <v>831</v>
+        <v>748</v>
       </c>
       <c r="E349" t="s">
         <v>447</v>
@@ -50462,7 +50531,7 @@
         <v>157</v>
       </c>
       <c r="D350" t="s">
-        <v>831</v>
+        <v>748</v>
       </c>
       <c r="E350" t="s">
         <v>450</v>
@@ -50494,7 +50563,7 @@
         <v>157</v>
       </c>
       <c r="D351" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="E351" t="s">
         <v>447</v>
@@ -50523,19 +50592,19 @@
         <v>42736</v>
       </c>
       <c r="C352" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="D352" t="s">
-        <v>740</v>
+        <v>831</v>
       </c>
       <c r="E352" t="s">
-        <v>51</v>
+        <v>450</v>
       </c>
       <c r="F352">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G352" t="s">
-        <v>1178</v>
+        <v>1258</v>
       </c>
       <c r="H352" t="s">
         <v>1253</v>
@@ -50544,7 +50613,7 @@
         <v>1254</v>
       </c>
       <c r="J352">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P352" t="s">
         <v>405</v>
@@ -50555,19 +50624,19 @@
         <v>42736</v>
       </c>
       <c r="C353" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="D353" t="s">
-        <v>744</v>
+        <v>832</v>
       </c>
       <c r="E353" t="s">
-        <v>51</v>
+        <v>447</v>
       </c>
       <c r="F353">
         <v>1</v>
       </c>
       <c r="G353" t="s">
-        <v>1178</v>
+        <v>1258</v>
       </c>
       <c r="H353" t="s">
         <v>1253</v>
@@ -50590,7 +50659,7 @@
         <v>161</v>
       </c>
       <c r="D354" t="s">
-        <v>833</v>
+        <v>740</v>
       </c>
       <c r="E354" t="s">
         <v>51</v>
@@ -50616,22 +50685,22 @@
     </row>
     <row r="355" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A355" s="1">
-        <v>42741</v>
+        <v>42736</v>
       </c>
       <c r="C355" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D355" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="E355" t="s">
-        <v>163</v>
+        <v>51</v>
       </c>
       <c r="F355">
         <v>1</v>
       </c>
       <c r="G355" t="s">
-        <v>1252</v>
+        <v>1178</v>
       </c>
       <c r="H355" t="s">
         <v>1253</v>
@@ -50648,22 +50717,22 @@
     </row>
     <row r="356" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A356" s="1">
-        <v>42742</v>
+        <v>42736</v>
       </c>
       <c r="C356" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D356" t="s">
-        <v>740</v>
+        <v>833</v>
       </c>
       <c r="E356" t="s">
-        <v>165</v>
+        <v>51</v>
       </c>
       <c r="F356">
         <v>1</v>
       </c>
       <c r="G356" t="s">
-        <v>1252</v>
+        <v>1178</v>
       </c>
       <c r="H356" t="s">
         <v>1253</v>
@@ -50680,7 +50749,7 @@
     </row>
     <row r="357" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A357" s="1">
-        <v>42743</v>
+        <v>42741</v>
       </c>
       <c r="C357" t="s">
         <v>162</v>
@@ -50689,7 +50758,7 @@
         <v>740</v>
       </c>
       <c r="E357" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="F357">
         <v>1</v>
@@ -50712,7 +50781,7 @@
     </row>
     <row r="358" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A358" s="1">
-        <v>42744</v>
+        <v>42742</v>
       </c>
       <c r="C358" t="s">
         <v>162</v>
@@ -50721,7 +50790,7 @@
         <v>740</v>
       </c>
       <c r="E358" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="F358">
         <v>1</v>
@@ -50744,7 +50813,7 @@
     </row>
     <row r="359" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A359" s="1">
-        <v>42741</v>
+        <v>42743</v>
       </c>
       <c r="C359" t="s">
         <v>162</v>
@@ -50753,7 +50822,7 @@
         <v>740</v>
       </c>
       <c r="E359" t="s">
-        <v>458</v>
+        <v>167</v>
       </c>
       <c r="F359">
         <v>1</v>
@@ -50776,7 +50845,7 @@
     </row>
     <row r="360" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A360" s="1">
-        <v>42742</v>
+        <v>42744</v>
       </c>
       <c r="C360" t="s">
         <v>162</v>
@@ -50785,7 +50854,7 @@
         <v>740</v>
       </c>
       <c r="E360" t="s">
-        <v>460</v>
+        <v>169</v>
       </c>
       <c r="F360">
         <v>1</v>
@@ -50808,7 +50877,7 @@
     </row>
     <row r="361" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A361" s="1">
-        <v>42743</v>
+        <v>42741</v>
       </c>
       <c r="C361" t="s">
         <v>162</v>
@@ -50817,7 +50886,7 @@
         <v>740</v>
       </c>
       <c r="E361" t="s">
-        <v>463</v>
+        <v>458</v>
       </c>
       <c r="F361">
         <v>1</v>
@@ -50835,6 +50904,70 @@
         <v>1</v>
       </c>
       <c r="P361" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="362" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A362" s="1">
+        <v>42742</v>
+      </c>
+      <c r="C362" t="s">
+        <v>162</v>
+      </c>
+      <c r="D362" t="s">
+        <v>740</v>
+      </c>
+      <c r="E362" t="s">
+        <v>460</v>
+      </c>
+      <c r="F362">
+        <v>1</v>
+      </c>
+      <c r="G362" t="s">
+        <v>1252</v>
+      </c>
+      <c r="H362" t="s">
+        <v>1253</v>
+      </c>
+      <c r="I362" t="s">
+        <v>1254</v>
+      </c>
+      <c r="J362">
+        <v>1</v>
+      </c>
+      <c r="P362" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="363" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A363" s="1">
+        <v>42743</v>
+      </c>
+      <c r="C363" t="s">
+        <v>162</v>
+      </c>
+      <c r="D363" t="s">
+        <v>740</v>
+      </c>
+      <c r="E363" t="s">
+        <v>463</v>
+      </c>
+      <c r="F363">
+        <v>1</v>
+      </c>
+      <c r="G363" t="s">
+        <v>1252</v>
+      </c>
+      <c r="H363" t="s">
+        <v>1253</v>
+      </c>
+      <c r="I363" t="s">
+        <v>1254</v>
+      </c>
+      <c r="J363">
+        <v>1</v>
+      </c>
+      <c r="P363" t="s">
         <v>405</v>
       </c>
     </row>
@@ -56503,8 +56636,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Q310"/>
+  <dimension ref="A1:Q311"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="29.5" customWidth="1"/>
+    <col min="4" max="4" width="29.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -62616,13 +62753,13 @@
         <v>42736</v>
       </c>
       <c r="C260" t="s">
-        <v>138</v>
+        <v>114</v>
       </c>
       <c r="D260" t="s">
-        <v>47</v>
+        <v>1537</v>
       </c>
       <c r="E260" t="s">
-        <v>47</v>
+        <v>1537</v>
       </c>
       <c r="G260" t="s">
         <v>224</v>
@@ -62639,7 +62776,7 @@
         <v>42736</v>
       </c>
       <c r="C261" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D261" t="s">
         <v>47</v>
@@ -62662,16 +62799,16 @@
         <v>42736</v>
       </c>
       <c r="C262" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D262" t="s">
-        <v>239</v>
+        <v>47</v>
       </c>
       <c r="E262" t="s">
-        <v>240</v>
+        <v>47</v>
       </c>
       <c r="G262" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="K262" t="s">
         <v>218</v>
@@ -62688,13 +62825,13 @@
         <v>140</v>
       </c>
       <c r="D263" t="s">
-        <v>141</v>
+        <v>239</v>
       </c>
       <c r="E263" t="s">
-        <v>434</v>
+        <v>240</v>
       </c>
       <c r="G263" t="s">
-        <v>435</v>
+        <v>214</v>
       </c>
       <c r="K263" t="s">
         <v>218</v>
@@ -62711,10 +62848,10 @@
         <v>140</v>
       </c>
       <c r="D264" t="s">
-        <v>436</v>
+        <v>141</v>
       </c>
       <c r="E264" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="G264" t="s">
         <v>435</v>
@@ -62734,10 +62871,10 @@
         <v>140</v>
       </c>
       <c r="D265" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E265" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="G265" t="s">
         <v>435</v>
@@ -62757,13 +62894,13 @@
         <v>140</v>
       </c>
       <c r="D266" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E266" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="G266" t="s">
-        <v>291</v>
+        <v>435</v>
       </c>
       <c r="K266" t="s">
         <v>218</v>
@@ -62780,10 +62917,10 @@
         <v>140</v>
       </c>
       <c r="D267" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E267" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="G267" t="s">
         <v>291</v>
@@ -62803,10 +62940,10 @@
         <v>140</v>
       </c>
       <c r="D268" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E268" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="G268" t="s">
         <v>291</v>
@@ -62826,13 +62963,13 @@
         <v>140</v>
       </c>
       <c r="D269" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E269" t="s">
-        <v>293</v>
+        <v>445</v>
       </c>
       <c r="G269" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="K269" t="s">
         <v>218</v>
@@ -62846,16 +62983,16 @@
         <v>42736</v>
       </c>
       <c r="C270" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="D270" t="s">
-        <v>51</v>
+        <v>446</v>
       </c>
       <c r="E270" t="s">
-        <v>52</v>
+        <v>293</v>
       </c>
       <c r="G270" t="s">
-        <v>51</v>
+        <v>294</v>
       </c>
       <c r="K270" t="s">
         <v>218</v>
@@ -62872,13 +63009,13 @@
         <v>149</v>
       </c>
       <c r="D271" t="s">
-        <v>239</v>
+        <v>51</v>
       </c>
       <c r="E271" t="s">
-        <v>240</v>
+        <v>52</v>
       </c>
       <c r="G271" t="s">
-        <v>214</v>
+        <v>51</v>
       </c>
       <c r="K271" t="s">
         <v>218</v>
@@ -62892,7 +63029,7 @@
         <v>42736</v>
       </c>
       <c r="C272" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D272" t="s">
         <v>239</v>
@@ -62918,13 +63055,13 @@
         <v>150</v>
       </c>
       <c r="D273" t="s">
-        <v>141</v>
+        <v>239</v>
       </c>
       <c r="E273" t="s">
-        <v>434</v>
+        <v>240</v>
       </c>
       <c r="G273" t="s">
-        <v>435</v>
+        <v>214</v>
       </c>
       <c r="K273" t="s">
         <v>218</v>
@@ -62941,10 +63078,10 @@
         <v>150</v>
       </c>
       <c r="D274" t="s">
-        <v>436</v>
+        <v>141</v>
       </c>
       <c r="E274" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="G274" t="s">
         <v>435</v>
@@ -62964,10 +63101,10 @@
         <v>150</v>
       </c>
       <c r="D275" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E275" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="G275" t="s">
         <v>435</v>
@@ -62987,13 +63124,13 @@
         <v>150</v>
       </c>
       <c r="D276" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E276" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="G276" t="s">
-        <v>291</v>
+        <v>435</v>
       </c>
       <c r="K276" t="s">
         <v>218</v>
@@ -63010,10 +63147,10 @@
         <v>150</v>
       </c>
       <c r="D277" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E277" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="G277" t="s">
         <v>291</v>
@@ -63033,10 +63170,10 @@
         <v>150</v>
       </c>
       <c r="D278" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E278" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="G278" t="s">
         <v>291</v>
@@ -63056,13 +63193,13 @@
         <v>150</v>
       </c>
       <c r="D279" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E279" t="s">
-        <v>293</v>
+        <v>445</v>
       </c>
       <c r="G279" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="K279" t="s">
         <v>218</v>
@@ -63076,16 +63213,16 @@
         <v>42736</v>
       </c>
       <c r="C280" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D280" t="s">
-        <v>239</v>
+        <v>446</v>
       </c>
       <c r="E280" t="s">
-        <v>240</v>
+        <v>293</v>
       </c>
       <c r="G280" t="s">
-        <v>214</v>
+        <v>294</v>
       </c>
       <c r="K280" t="s">
         <v>218</v>
@@ -63102,13 +63239,13 @@
         <v>151</v>
       </c>
       <c r="D281" t="s">
-        <v>141</v>
+        <v>239</v>
       </c>
       <c r="E281" t="s">
-        <v>434</v>
+        <v>240</v>
       </c>
       <c r="G281" t="s">
-        <v>435</v>
+        <v>214</v>
       </c>
       <c r="K281" t="s">
         <v>218</v>
@@ -63125,10 +63262,10 @@
         <v>151</v>
       </c>
       <c r="D282" t="s">
-        <v>436</v>
+        <v>141</v>
       </c>
       <c r="E282" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="G282" t="s">
         <v>435</v>
@@ -63148,10 +63285,10 @@
         <v>151</v>
       </c>
       <c r="D283" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E283" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="G283" t="s">
         <v>435</v>
@@ -63171,13 +63308,13 @@
         <v>151</v>
       </c>
       <c r="D284" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E284" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="G284" t="s">
-        <v>291</v>
+        <v>435</v>
       </c>
       <c r="K284" t="s">
         <v>218</v>
@@ -63194,10 +63331,10 @@
         <v>151</v>
       </c>
       <c r="D285" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E285" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="G285" t="s">
         <v>291</v>
@@ -63217,10 +63354,10 @@
         <v>151</v>
       </c>
       <c r="D286" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E286" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="G286" t="s">
         <v>291</v>
@@ -63240,13 +63377,13 @@
         <v>151</v>
       </c>
       <c r="D287" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E287" t="s">
-        <v>293</v>
+        <v>445</v>
       </c>
       <c r="G287" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="K287" t="s">
         <v>218</v>
@@ -63260,16 +63397,16 @@
         <v>42736</v>
       </c>
       <c r="C288" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D288" t="s">
-        <v>47</v>
+        <v>446</v>
       </c>
       <c r="E288" t="s">
-        <v>47</v>
+        <v>293</v>
       </c>
       <c r="G288" t="s">
-        <v>224</v>
+        <v>294</v>
       </c>
       <c r="K288" t="s">
         <v>218</v>
@@ -63283,7 +63420,7 @@
         <v>42736</v>
       </c>
       <c r="C289" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D289" t="s">
         <v>47</v>
@@ -63306,16 +63443,16 @@
         <v>42736</v>
       </c>
       <c r="C290" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D290" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E290" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G290" t="s">
-        <v>51</v>
+        <v>224</v>
       </c>
       <c r="K290" t="s">
         <v>218</v>
@@ -63332,13 +63469,13 @@
         <v>154</v>
       </c>
       <c r="D291" t="s">
-        <v>239</v>
+        <v>51</v>
       </c>
       <c r="E291" t="s">
-        <v>240</v>
+        <v>52</v>
       </c>
       <c r="G291" t="s">
-        <v>214</v>
+        <v>51</v>
       </c>
       <c r="K291" t="s">
         <v>218</v>
@@ -63352,16 +63489,16 @@
         <v>42736</v>
       </c>
       <c r="C292" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D292" t="s">
-        <v>47</v>
+        <v>239</v>
       </c>
       <c r="E292" t="s">
-        <v>47</v>
+        <v>240</v>
       </c>
       <c r="G292" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="K292" t="s">
         <v>218</v>
@@ -63375,13 +63512,13 @@
         <v>42736</v>
       </c>
       <c r="C293" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D293" t="s">
         <v>47</v>
       </c>
       <c r="E293" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G293" t="s">
         <v>224</v>
@@ -63401,13 +63538,13 @@
         <v>156</v>
       </c>
       <c r="D294" t="s">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="E294" t="s">
-        <v>117</v>
+        <v>48</v>
       </c>
       <c r="G294" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="K294" t="s">
         <v>218</v>
@@ -63424,13 +63561,13 @@
         <v>156</v>
       </c>
       <c r="D295" t="s">
-        <v>239</v>
+        <v>13</v>
       </c>
       <c r="E295" t="s">
-        <v>240</v>
+        <v>117</v>
       </c>
       <c r="G295" t="s">
-        <v>214</v>
+        <v>199</v>
       </c>
       <c r="K295" t="s">
         <v>218</v>
@@ -63444,19 +63581,16 @@
         <v>42736</v>
       </c>
       <c r="C296" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D296" t="s">
-        <v>447</v>
+        <v>239</v>
       </c>
       <c r="E296" t="s">
-        <v>448</v>
+        <v>240</v>
       </c>
       <c r="G296" t="s">
-        <v>206</v>
-      </c>
-      <c r="I296" t="s">
-        <v>449</v>
+        <v>214</v>
       </c>
       <c r="K296" t="s">
         <v>218</v>
@@ -63473,13 +63607,16 @@
         <v>157</v>
       </c>
       <c r="D297" t="s">
-        <v>158</v>
+        <v>447</v>
       </c>
       <c r="E297" t="s">
-        <v>158</v>
+        <v>448</v>
       </c>
       <c r="G297" t="s">
-        <v>224</v>
+        <v>206</v>
+      </c>
+      <c r="I297" t="s">
+        <v>449</v>
       </c>
       <c r="K297" t="s">
         <v>218</v>
@@ -63496,16 +63633,13 @@
         <v>157</v>
       </c>
       <c r="D298" t="s">
-        <v>450</v>
+        <v>158</v>
       </c>
       <c r="E298" t="s">
-        <v>451</v>
+        <v>158</v>
       </c>
       <c r="G298" t="s">
-        <v>206</v>
-      </c>
-      <c r="I298" t="s">
-        <v>452</v>
+        <v>224</v>
       </c>
       <c r="K298" t="s">
         <v>218</v>
@@ -63519,16 +63653,19 @@
         <v>42736</v>
       </c>
       <c r="C299" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D299" t="s">
-        <v>47</v>
+        <v>450</v>
       </c>
       <c r="E299" t="s">
-        <v>47</v>
+        <v>451</v>
       </c>
       <c r="G299" t="s">
-        <v>224</v>
+        <v>206</v>
+      </c>
+      <c r="I299" t="s">
+        <v>452</v>
       </c>
       <c r="K299" t="s">
         <v>218</v>
@@ -63542,7 +63679,7 @@
         <v>42736</v>
       </c>
       <c r="C300" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D300" t="s">
         <v>47</v>
@@ -63565,16 +63702,16 @@
         <v>42736</v>
       </c>
       <c r="C301" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D301" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E301" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G301" t="s">
-        <v>51</v>
+        <v>224</v>
       </c>
       <c r="K301" t="s">
         <v>218</v>
@@ -63591,13 +63728,13 @@
         <v>161</v>
       </c>
       <c r="D302" t="s">
-        <v>239</v>
+        <v>51</v>
       </c>
       <c r="E302" t="s">
-        <v>240</v>
+        <v>52</v>
       </c>
       <c r="G302" t="s">
-        <v>214</v>
+        <v>51</v>
       </c>
       <c r="K302" t="s">
         <v>218</v>
@@ -63611,19 +63748,16 @@
         <v>42736</v>
       </c>
       <c r="C303" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D303" t="s">
-        <v>163</v>
+        <v>239</v>
       </c>
       <c r="E303" t="s">
-        <v>164</v>
+        <v>240</v>
       </c>
       <c r="G303" t="s">
-        <v>216</v>
-      </c>
-      <c r="H303" t="s">
-        <v>453</v>
+        <v>214</v>
       </c>
       <c r="K303" t="s">
         <v>218</v>
@@ -63640,16 +63774,16 @@
         <v>162</v>
       </c>
       <c r="D304" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E304" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="G304" t="s">
         <v>216</v>
       </c>
       <c r="H304" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="K304" t="s">
         <v>218</v>
@@ -63666,14 +63800,17 @@
         <v>162</v>
       </c>
       <c r="D305" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="E305" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="G305" t="s">
         <v>216</v>
       </c>
+      <c r="H305" t="s">
+        <v>454</v>
+      </c>
       <c r="K305" t="s">
         <v>218</v>
       </c>
@@ -63689,13 +63826,13 @@
         <v>162</v>
       </c>
       <c r="D306" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E306" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="G306" t="s">
-        <v>455</v>
+        <v>216</v>
       </c>
       <c r="K306" t="s">
         <v>218</v>
@@ -63712,13 +63849,13 @@
         <v>162</v>
       </c>
       <c r="D307" t="s">
-        <v>456</v>
+        <v>169</v>
       </c>
       <c r="E307" t="s">
-        <v>457</v>
+        <v>170</v>
       </c>
       <c r="G307" t="s">
-        <v>224</v>
+        <v>455</v>
       </c>
       <c r="K307" t="s">
         <v>218</v>
@@ -63735,19 +63872,13 @@
         <v>162</v>
       </c>
       <c r="D308" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="E308" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="G308" t="s">
-        <v>206</v>
-      </c>
-      <c r="H308" t="s">
-        <v>453</v>
-      </c>
-      <c r="I308" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="K308" t="s">
         <v>218</v>
@@ -63764,16 +63895,19 @@
         <v>162</v>
       </c>
       <c r="D309" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="E309" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="G309" t="s">
         <v>206</v>
       </c>
+      <c r="H309" t="s">
+        <v>453</v>
+      </c>
       <c r="I309" t="s">
-        <v>462</v>
+        <v>216</v>
       </c>
       <c r="K309" t="s">
         <v>218</v>
@@ -63790,21 +63924,47 @@
         <v>162</v>
       </c>
       <c r="D310" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="E310" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="G310" t="s">
         <v>206</v>
       </c>
       <c r="I310" t="s">
-        <v>216</v>
+        <v>462</v>
       </c>
       <c r="K310" t="s">
         <v>218</v>
       </c>
       <c r="N310" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="311" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A311" s="1">
+        <v>42736</v>
+      </c>
+      <c r="C311" t="s">
+        <v>162</v>
+      </c>
+      <c r="D311" t="s">
+        <v>463</v>
+      </c>
+      <c r="E311" t="s">
+        <v>464</v>
+      </c>
+      <c r="G311" t="s">
+        <v>206</v>
+      </c>
+      <c r="I311" t="s">
+        <v>216</v>
+      </c>
+      <c r="K311" t="s">
+        <v>218</v>
+      </c>
+      <c r="N311" t="s">
         <v>197</v>
       </c>
     </row>

</xml_diff>